<commit_message>
Update risk_diff.xlsx: Replace existing binary file with a new version to reflect recent changes in risk assessment data.
</commit_message>
<xml_diff>
--- a/formatter/risk_diff.xlsx
+++ b/formatter/risk_diff.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hzeng\Desktop\howard-toolbox\formatter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F3286CC-E2DF-4385-BB2C-292C25A80992}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7B1630A-C22A-499C-8ADD-C904AAA776A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16785" yWindow="-16680" windowWidth="44655" windowHeight="21285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1190" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1191" uniqueCount="310">
   <si>
     <t>Base</t>
   </si>
@@ -1990,43 +1990,43 @@
         <v>0</v>
       </c>
       <c r="R4" s="74">
-        <v>5.5584029700000004</v>
+        <v>5.5838095210000001</v>
       </c>
       <c r="S4" s="63">
-        <v>197.355285952</v>
+        <v>200.87005390600001</v>
       </c>
       <c r="T4" s="75">
-        <v>0.70583887300000003</v>
+        <v>0.70895033299999999</v>
       </c>
       <c r="U4" s="75">
-        <v>8.6697595057030397E-2</v>
+        <v>7.9667938212922895E-2</v>
       </c>
       <c r="V4" s="20">
-        <v>0.66753172243345804</v>
+        <v>0.67033666920151302</v>
       </c>
       <c r="W4" s="20">
-        <v>1.3216746559999999</v>
+        <v>1.349120509</v>
       </c>
       <c r="X4" s="20">
-        <v>4.4605877000000002E-2</v>
+        <v>4.5772753999999999E-2</v>
       </c>
       <c r="Y4" s="63">
-        <v>3.3749513768386898</v>
+        <v>3.3927846841441802</v>
       </c>
       <c r="Z4" s="63">
         <v>0</v>
       </c>
       <c r="AA4" s="76">
         <f t="shared" ref="AA4" si="0">I4-R4</f>
-        <v>6.1249605999999623E-2</v>
+        <v>3.5843054999999957E-2</v>
       </c>
       <c r="AB4" s="61">
         <f t="shared" ref="AB4" si="1">J4-S4</f>
-        <v>6.1681730420000065</v>
+        <v>2.6534050879999995</v>
       </c>
       <c r="AC4" s="77">
         <f t="shared" ref="AC4" si="2">K4-T4</f>
-        <v>5.9093270000000198E-3</v>
+        <v>2.7978670000000649E-3</v>
       </c>
       <c r="AD4" s="77" t="e">
         <f t="shared" ref="AD4" si="3">L4-U4</f>
@@ -2034,19 +2034,19 @@
       </c>
       <c r="AE4" s="15">
         <f t="shared" ref="AE4" si="4">M4-V4</f>
-        <v>5.1648897338330002E-3</v>
+        <v>2.3599429657780169E-3</v>
       </c>
       <c r="AF4" s="15">
         <f t="shared" ref="AF4" si="5">N4-W4</f>
-        <v>2.6423881000000149E-2</v>
+        <v>-1.0219719999999821E-3</v>
       </c>
       <c r="AG4" s="15">
         <f t="shared" ref="AG4" si="6">O4-X4</f>
-        <v>1.072954000000001E-3</v>
+        <v>-9.392299999999576E-5</v>
       </c>
       <c r="AH4" s="77">
         <f t="shared" ref="AH4" si="7">P4-Y4</f>
-        <v>1.3438250944130203E-2</v>
+        <v>-4.3950563613601723E-3</v>
       </c>
       <c r="AI4" s="78">
         <f t="shared" ref="AI4" si="8">Q4-Z4</f>
@@ -2103,43 +2103,43 @@
         <v>0</v>
       </c>
       <c r="R5">
-        <v>5.4408795259999998</v>
+        <v>5.9673139439999998</v>
       </c>
       <c r="S5">
-        <v>184.00562770100001</v>
+        <v>212.17334095800001</v>
       </c>
       <c r="T5">
-        <v>0.66944444400000003</v>
+        <v>6.3374329280000001</v>
       </c>
       <c r="U5">
-        <v>8.1388815564667399E-2</v>
+        <v>0.50461208117763801</v>
       </c>
       <c r="V5">
-        <v>0.63915963982368396</v>
+        <v>4.6880088007445799</v>
       </c>
       <c r="W5">
-        <v>0.46145217100000002</v>
+        <v>7.8622499999999999E-4</v>
       </c>
       <c r="X5">
-        <v>1.7424296999999998E-2</v>
-      </c>
-      <c r="Y5">
-        <v>3.77597031610888</v>
+        <v>0</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>248</v>
       </c>
       <c r="Z5">
         <v>0</v>
       </c>
       <c r="AA5" s="76">
         <f t="shared" ref="AA5:AA26" si="9">I5-R5</f>
-        <v>0</v>
+        <v>-0.52643441800000002</v>
       </c>
       <c r="AB5" s="61">
         <f t="shared" ref="AB5:AB26" si="10">J5-S5</f>
-        <v>0</v>
+        <v>-28.167713257000003</v>
       </c>
       <c r="AC5" s="77">
         <f t="shared" ref="AC5:AC26" si="11">K5-T5</f>
-        <v>0</v>
+        <v>-5.6679884840000003</v>
       </c>
       <c r="AD5" s="77" t="e">
         <f t="shared" ref="AD5:AD26" si="12">L5-U5</f>
@@ -2147,19 +2147,19 @@
       </c>
       <c r="AE5" s="15">
         <f t="shared" ref="AE5:AE26" si="13">M5-V5</f>
-        <v>0</v>
+        <v>-4.0488491609208959</v>
       </c>
       <c r="AF5" s="15">
         <f t="shared" ref="AF5:AF26" si="14">N5-W5</f>
-        <v>1.2808314999999959E-2</v>
+        <v>0.47347426100000001</v>
       </c>
       <c r="AG5" s="15">
         <f t="shared" ref="AG5:AG26" si="15">O5-X5</f>
-        <v>-3.4359999999990232E-6</v>
-      </c>
-      <c r="AH5" s="77">
+        <v>1.7420860999999999E-2</v>
+      </c>
+      <c r="AH5" s="77" t="e">
         <f t="shared" ref="AH5:AH26" si="16">P5-Y5</f>
-        <v>-0.10270182458204991</v>
+        <v>#VALUE!</v>
       </c>
       <c r="AI5" s="78">
         <f t="shared" ref="AI5:AI26" si="17">Q5-Z5</f>
@@ -2216,43 +2216,43 @@
         <v>0</v>
       </c>
       <c r="R6">
-        <v>5.4188675399999999</v>
+        <v>5.4162452859999997</v>
       </c>
       <c r="S6">
-        <v>183.815661038</v>
+        <v>182.37647052700001</v>
       </c>
       <c r="T6">
-        <v>0.75</v>
+        <v>0.66666666699999999</v>
       </c>
       <c r="U6">
-        <v>8.21372950075661E-2</v>
+        <v>7.8800858489135997E-2</v>
       </c>
       <c r="V6">
-        <v>0.71498202723147297</v>
+        <v>0.636702160449926</v>
       </c>
       <c r="W6">
-        <v>0.72538338700000005</v>
+        <v>0.47420277900000002</v>
       </c>
       <c r="X6">
-        <v>3.6494427000000003E-2</v>
+        <v>1.7397675000000001E-2</v>
       </c>
       <c r="Y6">
-        <v>5.0310535992465502</v>
+        <v>3.66882603191155</v>
       </c>
       <c r="Z6">
         <v>0</v>
       </c>
       <c r="AA6" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>2.6222540000002681E-3</v>
       </c>
       <c r="AB6" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1.4391905109999925</v>
       </c>
       <c r="AC6" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>8.3333333000000009E-2</v>
       </c>
       <c r="AD6" s="77" t="e">
         <f t="shared" si="12"/>
@@ -2260,19 +2260,19 @@
       </c>
       <c r="AE6" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>7.827986678154697E-2</v>
       </c>
       <c r="AF6" s="15">
         <f t="shared" si="14"/>
-        <v>3.2700017999999997E-2</v>
+        <v>0.28388062600000002</v>
       </c>
       <c r="AG6" s="15">
         <f t="shared" si="15"/>
-        <v>1.7541399999999943E-3</v>
+        <v>2.0850891999999996E-2</v>
       </c>
       <c r="AH6" s="77">
         <f t="shared" si="16"/>
-        <v>1.4376329403579469E-2</v>
+        <v>1.3766038967385796</v>
       </c>
       <c r="AI6" s="78">
         <f t="shared" si="17"/>
@@ -2329,43 +2329,43 @@
         <v>0</v>
       </c>
       <c r="R7">
-        <v>5.4801712609999997</v>
+        <v>5.394855776</v>
       </c>
       <c r="S7">
-        <v>193.89303531100001</v>
+        <v>182.37293944699999</v>
       </c>
       <c r="T7">
-        <v>0.91666666699999999</v>
+        <v>0.74722222199999999</v>
       </c>
       <c r="U7">
-        <v>8.8068519961977398E-2</v>
+        <v>7.9563839515881099E-2</v>
       </c>
       <c r="V7">
-        <v>0.86301258650189405</v>
+        <v>0.71255796284418305</v>
       </c>
       <c r="W7">
-        <v>0.82205869799999998</v>
+        <v>0.75874397500000001</v>
       </c>
       <c r="X7">
-        <v>4.6496356000000003E-2</v>
+        <v>3.8194080999999998E-2</v>
       </c>
       <c r="Y7">
-        <v>5.6560871034053601</v>
+        <v>5.0338562490726897</v>
       </c>
       <c r="Z7">
         <v>0</v>
       </c>
       <c r="AA7" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>8.5315484999999747E-2</v>
       </c>
       <c r="AB7" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>11.520095864000012</v>
       </c>
       <c r="AC7" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>0.169444445</v>
       </c>
       <c r="AD7" s="77" t="e">
         <f t="shared" si="12"/>
@@ -2373,19 +2373,19 @@
       </c>
       <c r="AE7" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>0.15045462365771101</v>
       </c>
       <c r="AF7" s="15">
         <f t="shared" si="14"/>
-        <v>1.9400469000000031E-2</v>
+        <v>8.2715191999999993E-2</v>
       </c>
       <c r="AG7" s="15">
         <f t="shared" si="15"/>
-        <v>-1.9885099999999989E-4</v>
+        <v>8.1034240000000049E-3</v>
       </c>
       <c r="AH7" s="77">
         <f t="shared" si="16"/>
-        <v>-0.15403699620152</v>
+        <v>0.46819385813115044</v>
       </c>
       <c r="AI7" s="78">
         <f t="shared" si="17"/>
@@ -2442,43 +2442,43 @@
         <v>0</v>
       </c>
       <c r="R8">
-        <v>5.3407397970000003</v>
+        <v>5.4520652289999996</v>
       </c>
       <c r="S8">
-        <v>181.72970571100001</v>
+        <v>192.28782708400001</v>
       </c>
       <c r="T8">
-        <v>1.0833333329999999</v>
+        <v>0.91388888899999998</v>
       </c>
       <c r="U8">
-        <v>0.10173805737804401</v>
+        <v>8.5550964828893905E-2</v>
       </c>
       <c r="V8">
-        <v>0.99981040095315199</v>
+        <v>0.86070366920151897</v>
       </c>
       <c r="W8">
-        <v>0.62044170899999995</v>
+        <v>0.84244585599999999</v>
       </c>
       <c r="X8">
-        <v>3.2623968000000003E-2</v>
+        <v>4.6281238000000002E-2</v>
       </c>
       <c r="Y8">
-        <v>5.2581842140467696</v>
+        <v>5.4936750736417697</v>
       </c>
       <c r="Z8">
         <v>0</v>
       </c>
       <c r="AA8" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>-0.11132543199999922</v>
       </c>
       <c r="AB8" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>-10.558121373000006</v>
       </c>
       <c r="AC8" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>0.16944444399999992</v>
       </c>
       <c r="AD8" s="77" t="e">
         <f t="shared" si="12"/>
@@ -2486,19 +2486,19 @@
       </c>
       <c r="AE8" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>0.13910673175163302</v>
       </c>
       <c r="AF8" s="15">
         <f t="shared" si="14"/>
-        <v>1.8398420999999998E-2</v>
+        <v>-0.20360572600000004</v>
       </c>
       <c r="AG8" s="15">
         <f t="shared" si="15"/>
-        <v>8.045500000000011E-5</v>
+        <v>-1.3576814999999999E-2</v>
       </c>
       <c r="AH8" s="77">
         <f t="shared" si="16"/>
-        <v>-0.13884034940883971</v>
+        <v>-0.37433120900383976</v>
       </c>
       <c r="AI8" s="78">
         <f t="shared" si="17"/>
@@ -2555,43 +2555,43 @@
         <v>0</v>
       </c>
       <c r="R9">
-        <v>5.2604561170000004</v>
+        <v>5.3653236150000003</v>
       </c>
       <c r="S9">
-        <v>174.482540986</v>
+        <v>185.709916792</v>
       </c>
       <c r="T9">
-        <v>1.25</v>
+        <v>1.080555556</v>
       </c>
       <c r="U9">
-        <v>0.117238807223481</v>
+        <v>9.8789601760906801E-2</v>
       </c>
       <c r="V9">
-        <v>1.1385441805869201</v>
+        <v>0.99733899337993903</v>
       </c>
       <c r="W9">
-        <v>0.731443811</v>
+        <v>0.63911900300000002</v>
       </c>
       <c r="X9">
-        <v>3.7956471999999998E-2</v>
+        <v>3.2756825000000003E-2</v>
       </c>
       <c r="Y9">
-        <v>5.1892532863334297</v>
+        <v>5.1253091906578803</v>
       </c>
       <c r="Z9">
         <v>0</v>
       </c>
       <c r="AA9" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>-0.10486749799999995</v>
       </c>
       <c r="AB9" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>-11.227375805999998</v>
       </c>
       <c r="AC9" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>0.16944444400000003</v>
       </c>
       <c r="AD9" s="77" t="e">
         <f t="shared" si="12"/>
@@ -2599,19 +2599,19 @@
       </c>
       <c r="AE9" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>0.14120518720698105</v>
       </c>
       <c r="AF9" s="15">
         <f t="shared" si="14"/>
-        <v>1.3271327999999971E-2</v>
+        <v>0.10559613599999995</v>
       </c>
       <c r="AG9" s="15">
         <f t="shared" si="15"/>
-        <v>1.0139430000000033E-3</v>
+        <v>6.213589999999998E-3</v>
       </c>
       <c r="AH9" s="77">
         <f t="shared" si="16"/>
-        <v>4.3675784012759955E-2</v>
+        <v>0.10761987968830944</v>
       </c>
       <c r="AI9" s="78">
         <f t="shared" si="17"/>
@@ -2668,43 +2668,43 @@
         <v>0</v>
       </c>
       <c r="R10">
-        <v>5.2597473170000004</v>
+        <v>5.2254814850000004</v>
       </c>
       <c r="S10">
-        <v>174.78145048900001</v>
+        <v>172.90878689199999</v>
       </c>
       <c r="T10">
-        <v>1.3333333329999999</v>
+        <v>1.247222222</v>
       </c>
       <c r="U10">
-        <v>0.131982746136868</v>
+        <v>0.114868992325053</v>
       </c>
       <c r="V10">
-        <v>1.2018001227373101</v>
+        <v>1.13650455440181</v>
       </c>
       <c r="W10">
-        <v>0.79661953900000004</v>
+        <v>0.74589581100000002</v>
       </c>
       <c r="X10">
-        <v>4.9243515000000002E-2</v>
+        <v>3.8968309E-2</v>
       </c>
       <c r="Y10">
-        <v>6.1815600282432897</v>
+        <v>5.22436356731329</v>
       </c>
       <c r="Z10">
         <v>0</v>
       </c>
       <c r="AA10" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>3.4265831999999996E-2</v>
       </c>
       <c r="AB10" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1.8726635970000132</v>
       </c>
       <c r="AC10" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>8.6111110999999907E-2</v>
       </c>
       <c r="AD10" s="77" t="e">
         <f t="shared" si="12"/>
@@ -2712,19 +2712,19 @@
       </c>
       <c r="AE10" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>6.5295568335500098E-2</v>
       </c>
       <c r="AF10" s="15">
         <f t="shared" si="14"/>
-        <v>5.4917852999999961E-2</v>
+        <v>0.10564158099999998</v>
       </c>
       <c r="AG10" s="15">
         <f t="shared" si="15"/>
-        <v>9.2149600000000081E-4</v>
+        <v>1.1196702000000003E-2</v>
       </c>
       <c r="AH10" s="77">
         <f t="shared" si="16"/>
-        <v>-0.29044925949855926</v>
+        <v>0.66674720143144039</v>
       </c>
       <c r="AI10" s="78">
         <f t="shared" si="17"/>
@@ -2781,43 +2781,43 @@
         <v>0</v>
       </c>
       <c r="R11">
-        <v>5.2094194150000002</v>
+        <v>5.3463423859999999</v>
       </c>
       <c r="S11">
-        <v>165.01399560199999</v>
+        <v>185.56424450399999</v>
       </c>
       <c r="T11">
-        <v>4.0833333329999997</v>
+        <v>1.330555556</v>
       </c>
       <c r="U11">
-        <v>0.34953513111385398</v>
+        <v>0.128226546443962</v>
       </c>
       <c r="V11">
-        <v>3.3423688401150899</v>
+        <v>1.1990315888472001</v>
       </c>
       <c r="W11">
-        <v>1.8840514479999999</v>
+        <v>0.85152371900000001</v>
       </c>
       <c r="X11">
-        <v>0.134272804</v>
+        <v>5.0035835000000001E-2</v>
       </c>
       <c r="Y11">
-        <v>7.1268119637887901</v>
+        <v>5.8760353802898599</v>
       </c>
       <c r="Z11">
         <v>0</v>
       </c>
       <c r="AA11" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>-0.13692297099999973</v>
       </c>
       <c r="AB11" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>-20.550248901999993</v>
       </c>
       <c r="AC11" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>2.7527777769999995</v>
       </c>
       <c r="AD11" s="77" t="e">
         <f t="shared" si="12"/>
@@ -2825,19 +2825,19 @@
       </c>
       <c r="AE11" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>2.1433372512678899</v>
       </c>
       <c r="AF11" s="15">
         <f t="shared" si="14"/>
-        <v>-3.049209499999983E-2</v>
+        <v>1.0020356340000001</v>
       </c>
       <c r="AG11" s="15">
         <f t="shared" si="15"/>
-        <v>-2.9122869999999856E-3</v>
+        <v>8.1324682000000009E-2</v>
       </c>
       <c r="AH11" s="77">
         <f t="shared" si="16"/>
-        <v>-3.9878557130299974E-2</v>
+        <v>1.2108980263686302</v>
       </c>
       <c r="AI11" s="78">
         <f t="shared" si="17"/>
@@ -2894,43 +2894,43 @@
         <v>0</v>
       </c>
       <c r="R12">
-        <v>5.3547026119999996</v>
+        <v>5.1692215450000001</v>
       </c>
       <c r="S12">
-        <v>173.99358740700001</v>
+        <v>166.04340361600001</v>
       </c>
       <c r="T12">
-        <v>4.9222222220000003</v>
+        <v>4.0805555560000002</v>
       </c>
       <c r="U12">
-        <v>0.231607104267777</v>
+        <v>0.34808256802301901</v>
       </c>
       <c r="V12">
-        <v>4.0762860032357002</v>
+        <v>3.3431574278668301</v>
       </c>
       <c r="W12">
-        <v>0.33921164199999998</v>
+        <v>1.8558750399999999</v>
       </c>
       <c r="X12">
-        <v>1.3294804E-2</v>
+        <v>0.131505979</v>
       </c>
       <c r="Y12">
-        <v>3.9193242076284598</v>
+        <v>7.0859285332055499</v>
       </c>
       <c r="Z12">
         <v>0</v>
       </c>
       <c r="AA12" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>0.18548106699999956</v>
       </c>
       <c r="AB12" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>7.9501837910000006</v>
       </c>
       <c r="AC12" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>0.84166666600000006</v>
       </c>
       <c r="AD12" s="77" t="e">
         <f t="shared" si="12"/>
@@ -2938,19 +2938,19 @@
       </c>
       <c r="AE12" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>0.73312857536887011</v>
       </c>
       <c r="AF12" s="15">
         <f t="shared" si="14"/>
-        <v>1.5491230000000411E-3</v>
+        <v>-1.515114275</v>
       </c>
       <c r="AG12" s="15">
         <f t="shared" si="15"/>
-        <v>1.2479599999999993E-4</v>
+        <v>-0.11808637899999999</v>
       </c>
       <c r="AH12" s="77">
         <f t="shared" si="16"/>
-        <v>1.8805230483350144E-2</v>
+        <v>-3.14779909509374</v>
       </c>
       <c r="AI12" s="78">
         <f t="shared" si="17"/>
@@ -3007,43 +3007,43 @@
         <v>0</v>
       </c>
       <c r="R13">
-        <v>5.7211392060000001</v>
+        <v>5.313084506</v>
       </c>
       <c r="S13">
-        <v>188.554386346</v>
+        <v>175.39506898299999</v>
       </c>
       <c r="T13">
-        <v>7.8786249689999996</v>
+        <v>4.9194444439999998</v>
       </c>
       <c r="U13">
-        <v>0.47862046644101802</v>
+        <v>0.23048007497907899</v>
       </c>
       <c r="V13">
-        <v>5.8228585519689497</v>
+        <v>4.0785157569874402</v>
       </c>
       <c r="W13">
-        <v>0.29744573600000002</v>
+        <v>0.34086098100000001</v>
       </c>
       <c r="X13">
-        <v>1.3360021999999999E-2</v>
+        <v>1.3329967999999999E-2</v>
       </c>
       <c r="Y13">
-        <v>4.4915829622113002</v>
+        <v>3.9106758306255101</v>
       </c>
       <c r="Z13">
         <v>0</v>
       </c>
       <c r="AA13" s="76">
         <f t="shared" si="9"/>
-        <v>1.3324832999999536E-2</v>
+        <v>0.42137953299999964</v>
       </c>
       <c r="AB13" s="61">
         <f t="shared" si="10"/>
-        <v>1.1061983339999983</v>
+        <v>14.265515697000012</v>
       </c>
       <c r="AC13" s="77">
         <f t="shared" si="11"/>
-        <v>3.8041698000000679E-2</v>
+        <v>2.9972222230000005</v>
       </c>
       <c r="AD13" s="77" t="e">
         <f t="shared" si="12"/>
@@ -3051,19 +3051,19 @@
       </c>
       <c r="AE13" s="15">
         <f t="shared" si="13"/>
-        <v>2.0105560142010148E-2</v>
+        <v>1.7644483551235197</v>
       </c>
       <c r="AF13" s="15">
         <f t="shared" si="14"/>
-        <v>9.0600100000000072E-3</v>
+        <v>-3.4355234999999984E-2</v>
       </c>
       <c r="AG13" s="15">
         <f t="shared" si="15"/>
-        <v>1.5769700000000005E-4</v>
+        <v>1.8775099999999989E-4</v>
       </c>
       <c r="AH13" s="77">
         <f t="shared" si="16"/>
-        <v>-8.1316865601159805E-2</v>
+        <v>0.4995902659846303</v>
       </c>
       <c r="AI13" s="78">
         <f t="shared" si="17"/>
@@ -3120,43 +3120,43 @@
         <v>0</v>
       </c>
       <c r="R14">
-        <v>5.3485899310000002</v>
+        <v>5.6962580999999997</v>
       </c>
       <c r="S14">
-        <v>174.75661690199999</v>
+        <v>190.57301950300001</v>
       </c>
       <c r="T14">
-        <v>0.66944444400000003</v>
+        <v>7.9138888889999999</v>
       </c>
       <c r="U14">
-        <v>8.4534647087133305E-2</v>
+        <v>0.54706124411788903</v>
       </c>
       <c r="V14">
-        <v>0.63685947424169798</v>
+        <v>5.8496912787913899</v>
       </c>
       <c r="W14">
-        <v>0.32726863</v>
+        <v>0.307282895</v>
       </c>
       <c r="X14">
-        <v>1.3332947E-2</v>
+        <v>1.3540638000000001E-2</v>
       </c>
       <c r="Y14">
-        <v>4.0740070320824797</v>
+        <v>4.4065706944084901</v>
       </c>
       <c r="Z14">
         <v>0</v>
       </c>
       <c r="AA14" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>-0.34766816899999942</v>
       </c>
       <c r="AB14" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>-15.816402601000021</v>
       </c>
       <c r="AC14" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>-7.2444444450000001</v>
       </c>
       <c r="AD14" s="77" t="e">
         <f t="shared" si="12"/>
@@ -3164,19 +3164,19 @@
       </c>
       <c r="AE14" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>-5.2128318045496922</v>
       </c>
       <c r="AF14" s="15">
         <f t="shared" si="14"/>
-        <v>7.2326209999999946E-3</v>
+        <v>2.7218355999999999E-2</v>
       </c>
       <c r="AG14" s="15">
         <f t="shared" si="15"/>
-        <v>3.7258000000000083E-5</v>
+        <v>-1.7043300000000108E-4</v>
       </c>
       <c r="AH14" s="77">
         <f t="shared" si="16"/>
-        <v>-7.6950231837509708E-2</v>
+        <v>-0.40951389416352013</v>
       </c>
       <c r="AI14" s="78">
         <f t="shared" si="17"/>
@@ -3233,43 +3233,43 @@
         <v>0</v>
       </c>
       <c r="R15">
-        <v>5.2493617439999998</v>
+        <v>5.3176337020000002</v>
       </c>
       <c r="S15">
-        <v>166.83586101099999</v>
+        <v>172.493607406</v>
       </c>
       <c r="T15">
-        <v>0.75</v>
+        <v>0.66666666699999999</v>
       </c>
       <c r="U15">
-        <v>8.6718935882876005E-2</v>
+        <v>8.1976883004335102E-2</v>
       </c>
       <c r="V15">
-        <v>0.71210206919628705</v>
+        <v>0.63444388348580505</v>
       </c>
       <c r="W15">
-        <v>0.39296709099999999</v>
+        <v>0.33514227600000002</v>
       </c>
       <c r="X15">
-        <v>2.0223879E-2</v>
+        <v>1.336057E-2</v>
       </c>
       <c r="Y15">
-        <v>5.1464561443390702</v>
+        <v>3.98653675073807</v>
       </c>
       <c r="Z15">
         <v>0</v>
       </c>
       <c r="AA15" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>-6.827195800000041E-2</v>
       </c>
       <c r="AB15" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>-5.6577463950000038</v>
       </c>
       <c r="AC15" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>8.3333333000000009E-2</v>
       </c>
       <c r="AD15" s="77" t="e">
         <f t="shared" si="12"/>
@@ -3277,19 +3277,19 @@
       </c>
       <c r="AE15" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>7.7658185710481997E-2</v>
       </c>
       <c r="AF15" s="15">
         <f t="shared" si="14"/>
-        <v>7.7181410000000117E-3</v>
+        <v>6.5542955999999986E-2</v>
       </c>
       <c r="AG15" s="15">
         <f t="shared" si="15"/>
-        <v>-1.5631500000000062E-4</v>
+        <v>6.7069939999999991E-3</v>
       </c>
       <c r="AH15" s="77">
         <f t="shared" si="16"/>
-        <v>-0.13814478236704009</v>
+        <v>1.0217746112339601</v>
       </c>
       <c r="AI15" s="78">
         <f t="shared" si="17"/>
@@ -3346,43 +3346,43 @@
         <v>0</v>
       </c>
       <c r="R16">
-        <v>5.3488216470000003</v>
+        <v>5.4615960169999997</v>
       </c>
       <c r="S16">
-        <v>172.76432298700001</v>
+        <v>189.01540915499999</v>
       </c>
       <c r="T16">
-        <v>0.58333333300000001</v>
+        <v>0.74722222199999999</v>
       </c>
       <c r="U16">
-        <v>8.2134625996952204E-2</v>
+        <v>8.2919137845634303E-2</v>
       </c>
       <c r="V16">
-        <v>0.55975120657534105</v>
+        <v>0.70885907110864099</v>
       </c>
       <c r="W16">
-        <v>0.45854962300000002</v>
+        <v>0.40015246500000001</v>
       </c>
       <c r="X16">
-        <v>2.8326638000000001E-2</v>
+        <v>2.0002501999999998E-2</v>
       </c>
       <c r="Y16">
-        <v>6.1774422176332298</v>
+        <v>4.9987201753211696</v>
       </c>
       <c r="Z16">
         <v>0</v>
       </c>
       <c r="AA16" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>-0.11277436999999946</v>
       </c>
       <c r="AB16" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>-16.251086167999972</v>
       </c>
       <c r="AC16" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>-0.16388888899999998</v>
       </c>
       <c r="AD16" s="77" t="e">
         <f t="shared" si="12"/>
@@ -3390,19 +3390,19 @@
       </c>
       <c r="AE16" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>-0.14910786453329994</v>
       </c>
       <c r="AF16" s="15">
         <f t="shared" si="14"/>
-        <v>6.8140879999999959E-3</v>
+        <v>6.5211246E-2</v>
       </c>
       <c r="AG16" s="15">
         <f t="shared" si="15"/>
-        <v>3.0679200000000018E-4</v>
+        <v>8.630928000000003E-3</v>
       </c>
       <c r="AH16" s="77">
         <f t="shared" si="16"/>
-        <v>-2.4527986639399479E-2</v>
+        <v>1.1541940556726606</v>
       </c>
       <c r="AI16" s="78">
         <f t="shared" si="17"/>
@@ -3459,43 +3459,43 @@
         <v>0</v>
       </c>
       <c r="R17">
-        <v>5.3976119889999996</v>
+        <v>5.3210423049999998</v>
       </c>
       <c r="S17">
-        <v>183.83193711600001</v>
+        <v>170.70106768400001</v>
       </c>
       <c r="T17">
-        <v>0.84166666700000003</v>
+        <v>0.58055555599999997</v>
       </c>
       <c r="U17">
-        <v>8.5246941768510304E-2</v>
+        <v>7.9541993789952206E-2</v>
       </c>
       <c r="V17">
-        <v>0.79595662209441698</v>
+        <v>0.55727185436834503</v>
       </c>
       <c r="W17">
-        <v>0.54806489000000003</v>
+        <v>0.46512917399999998</v>
       </c>
       <c r="X17">
-        <v>4.6488504999999999E-2</v>
+        <v>2.8592039E-2</v>
       </c>
       <c r="Y17">
-        <v>8.4822994226103408</v>
+        <v>6.14711796168692</v>
       </c>
       <c r="Z17">
         <v>0</v>
       </c>
       <c r="AA17" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>7.656968399999986E-2</v>
       </c>
       <c r="AB17" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>13.130869431999997</v>
       </c>
       <c r="AC17" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>0.26111111100000006</v>
       </c>
       <c r="AD17" s="77" t="e">
         <f t="shared" si="12"/>
@@ -3503,19 +3503,19 @@
       </c>
       <c r="AE17" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>0.23868476772607194</v>
       </c>
       <c r="AF17" s="15">
         <f t="shared" si="14"/>
-        <v>1.0689815999999963E-2</v>
+        <v>9.3625532000000011E-2</v>
       </c>
       <c r="AG17" s="15">
         <f t="shared" si="15"/>
-        <v>2.531240000000004E-4</v>
+        <v>1.814959E-2</v>
       </c>
       <c r="AH17" s="77">
         <f t="shared" si="16"/>
-        <v>-0.1169776636916815</v>
+        <v>2.2182037972317392</v>
       </c>
       <c r="AI17" s="78">
         <f t="shared" si="17"/>
@@ -3572,43 +3572,43 @@
         <v>0</v>
       </c>
       <c r="R18">
-        <v>5.3262044230000001</v>
+        <v>5.3709643140000001</v>
       </c>
       <c r="S18">
-        <v>179.953175195</v>
+        <v>182.25207087800001</v>
       </c>
       <c r="T18">
-        <v>1</v>
+        <v>0.83888888900000003</v>
       </c>
       <c r="U18">
-        <v>9.4675754213442001E-2</v>
+        <v>8.2703730649423601E-2</v>
       </c>
       <c r="V18">
-        <v>0.93653116453498397</v>
+        <v>0.79359373592140303</v>
       </c>
       <c r="W18">
-        <v>0.60749518000000002</v>
+        <v>0.55707205000000004</v>
       </c>
       <c r="X18">
-        <v>3.8951225999999999E-2</v>
+        <v>4.6738254E-2</v>
       </c>
       <c r="Y18">
-        <v>6.41177531647247</v>
+        <v>8.3899836654881508</v>
       </c>
       <c r="Z18">
         <v>0</v>
       </c>
       <c r="AA18" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>-4.4759890999999996E-2</v>
       </c>
       <c r="AB18" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>-2.298895683000012</v>
       </c>
       <c r="AC18" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>0.16111111099999997</v>
       </c>
       <c r="AD18" s="77" t="e">
         <f t="shared" si="12"/>
@@ -3616,19 +3616,19 @@
       </c>
       <c r="AE18" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>0.14293742861358094</v>
       </c>
       <c r="AF18" s="15">
         <f t="shared" si="14"/>
-        <v>1.1243969999999992E-2</v>
+        <v>6.1667099999999975E-2</v>
       </c>
       <c r="AG18" s="15">
         <f t="shared" si="15"/>
-        <v>-1.3681699999999741E-4</v>
+        <v>-7.9238449999999988E-3</v>
       </c>
       <c r="AH18" s="77">
         <f t="shared" si="16"/>
-        <v>-0.13862951666328982</v>
+        <v>-2.1168378656789706</v>
       </c>
       <c r="AI18" s="78">
         <f t="shared" si="17"/>
@@ -3685,43 +3685,43 @@
         <v>0</v>
       </c>
       <c r="R19">
-        <v>5.4499843129999999</v>
+        <v>5.2952201370000003</v>
       </c>
       <c r="S19">
-        <v>192.607225747</v>
+        <v>178.20755517200001</v>
       </c>
       <c r="T19">
-        <v>1.0833333329999999</v>
+        <v>0.99722222199999999</v>
       </c>
       <c r="U19">
-        <v>0.107534489365395</v>
+        <v>9.2193597970580604E-2</v>
       </c>
       <c r="V19">
-        <v>0.99298397061939103</v>
+        <v>0.93429121610334098</v>
       </c>
       <c r="W19">
-        <v>0.65545010000000004</v>
+        <v>0.61907869900000001</v>
       </c>
       <c r="X19">
-        <v>5.0176022000000001E-2</v>
+        <v>3.8780278000000001E-2</v>
       </c>
       <c r="Y19">
-        <v>7.6552009069798004</v>
+        <v>6.2641919456511603</v>
       </c>
       <c r="Z19">
         <v>0</v>
       </c>
       <c r="AA19" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>0.15476417599999959</v>
       </c>
       <c r="AB19" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>14.399670574999988</v>
       </c>
       <c r="AC19" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>8.6111110999999907E-2</v>
       </c>
       <c r="AD19" s="77" t="e">
         <f t="shared" si="12"/>
@@ -3729,19 +3729,19 @@
       </c>
       <c r="AE19" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>5.869275451605005E-2</v>
       </c>
       <c r="AF19" s="15">
         <f t="shared" si="14"/>
-        <v>2.3216979999999277E-3</v>
+        <v>3.8693098999999953E-2</v>
       </c>
       <c r="AG19" s="15">
         <f t="shared" si="15"/>
-        <v>-4.2748699999999723E-4</v>
+        <v>1.0968257000000002E-2</v>
       </c>
       <c r="AH19" s="77">
         <f t="shared" si="16"/>
-        <v>-9.20102759336201E-2</v>
+        <v>1.2989986853950199</v>
       </c>
       <c r="AI19" s="78">
         <f t="shared" si="17"/>
@@ -3798,43 +3798,43 @@
         <v>0</v>
       </c>
       <c r="R20">
-        <v>5.8026868980000001</v>
+        <v>5.4135034390000003</v>
       </c>
       <c r="S20">
-        <v>230.291131103</v>
+        <v>190.47670634100001</v>
       </c>
       <c r="T20">
-        <v>1.5888888889999999</v>
+        <v>1.080555556</v>
       </c>
       <c r="U20">
-        <v>0.14673994107598601</v>
+        <v>0.10512444929005001</v>
       </c>
       <c r="V20">
-        <v>1.4073854873845799</v>
+        <v>0.99086437436354402</v>
       </c>
       <c r="W20">
-        <v>1.053256543</v>
+        <v>0.65657367099999997</v>
       </c>
       <c r="X20">
-        <v>0.12680377700000001</v>
+        <v>4.9667061999999998E-2</v>
       </c>
       <c r="Y20">
-        <v>12.039210944640701</v>
+        <v>7.5645832590810702</v>
       </c>
       <c r="Z20">
         <v>0</v>
       </c>
       <c r="AA20" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>0.38918345899999984</v>
       </c>
       <c r="AB20" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>39.814424761999987</v>
       </c>
       <c r="AC20" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>0.50833333299999994</v>
       </c>
       <c r="AD20" s="77" t="e">
         <f t="shared" si="12"/>
@@ -3842,19 +3842,19 @@
       </c>
       <c r="AE20" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>0.41652111302103589</v>
       </c>
       <c r="AF20" s="15">
         <f t="shared" si="14"/>
-        <v>2.3253729999999972E-2</v>
+        <v>0.41993660200000005</v>
       </c>
       <c r="AG20" s="15">
         <f t="shared" si="15"/>
-        <v>-3.1162600000000096E-3</v>
+        <v>7.4020454999999999E-2</v>
       </c>
       <c r="AH20" s="77">
         <f t="shared" si="16"/>
-        <v>-0.54953731102919967</v>
+        <v>3.9250903745304306</v>
       </c>
       <c r="AI20" s="78">
         <f t="shared" si="17"/>
@@ -3911,43 +3911,43 @@
         <v>0</v>
       </c>
       <c r="R21">
-        <v>6.7875901179999998</v>
+        <v>5.7606618159999998</v>
       </c>
       <c r="S21">
-        <v>330.08829133900002</v>
+        <v>228.82854234300001</v>
       </c>
       <c r="T21">
-        <v>2.5833333330000001</v>
+        <v>1.5861111109999999</v>
       </c>
       <c r="U21">
-        <v>-1.2920510350305101</v>
+        <v>0.14449127980759699</v>
       </c>
       <c r="V21">
-        <v>2.2883072797506698</v>
+        <v>1.40565059665849</v>
       </c>
       <c r="W21">
-        <v>0.49775793200000001</v>
+        <v>1.0772370529999999</v>
       </c>
       <c r="X21">
-        <v>7.5065726999999999E-2</v>
+        <v>0.123706897</v>
       </c>
       <c r="Y21">
-        <v>15.080769621969599</v>
+        <v>11.483720937326501</v>
       </c>
       <c r="Z21">
         <v>0</v>
       </c>
       <c r="AA21" s="76">
         <f t="shared" si="9"/>
-        <v>-9.6913235999999792E-2</v>
+        <v>0.93001506600000017</v>
       </c>
       <c r="AB21" s="61">
         <f t="shared" si="10"/>
-        <v>-9.4620372120000411</v>
+        <v>91.797711783999972</v>
       </c>
       <c r="AC21" s="77">
         <f t="shared" si="11"/>
-        <v>-0.16666666600000024</v>
+        <v>0.83055555599999997</v>
       </c>
       <c r="AD21" s="77" t="e">
         <f t="shared" si="12"/>
@@ -3955,19 +3955,19 @@
       </c>
       <c r="AE21" s="15">
         <f t="shared" si="13"/>
-        <v>-0.1352325135079897</v>
+        <v>0.74742416958419011</v>
       </c>
       <c r="AF21" s="15">
         <f t="shared" si="14"/>
-        <v>6.7949180000000386E-3</v>
+        <v>-0.57268420299999989</v>
       </c>
       <c r="AG21" s="15">
         <f t="shared" si="15"/>
-        <v>8.1591200000000197E-4</v>
+        <v>-4.7825257999999995E-2</v>
       </c>
       <c r="AH21" s="77">
         <f t="shared" si="16"/>
-        <v>-4.1385937980900067E-2</v>
+        <v>3.5556627466621986</v>
       </c>
       <c r="AI21" s="78">
         <f t="shared" si="17"/>
@@ -4024,43 +4024,43 @@
         <v>0</v>
       </c>
       <c r="R22">
-        <v>5.3343486569999996</v>
+        <v>6.6533275639999996</v>
       </c>
       <c r="S22">
-        <v>179.73728940000001</v>
+        <v>321.056554914</v>
       </c>
       <c r="T22">
-        <v>0.97080355399999996</v>
+        <v>2.4138888889999999</v>
       </c>
       <c r="U22">
-        <v>-1.1170182739094E-2</v>
+        <v>-1.7368872058628799</v>
       </c>
       <c r="V22">
-        <v>0.92874862747044695</v>
+        <v>2.1518868944271299</v>
       </c>
       <c r="W22">
-        <v>0.49775793200000001</v>
+        <v>0.50234702799999997</v>
       </c>
       <c r="X22">
-        <v>7.5065726999999999E-2</v>
+        <v>7.5873533000000007E-2</v>
       </c>
       <c r="Y22">
-        <v>15.080769621969599</v>
+        <v>15.1038084771948</v>
       </c>
       <c r="Z22">
         <v>0</v>
       </c>
       <c r="AA22" s="76">
         <f t="shared" si="9"/>
-        <v>-5.3486571999999732E-2</v>
+        <v>-1.3724654789999997</v>
       </c>
       <c r="AB22" s="61">
         <f t="shared" si="10"/>
-        <v>-6.5934847139999988</v>
+        <v>-147.91275022799999</v>
       </c>
       <c r="AC22" s="77">
         <f t="shared" si="11"/>
-        <v>-9.2424002000000005E-2</v>
+        <v>-1.5355093369999999</v>
       </c>
       <c r="AD22" s="77" t="e">
         <f t="shared" si="12"/>
@@ -4068,19 +4068,19 @@
       </c>
       <c r="AE22" s="15">
         <f t="shared" si="13"/>
-        <v>-8.6351631740984924E-2</v>
+        <v>-1.309489898697668</v>
       </c>
       <c r="AF22" s="15">
         <f t="shared" si="14"/>
-        <v>6.7949180000000386E-3</v>
+        <v>2.2058220000000794E-3</v>
       </c>
       <c r="AG22" s="15">
         <f t="shared" si="15"/>
-        <v>8.1591200000000197E-4</v>
+        <v>8.1059999999938404E-6</v>
       </c>
       <c r="AH22" s="77">
         <f t="shared" si="16"/>
-        <v>-4.1385937980900067E-2</v>
+        <v>-6.4424793206100617E-2</v>
       </c>
       <c r="AI22" s="78">
         <f t="shared" si="17"/>
@@ -4137,43 +4137,43 @@
         <v>0</v>
       </c>
       <c r="R23">
-        <v>5.1379376849999998</v>
+        <v>5.2611168800000003</v>
       </c>
       <c r="S23">
-        <v>163.66718266500001</v>
+        <v>172.343188441</v>
       </c>
       <c r="T23">
-        <v>1.458990002</v>
+        <v>0.86755764000000002</v>
       </c>
       <c r="U23">
-        <v>-0.66397573529987897</v>
+        <v>-0.13760582282252901</v>
       </c>
       <c r="V23">
-        <v>1.37256305240455</v>
+        <v>0.83240961267255298</v>
       </c>
       <c r="W23">
-        <v>0.49775793200000001</v>
+        <v>0.50234702799999997</v>
       </c>
       <c r="X23">
-        <v>7.5065726999999999E-2</v>
+        <v>7.5873533000000007E-2</v>
       </c>
       <c r="Y23">
-        <v>15.080769621969599</v>
+        <v>15.1038084771948</v>
       </c>
       <c r="Z23">
         <v>0</v>
       </c>
       <c r="AA23" s="76">
         <f t="shared" si="9"/>
-        <v>-9.820133399999964E-2</v>
+        <v>-0.22138052900000016</v>
       </c>
       <c r="AB23" s="61">
         <f t="shared" si="10"/>
-        <v>-10.399250341000027</v>
+        <v>-19.075256117000009</v>
       </c>
       <c r="AC23" s="77">
         <f t="shared" si="11"/>
-        <v>-0.10940627399999991</v>
+        <v>0.48202608800000002</v>
       </c>
       <c r="AD23" s="77" t="e">
         <f t="shared" si="12"/>
@@ -4181,19 +4181,19 @@
       </c>
       <c r="AE23" s="15">
         <f t="shared" si="13"/>
-        <v>-9.8202196701030031E-2</v>
+        <v>0.441951243030967</v>
       </c>
       <c r="AF23" s="15">
         <f t="shared" si="14"/>
-        <v>6.7949180000000386E-3</v>
+        <v>2.2058220000000794E-3</v>
       </c>
       <c r="AG23" s="15">
         <f t="shared" si="15"/>
-        <v>8.1591200000000197E-4</v>
+        <v>8.1059999999938404E-6</v>
       </c>
       <c r="AH23" s="77">
         <f t="shared" si="16"/>
-        <v>-4.1385937980900067E-2</v>
+        <v>-6.4424793206100617E-2</v>
       </c>
       <c r="AI23" s="78">
         <f t="shared" si="17"/>
@@ -4250,43 +4250,43 @@
         <v>0</v>
       </c>
       <c r="R24">
-        <v>5.6889637000000004</v>
+        <v>5.0015776340000002</v>
       </c>
       <c r="S24">
-        <v>220.75234184600001</v>
+        <v>151.62071035299999</v>
       </c>
       <c r="T24">
-        <v>2.1947377540000002</v>
+        <v>1.3332607540000001</v>
       </c>
       <c r="U24">
-        <v>-1.07355920096851</v>
+        <v>-0.85145093336308397</v>
       </c>
       <c r="V24">
-        <v>2.0044295970944401</v>
+        <v>1.2599122151373601</v>
       </c>
       <c r="W24">
-        <v>0.49775793200000001</v>
+        <v>0.50234702799999997</v>
       </c>
       <c r="X24">
-        <v>7.5065726999999999E-2</v>
+        <v>7.5873533000000007E-2</v>
       </c>
       <c r="Y24">
-        <v>15.080769621969599</v>
+        <v>15.1038084771948</v>
       </c>
       <c r="Z24">
         <v>0</v>
       </c>
       <c r="AA24" s="76">
         <f t="shared" si="9"/>
-        <v>-5.4484371000000031E-2</v>
+        <v>0.63290169500000015</v>
       </c>
       <c r="AB24" s="61">
         <f t="shared" si="10"/>
-        <v>-5.4543361919999995</v>
+        <v>63.677295301000015</v>
       </c>
       <c r="AC24" s="77">
         <f t="shared" si="11"/>
-        <v>-8.822299400000011E-2</v>
+        <v>0.77325400599999994</v>
       </c>
       <c r="AD24" s="77" t="e">
         <f t="shared" si="12"/>
@@ -4294,19 +4294,19 @@
       </c>
       <c r="AE24" s="15">
         <f t="shared" si="13"/>
-        <v>-7.4521941888630039E-2</v>
+        <v>0.66999544006845002</v>
       </c>
       <c r="AF24" s="15">
         <f t="shared" si="14"/>
-        <v>6.7949180000000386E-3</v>
+        <v>2.2058220000000794E-3</v>
       </c>
       <c r="AG24" s="15">
         <f t="shared" si="15"/>
-        <v>8.1591200000000197E-4</v>
+        <v>8.1059999999938404E-6</v>
       </c>
       <c r="AH24" s="77">
         <f t="shared" si="16"/>
-        <v>-4.1385937980900067E-2</v>
+        <v>-6.4424793206100617E-2</v>
       </c>
       <c r="AI24" s="78">
         <f t="shared" si="17"/>
@@ -4363,43 +4363,43 @@
         <v>0</v>
       </c>
       <c r="R25">
-        <v>5.9510107220000004</v>
+        <v>5.5870382999999997</v>
       </c>
       <c r="S25">
-        <v>246.43036474100001</v>
+        <v>214.39269253399999</v>
       </c>
       <c r="T25">
-        <v>2.5833333330000001</v>
+        <v>2.0876789740000001</v>
       </c>
       <c r="U25">
-        <v>-4.2778031999994401E-2</v>
+        <v>-1.4720541491525401</v>
       </c>
       <c r="V25">
-        <v>2.2971036668235398</v>
+        <v>1.9147745975786901</v>
       </c>
       <c r="W25">
-        <v>1.919839436</v>
+        <v>0.50234702799999997</v>
       </c>
       <c r="X25">
-        <v>0.23438508199999999</v>
+        <v>7.5873533000000007E-2</v>
       </c>
       <c r="Y25">
-        <v>12.2085773218797</v>
+        <v>15.1038084771948</v>
       </c>
       <c r="Z25">
         <v>0</v>
       </c>
       <c r="AA25" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>0.36397242200000068</v>
       </c>
       <c r="AB25" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>32.037672207000014</v>
       </c>
       <c r="AC25" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>0.49565435899999999</v>
       </c>
       <c r="AD25" s="77" t="e">
         <f t="shared" si="12"/>
@@ -4407,19 +4407,19 @@
       </c>
       <c r="AE25" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>0.38232906924484977</v>
       </c>
       <c r="AF25" s="15">
         <f t="shared" si="14"/>
-        <v>6.5890071999999966E-2</v>
+        <v>1.4833824799999999</v>
       </c>
       <c r="AG25" s="15">
         <f t="shared" si="15"/>
-        <v>6.3147620000000015E-3</v>
+        <v>0.164826311</v>
       </c>
       <c r="AH25" s="77">
         <f t="shared" si="16"/>
-        <v>-8.7095366241699779E-2</v>
+        <v>-2.9823265215568</v>
       </c>
       <c r="AI25" s="78">
         <f t="shared" si="17"/>
@@ -4476,43 +4476,43 @@
         <v>0</v>
       </c>
       <c r="R26">
-        <v>6.1598139950000004</v>
+        <v>5.9858454559999998</v>
       </c>
       <c r="S26">
-        <v>267.15818930900002</v>
+        <v>254.17028324</v>
       </c>
       <c r="T26">
-        <v>2.6666666669999999</v>
+        <v>2.5805555560000002</v>
       </c>
       <c r="U26">
-        <v>0.14731815405406001</v>
+        <v>0.134929649971605</v>
       </c>
       <c r="V26">
-        <v>2.3117724765765701</v>
+        <v>2.2581962830210101</v>
       </c>
       <c r="W26">
-        <v>1.7559363619999999</v>
+        <v>1.915477533</v>
       </c>
       <c r="X26">
-        <v>0.26462306499999999</v>
+        <v>0.23445213600000001</v>
       </c>
       <c r="Y26">
-        <v>15.070196775160801</v>
+        <v>12.2398791925689</v>
       </c>
       <c r="Z26">
         <v>0</v>
       </c>
       <c r="AA26" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>0.17396853900000053</v>
       </c>
       <c r="AB26" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>12.987906069000019</v>
       </c>
       <c r="AC26" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>8.6111110999999685E-2</v>
       </c>
       <c r="AD26" s="77" t="e">
         <f t="shared" si="12"/>
@@ -4520,19 +4520,19 @@
       </c>
       <c r="AE26" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>5.3576193555560092E-2</v>
       </c>
       <c r="AF26" s="15">
         <f t="shared" si="14"/>
-        <v>7.2900700000011476E-4</v>
+        <v>-0.15881216399999998</v>
       </c>
       <c r="AG26" s="15">
         <f t="shared" si="15"/>
-        <v>-1.2366545000000007E-2</v>
+        <v>1.7804383999999979E-2</v>
       </c>
       <c r="AH26" s="77">
         <f t="shared" si="16"/>
-        <v>-0.71023246712640109</v>
+        <v>2.1200851154654998</v>
       </c>
       <c r="AI26" s="78">
         <f t="shared" si="17"/>
@@ -4589,43 +4589,43 @@
         <v>0</v>
       </c>
       <c r="R27">
-        <v>6.4500495950000003</v>
+        <v>5.5811964359999999</v>
       </c>
       <c r="S27">
-        <v>291.13234564999999</v>
+        <v>213.77086694900001</v>
       </c>
       <c r="T27">
-        <v>0.87233357700000003</v>
+        <v>2.5805555560000002</v>
       </c>
       <c r="U27">
-        <v>-0.11003694957064999</v>
+        <v>5.4688688382957797E-2</v>
       </c>
       <c r="V27">
-        <v>0.81671505476149797</v>
+        <v>2.30098428768243</v>
       </c>
       <c r="W27">
-        <v>1.9380790640000001</v>
+        <v>1.98165094</v>
       </c>
       <c r="X27">
-        <v>0.18546258199999999</v>
+        <v>0.239670205</v>
       </c>
       <c r="Y27">
-        <v>9.5694022728476291</v>
+        <v>12.094471340144301</v>
       </c>
       <c r="Z27">
         <v>0</v>
       </c>
       <c r="AA27" s="76">
         <f t="shared" ref="AA27:AA39" si="18">I27-R27</f>
-        <v>2.3981170999999968E-2</v>
+        <v>0.89283433000000034</v>
       </c>
       <c r="AB27" s="61">
         <f t="shared" ref="AB27:AB39" si="19">J27-S27</f>
-        <v>2.4555979730000104</v>
+        <v>79.817076673999992</v>
       </c>
       <c r="AC27" s="77">
         <f t="shared" ref="AC27:AC39" si="20">K27-T27</f>
-        <v>6.2760619999999712E-3</v>
+        <v>-1.7019459170000002</v>
       </c>
       <c r="AD27" s="77" t="e">
         <f t="shared" ref="AD27:AD39" si="21">L27-U27</f>
@@ -4633,19 +4633,19 @@
       </c>
       <c r="AE27" s="15">
         <f t="shared" ref="AE27:AE39" si="22">M27-V27</f>
-        <v>5.4501914345280733E-3</v>
+        <v>-1.478819041486404</v>
       </c>
       <c r="AF27" s="15">
         <f t="shared" ref="AF27:AF39" si="23">N27-W27</f>
-        <v>5.0599826999999875E-2</v>
+        <v>7.0279509999999767E-3</v>
       </c>
       <c r="AG27" s="15">
         <f t="shared" ref="AG27:AG39" si="24">O27-X27</f>
-        <v>2.7575260000000101E-3</v>
+        <v>-5.1450097E-2</v>
       </c>
       <c r="AH27" s="77">
         <f t="shared" ref="AH27:AH39" si="25">P27-Y27</f>
-        <v>-0.10482210096506961</v>
+        <v>-2.6298911682617412</v>
       </c>
       <c r="AI27" s="78">
         <f t="shared" ref="AI27:AI39" si="26">Q27-Z27</f>
@@ -4702,43 +4702,43 @@
         <v>0</v>
       </c>
       <c r="R28">
-        <v>6.1052259439999998</v>
+        <v>6.1202938820000004</v>
       </c>
       <c r="S28">
-        <v>262.02352718899999</v>
+        <v>267.56749742599999</v>
       </c>
       <c r="T28">
-        <v>2.4166666669999999</v>
+        <v>2.6638888889999999</v>
       </c>
       <c r="U28">
-        <v>0.13408378627339401</v>
+        <v>-0.13160764504505101</v>
       </c>
       <c r="V28">
-        <v>2.11736945479297</v>
+        <v>2.3109096558558599</v>
       </c>
       <c r="W28">
-        <v>2.3026480839999999</v>
+        <v>1.75663843</v>
       </c>
       <c r="X28">
-        <v>0.29341244799999999</v>
+        <v>0.25274846499999998</v>
       </c>
       <c r="Y28">
-        <v>12.7423921196983</v>
+        <v>14.388189435204399</v>
       </c>
       <c r="Z28">
         <v>0</v>
       </c>
       <c r="AA28" s="76">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>-1.5067938000000503E-2</v>
       </c>
       <c r="AB28" s="61">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>-5.5439702369999964</v>
       </c>
       <c r="AC28" s="77">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>-0.24722222199999999</v>
       </c>
       <c r="AD28" s="77" t="e">
         <f t="shared" si="21"/>
@@ -4746,19 +4746,19 @@
       </c>
       <c r="AE28" s="15">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>-0.19354020106288994</v>
       </c>
       <c r="AF28" s="15">
         <f t="shared" si="23"/>
-        <v>7.5336137000000303E-2</v>
+        <v>0.6213457910000002</v>
       </c>
       <c r="AG28" s="15">
         <f t="shared" si="24"/>
-        <v>3.2236280000000339E-3</v>
+        <v>4.3887611000000049E-2</v>
       </c>
       <c r="AH28" s="77">
         <f t="shared" si="25"/>
-        <v>-0.26812616871329986</v>
+        <v>-1.9139234842193993</v>
       </c>
       <c r="AI28" s="78">
         <f t="shared" si="26"/>
@@ -4815,43 +4815,43 @@
         <v>0</v>
       </c>
       <c r="R29">
-        <v>5.5330544770000003</v>
+        <v>6.4406517320000001</v>
       </c>
       <c r="S29">
-        <v>195.25748501800001</v>
+        <v>292.02788993799999</v>
       </c>
       <c r="T29">
-        <v>0.75</v>
+        <v>0.87462047200000004</v>
       </c>
       <c r="U29">
-        <v>7.8584985747600006E-2</v>
+        <v>-0.130432525732085</v>
       </c>
       <c r="V29">
-        <v>0.71735371254445102</v>
+        <v>0.81882725010500301</v>
       </c>
       <c r="W29">
-        <v>1.0527491440000001</v>
+        <v>1.9874791890000001</v>
       </c>
       <c r="X29">
-        <v>9.7628349000000003E-2</v>
+        <v>0.186758375</v>
       </c>
       <c r="Y29">
-        <v>9.2736574098795899</v>
+        <v>9.39674619153962</v>
       </c>
       <c r="Z29">
         <v>0</v>
       </c>
       <c r="AA29" s="76">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>-0.90759725499999977</v>
       </c>
       <c r="AB29" s="61">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>-96.770404919999976</v>
       </c>
       <c r="AC29" s="77">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>-0.12462047200000004</v>
       </c>
       <c r="AD29" s="77" t="e">
         <f t="shared" si="21"/>
@@ -4859,19 +4859,19 @@
       </c>
       <c r="AE29" s="15">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>-0.101473537560552</v>
       </c>
       <c r="AF29" s="15">
         <f t="shared" si="23"/>
-        <v>2.8672188999999904E-2</v>
+        <v>-0.90605785600000011</v>
       </c>
       <c r="AG29" s="15">
         <f t="shared" si="24"/>
-        <v>6.082619999999983E-4</v>
+        <v>-8.8521764000000003E-2</v>
       </c>
       <c r="AH29" s="77">
         <f t="shared" si="25"/>
-        <v>-0.18962993582568011</v>
+        <v>-0.31271871748571023</v>
       </c>
       <c r="AI29" s="78">
         <f t="shared" si="26"/>
@@ -4928,43 +4928,43 @@
         <v>0</v>
       </c>
       <c r="R30">
-        <v>6.5271280819999999</v>
+        <v>6.066222883</v>
       </c>
       <c r="S30">
-        <v>303.76831997699998</v>
+        <v>262.256762294</v>
       </c>
       <c r="T30">
-        <v>2.755555556</v>
+        <v>2.4138888889999999</v>
       </c>
       <c r="U30">
-        <v>-0.67286029435666905</v>
+        <v>0.132027533976185</v>
       </c>
       <c r="V30">
-        <v>2.3712138058690702</v>
+        <v>2.1162442609188798</v>
       </c>
       <c r="W30">
-        <v>2.0268362500000001</v>
+        <v>2.375416623</v>
       </c>
       <c r="X30">
-        <v>0.35032592600000001</v>
+        <v>0.29620568000000003</v>
       </c>
       <c r="Y30">
-        <v>17.284372430185201</v>
+        <v>12.4696306800241</v>
       </c>
       <c r="Z30">
         <v>0</v>
       </c>
       <c r="AA30" s="76">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>0.46090519899999993</v>
       </c>
       <c r="AB30" s="61">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>41.511557682999978</v>
       </c>
       <c r="AC30" s="77">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>0.34166666700000015</v>
       </c>
       <c r="AD30" s="77" t="e">
         <f t="shared" si="21"/>
@@ -4972,19 +4972,19 @@
       </c>
       <c r="AE30" s="15">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.25496954495019031</v>
       </c>
       <c r="AF30" s="15">
         <f t="shared" si="23"/>
-        <v>5.9503429999998581E-3</v>
+        <v>-0.34263003000000003</v>
       </c>
       <c r="AG30" s="15">
         <f t="shared" si="24"/>
-        <v>-1.843631999999984E-3</v>
+        <v>5.2276613999999999E-2</v>
       </c>
       <c r="AH30" s="77">
         <f t="shared" si="25"/>
-        <v>-0.14128937365499894</v>
+        <v>4.673452376506102</v>
       </c>
       <c r="AI30" s="78">
         <f t="shared" si="26"/>
@@ -5041,43 +5041,43 @@
         <v>0</v>
       </c>
       <c r="R31">
-        <v>5.8756560850000001</v>
+        <v>3.882717033</v>
       </c>
       <c r="S31">
-        <v>236.20028932899999</v>
+        <v>22.972483194999999</v>
       </c>
       <c r="T31">
-        <v>1.2636779440000001</v>
+        <v>0.27612560600000002</v>
       </c>
       <c r="U31">
-        <v>-0.94962831980677498</v>
+        <v>1.1580457717705699E-2</v>
       </c>
       <c r="V31">
-        <v>1.17784230917874</v>
+        <v>0.267413700757753</v>
       </c>
       <c r="W31">
-        <v>2.0268362500000001</v>
+        <v>1.574017268</v>
       </c>
       <c r="X31">
-        <v>0.35032592600000001</v>
+        <v>0.22515321399999999</v>
       </c>
       <c r="Y31">
-        <v>17.284372430185201</v>
+        <v>14.3043674664438</v>
       </c>
       <c r="Z31">
         <v>0</v>
       </c>
       <c r="AA31" s="76">
         <f t="shared" si="18"/>
-        <v>-0.18752929099999971</v>
+        <v>1.8054097610000004</v>
       </c>
       <c r="AB31" s="61">
         <f t="shared" si="19"/>
-        <v>-19.437507617999984</v>
+        <v>193.79029851600001</v>
       </c>
       <c r="AC31" s="77">
         <f t="shared" si="20"/>
-        <v>-8.6902018000000192E-2</v>
+        <v>0.90065031999999989</v>
       </c>
       <c r="AD31" s="77" t="e">
         <f t="shared" si="21"/>
@@ -5085,19 +5085,19 @@
       </c>
       <c r="AE31" s="15">
         <f t="shared" si="22"/>
-        <v>-7.6128417391299941E-2</v>
+        <v>0.834300191029687</v>
       </c>
       <c r="AF31" s="15">
         <f t="shared" si="23"/>
-        <v>5.9503429999998581E-3</v>
+        <v>0.45876932500000001</v>
       </c>
       <c r="AG31" s="15">
         <f t="shared" si="24"/>
-        <v>-1.843631999999984E-3</v>
+        <v>0.12332908000000004</v>
       </c>
       <c r="AH31" s="77">
         <f t="shared" si="25"/>
-        <v>-0.14128937365499894</v>
+        <v>2.8387155900864016</v>
       </c>
       <c r="AI31" s="78">
         <f t="shared" si="26"/>
@@ -5154,43 +5154,43 @@
         <v>0</v>
       </c>
       <c r="R32">
-        <v>6.3391694750000003</v>
+        <v>5.5138670909999998</v>
       </c>
       <c r="S32">
-        <v>285.260690485</v>
+        <v>194.29889766599999</v>
       </c>
       <c r="T32">
-        <v>2.5194598090000002</v>
+        <v>0.74722222199999999</v>
       </c>
       <c r="U32">
-        <v>-1.6556804240184699</v>
+        <v>-0.17980733360607301</v>
       </c>
       <c r="V32">
-        <v>2.2104979898383301</v>
+        <v>0.71489226811704099</v>
       </c>
       <c r="W32">
-        <v>2.0268362500000001</v>
+        <v>1.083001283</v>
       </c>
       <c r="X32">
-        <v>0.35032592600000001</v>
+        <v>9.8292900000000002E-2</v>
       </c>
       <c r="Y32">
-        <v>17.284372430185201</v>
+        <v>9.0759726274488592</v>
       </c>
       <c r="Z32">
         <v>0</v>
       </c>
       <c r="AA32" s="76">
         <f t="shared" si="18"/>
-        <v>-5.5284721000000481E-2</v>
+        <v>0.77001766299999996</v>
       </c>
       <c r="AB32" s="61">
         <f t="shared" si="19"/>
-        <v>-5.4959465580000142</v>
+        <v>85.465846260999996</v>
       </c>
       <c r="AC32" s="77">
         <f t="shared" si="20"/>
-        <v>-4.4326925000000017E-2</v>
+        <v>1.7279106620000002</v>
       </c>
       <c r="AD32" s="77" t="e">
         <f t="shared" si="21"/>
@@ -5198,19 +5198,19 @@
       </c>
       <c r="AE32" s="15">
         <f t="shared" si="22"/>
-        <v>-3.4258219861410311E-2</v>
+        <v>1.4613475018598789</v>
       </c>
       <c r="AF32" s="15">
         <f t="shared" si="23"/>
-        <v>5.9503429999998581E-3</v>
+        <v>0.94978530999999999</v>
       </c>
       <c r="AG32" s="15">
         <f t="shared" si="24"/>
-        <v>-1.843631999999984E-3</v>
+        <v>0.25018939400000001</v>
       </c>
       <c r="AH32" s="77">
         <f t="shared" si="25"/>
-        <v>-0.14128937365499894</v>
+        <v>8.0671104290813425</v>
       </c>
       <c r="AI32" s="78">
         <f t="shared" si="26"/>
@@ -5267,43 +5267,43 @@
         <v>0</v>
       </c>
       <c r="R33">
-        <v>5.4520720359999997</v>
+        <v>6.4873939959999998</v>
       </c>
       <c r="S33">
-        <v>192.59849264900001</v>
+        <v>304.23354872300001</v>
       </c>
       <c r="T33">
-        <v>1</v>
+        <v>2.752777778</v>
       </c>
       <c r="U33">
-        <v>5.5609422434281198E-3</v>
+        <v>-1.20535528397291</v>
       </c>
       <c r="V33">
-        <v>0.94271945393794498</v>
+        <v>2.3704580397291202</v>
       </c>
       <c r="W33">
-        <v>1.529261596</v>
+        <v>2.0306526709999999</v>
       </c>
       <c r="X33">
-        <v>3.6870298000000003E-2</v>
+        <v>0.34826253899999998</v>
       </c>
       <c r="Y33">
-        <v>2.4109869819813401</v>
+        <v>17.1502760651085</v>
       </c>
       <c r="Z33">
         <v>0</v>
       </c>
       <c r="AA33" s="76">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>-1.0353219600000001</v>
       </c>
       <c r="AB33" s="61">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>-111.635056074</v>
       </c>
       <c r="AC33" s="77">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>-1.752777778</v>
       </c>
       <c r="AD33" s="77" t="e">
         <f t="shared" si="21"/>
@@ -5311,19 +5311,19 @@
       </c>
       <c r="AE33" s="15">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>-1.4277385857911753</v>
       </c>
       <c r="AF33" s="15">
         <f t="shared" si="23"/>
-        <v>6.3029499999989191E-4</v>
+        <v>-0.50076078000000002</v>
       </c>
       <c r="AG33" s="15">
         <f t="shared" si="24"/>
-        <v>-9.7042300000000498E-4</v>
+        <v>-0.31236266400000001</v>
       </c>
       <c r="AH33" s="77">
         <f t="shared" si="25"/>
-        <v>-6.4424116252680186E-2</v>
+        <v>-14.803713199379839</v>
       </c>
       <c r="AI33" s="78">
         <f t="shared" si="26"/>
@@ -5380,43 +5380,43 @@
         <v>0</v>
       </c>
       <c r="R34">
-        <v>5.1927100490000004</v>
+        <v>5.6345304909999996</v>
       </c>
       <c r="S34">
-        <v>170.38030829799999</v>
+        <v>213.42573598499999</v>
       </c>
       <c r="T34">
-        <v>2.6666666669999999</v>
+        <v>1.1627018870000001</v>
       </c>
       <c r="U34">
-        <v>0.27284956105477098</v>
+        <v>-1.42700079613526</v>
       </c>
       <c r="V34">
-        <v>2.2481608348884401</v>
+        <v>1.0895973787439599</v>
       </c>
       <c r="W34">
-        <v>2.5053630259999999</v>
+        <v>2.0306526709999999</v>
       </c>
       <c r="X34">
-        <v>0.202979726</v>
+        <v>0.34826253899999998</v>
       </c>
       <c r="Y34">
-        <v>8.1018089551705597</v>
+        <v>17.1502760651085</v>
       </c>
       <c r="Z34">
         <v>0</v>
       </c>
       <c r="AA34" s="76">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>-0.44182044199999915</v>
       </c>
       <c r="AB34" s="61">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>-43.045427687</v>
       </c>
       <c r="AC34" s="77">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>1.5039647799999998</v>
       </c>
       <c r="AD34" s="77" t="e">
         <f t="shared" si="21"/>
@@ -5424,19 +5424,19 @@
       </c>
       <c r="AE34" s="15">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>1.1585634561444802</v>
       </c>
       <c r="AF34" s="15">
         <f t="shared" si="23"/>
-        <v>-5.9773853999999904E-2</v>
+        <v>0.41493650100000012</v>
       </c>
       <c r="AG34" s="15">
         <f t="shared" si="24"/>
-        <v>-1.1809254999999991E-2</v>
+        <v>-0.15709206799999997</v>
       </c>
       <c r="AH34" s="77">
         <f t="shared" si="25"/>
-        <v>-0.28485943688081949</v>
+        <v>-9.3333265468187605</v>
       </c>
       <c r="AI34" s="78">
         <f t="shared" si="26"/>
@@ -5493,43 +5493,43 @@
         <v>0</v>
       </c>
       <c r="R35">
-        <v>5.2446407319999997</v>
+        <v>6.2308050130000003</v>
       </c>
       <c r="S35">
-        <v>173.467495181</v>
+        <v>278.67510031799998</v>
       </c>
       <c r="T35">
-        <v>3.25</v>
+        <v>2.4613966469999999</v>
       </c>
       <c r="U35">
-        <v>0.27474344360902198</v>
+        <v>-2.1585909875288598</v>
       </c>
       <c r="V35">
-        <v>2.7293926842105298</v>
+        <v>2.1666686170900702</v>
       </c>
       <c r="W35">
-        <v>1.4520391530000001</v>
+        <v>2.0306526709999999</v>
       </c>
       <c r="X35">
-        <v>6.3781686000000004E-2</v>
+        <v>0.34826253899999998</v>
       </c>
       <c r="Y35">
-        <v>4.3925596543470098</v>
+        <v>17.1502760651085</v>
       </c>
       <c r="Z35">
         <v>0</v>
       </c>
       <c r="AA35" s="76">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>-0.98616428100000064</v>
       </c>
       <c r="AB35" s="61">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>-105.20760513699997</v>
       </c>
       <c r="AC35" s="77">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>0.78860335300000006</v>
       </c>
       <c r="AD35" s="77" t="e">
         <f t="shared" si="21"/>
@@ -5537,19 +5537,19 @@
       </c>
       <c r="AE35" s="15">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.56272406712045964</v>
       </c>
       <c r="AF35" s="15">
         <f t="shared" si="23"/>
-        <v>-3.6732548000000032E-2</v>
+        <v>-0.61534606599999986</v>
       </c>
       <c r="AG35" s="15">
         <f t="shared" si="24"/>
-        <v>-4.2036530000000016E-3</v>
+        <v>-0.28868450599999995</v>
       </c>
       <c r="AH35" s="77">
         <f t="shared" si="25"/>
-        <v>-0.18301009176300997</v>
+        <v>-12.9407265025245</v>
       </c>
       <c r="AI35" s="78">
         <f t="shared" si="26"/>

</xml_diff>

<commit_message>
Update toolbox workflows and reports
Document the new parser, workflow, and roll-rate reporting paths while capturing the generated artifacts needed for the current analysis sweep.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/formatter/risk_diff.xlsx
+++ b/formatter/risk_diff.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hzeng\Desktop\howard-toolbox\formatter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\QR\hzeng\howard-toolbox\formatter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7B1630A-C22A-499C-8ADD-C904AAA776A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE9F34B-D630-4AAC-B067-02B9A3FC6AFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16785" yWindow="-16680" windowWidth="44655" windowHeight="21285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10275" yWindow="-21750" windowWidth="49725" windowHeight="21285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1191" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1058" uniqueCount="314">
   <si>
     <t>Base</t>
   </si>
@@ -975,6 +975,18 @@
   <si>
     <t>83613FAF8</t>
   </si>
+  <si>
+    <t>JPMMT 2025-VIS2 M1</t>
+  </si>
+  <si>
+    <t>46659RAF4</t>
+  </si>
+  <si>
+    <t>NYMT 2025-INV2 B1</t>
+  </si>
+  <si>
+    <t>62957JAJ0</t>
+  </si>
 </sst>
 </file>
 
@@ -1756,7 +1768,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:AI39"/>
+  <dimension ref="B1:AI15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -1945,108 +1957,108 @@
         <v>207</v>
       </c>
       <c r="C4" s="19">
-        <v>46078</v>
+        <v>46161</v>
       </c>
       <c r="D4" s="79" t="s">
-        <v>208</v>
+        <v>19</v>
       </c>
       <c r="E4" s="79" t="s">
-        <v>209</v>
+        <v>20</v>
       </c>
       <c r="F4" t="s">
-        <v>210</v>
+        <v>21</v>
       </c>
       <c r="G4" s="20">
-        <v>13.031689999999999</v>
+        <v>8.0286019999999994</v>
       </c>
       <c r="H4" s="20">
-        <v>105.2</v>
+        <v>100.20417500000001</v>
       </c>
       <c r="I4" s="74">
-        <v>5.619652576</v>
+        <v>5.2787013780000001</v>
       </c>
       <c r="J4" s="63">
-        <v>203.52345899400001</v>
+        <v>161.749348575</v>
       </c>
       <c r="K4" s="75">
-        <v>0.71174820000000005</v>
-      </c>
-      <c r="L4" s="75" t="s">
-        <v>248</v>
+        <v>0.26666666700000002</v>
+      </c>
+      <c r="L4" s="75">
+        <v>0.25934644938696</v>
       </c>
       <c r="M4" s="20">
-        <v>0.67269661216729104</v>
+        <v>0.25934644938696</v>
       </c>
       <c r="N4" s="20">
-        <v>1.348098537</v>
+        <v>5.2435385349999999</v>
       </c>
       <c r="O4" s="20">
-        <v>4.5678831000000003E-2</v>
+        <v>3.0140479440000001</v>
       </c>
       <c r="P4" s="63">
-        <v>3.38838962778282</v>
+        <v>57.481182294772601</v>
       </c>
       <c r="Q4" s="63">
         <v>0</v>
       </c>
       <c r="R4" s="74">
-        <v>5.5838095210000001</v>
+        <v>5.2796413250000001</v>
       </c>
       <c r="S4" s="63">
-        <v>200.87005390600001</v>
+        <v>161.843345081</v>
       </c>
       <c r="T4" s="75">
-        <v>0.70895033299999999</v>
+        <v>0.26666666700000002</v>
       </c>
       <c r="U4" s="75">
-        <v>7.9667938212922895E-2</v>
+        <v>0.25934496541686403</v>
       </c>
       <c r="V4" s="20">
-        <v>0.67033666920151302</v>
+        <v>0.25934513906231699</v>
       </c>
       <c r="W4" s="20">
-        <v>1.349120509</v>
+        <v>6.355260039</v>
       </c>
       <c r="X4" s="20">
-        <v>4.5772753999999999E-2</v>
+        <v>3.5691158199999999</v>
       </c>
       <c r="Y4" s="63">
-        <v>3.3927846841441802</v>
+        <v>56.160028041300997</v>
       </c>
       <c r="Z4" s="63">
         <v>0</v>
       </c>
       <c r="AA4" s="76">
         <f t="shared" ref="AA4" si="0">I4-R4</f>
-        <v>3.5843054999999957E-2</v>
+        <v>-9.3994699999999654E-4</v>
       </c>
       <c r="AB4" s="61">
         <f t="shared" ref="AB4" si="1">J4-S4</f>
-        <v>2.6534050879999995</v>
+        <v>-9.3996505999996316E-2</v>
       </c>
       <c r="AC4" s="77">
         <f t="shared" ref="AC4" si="2">K4-T4</f>
-        <v>2.7978670000000649E-3</v>
-      </c>
-      <c r="AD4" s="77" t="e">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="77">
         <f t="shared" ref="AD4" si="3">L4-U4</f>
-        <v>#VALUE!</v>
+        <v>1.4839700959723423E-6</v>
       </c>
       <c r="AE4" s="15">
         <f t="shared" ref="AE4" si="4">M4-V4</f>
-        <v>2.3599429657780169E-3</v>
+        <v>1.3103246430112847E-6</v>
       </c>
       <c r="AF4" s="15">
         <f t="shared" ref="AF4" si="5">N4-W4</f>
-        <v>-1.0219719999999821E-3</v>
+        <v>-1.1117215040000001</v>
       </c>
       <c r="AG4" s="15">
         <f t="shared" ref="AG4" si="6">O4-X4</f>
-        <v>-9.392299999999576E-5</v>
+        <v>-0.55506787599999985</v>
       </c>
       <c r="AH4" s="77">
         <f t="shared" ref="AH4" si="7">P4-Y4</f>
-        <v>-4.3950563613601723E-3</v>
+        <v>1.3211542534716045</v>
       </c>
       <c r="AI4" s="78">
         <f t="shared" ref="AI4" si="8">Q4-Z4</f>
@@ -2058,111 +2070,111 @@
         <v>207</v>
       </c>
       <c r="C5" s="81">
-        <v>46078</v>
+        <v>46161</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>242</v>
       </c>
       <c r="F5" t="s">
-        <v>33</v>
+        <v>243</v>
       </c>
       <c r="G5">
-        <v>9.6672100000000007</v>
+        <v>8.4376490000000004</v>
       </c>
       <c r="H5">
-        <v>102.796875</v>
+        <v>101.100365</v>
       </c>
       <c r="I5">
-        <v>5.4408795259999998</v>
+        <v>7.4320456159999999</v>
       </c>
       <c r="J5">
-        <v>184.00562770100001</v>
+        <v>341.12813556700002</v>
       </c>
       <c r="K5">
-        <v>0.66944444400000003</v>
-      </c>
-      <c r="L5" t="s">
-        <v>248</v>
+        <v>1.683333333</v>
+      </c>
+      <c r="L5">
+        <v>1.5216896971638101</v>
       </c>
       <c r="M5">
-        <v>0.63915963982368396</v>
+        <v>1.5287060219812201</v>
       </c>
       <c r="N5">
-        <v>0.47426048599999998</v>
+        <v>3.4519561090000002</v>
       </c>
       <c r="O5">
-        <v>1.7420860999999999E-2</v>
+        <v>1.944633195</v>
       </c>
       <c r="P5">
-        <v>3.6732684915268301</v>
+        <v>56.334238721341698</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
       <c r="R5">
-        <v>5.9673139439999998</v>
+        <v>7.4623701259999997</v>
       </c>
       <c r="S5">
-        <v>212.17334095800001</v>
+        <v>344.16443956500001</v>
       </c>
       <c r="T5">
-        <v>6.3374329280000001</v>
+        <v>1.683333333</v>
       </c>
       <c r="U5">
-        <v>0.50461208117763801</v>
+        <v>1.52789555606451</v>
       </c>
       <c r="V5">
-        <v>4.6880088007445799</v>
+        <v>1.5282382175375899</v>
       </c>
       <c r="W5">
-        <v>7.8622499999999999E-4</v>
+        <v>5.1721002220000001</v>
       </c>
       <c r="X5">
-        <v>0</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>248</v>
+        <v>2.832427188</v>
+      </c>
+      <c r="Y5">
+        <v>54.763578941336299</v>
       </c>
       <c r="Z5">
         <v>0</v>
       </c>
       <c r="AA5" s="76">
-        <f t="shared" ref="AA5:AA26" si="9">I5-R5</f>
-        <v>-0.52643441800000002</v>
+        <f t="shared" ref="AA5:AA15" si="9">I5-R5</f>
+        <v>-3.0324509999999805E-2</v>
       </c>
       <c r="AB5" s="61">
-        <f t="shared" ref="AB5:AB26" si="10">J5-S5</f>
-        <v>-28.167713257000003</v>
+        <f t="shared" ref="AB5:AB15" si="10">J5-S5</f>
+        <v>-3.036303997999994</v>
       </c>
       <c r="AC5" s="77">
-        <f t="shared" ref="AC5:AC26" si="11">K5-T5</f>
-        <v>-5.6679884840000003</v>
-      </c>
-      <c r="AD5" s="77" t="e">
-        <f t="shared" ref="AD5:AD26" si="12">L5-U5</f>
-        <v>#VALUE!</v>
+        <f t="shared" ref="AC5:AC15" si="11">K5-T5</f>
+        <v>0</v>
+      </c>
+      <c r="AD5" s="77">
+        <f t="shared" ref="AD5:AD15" si="12">L5-U5</f>
+        <v>-6.2058589006999121E-3</v>
       </c>
       <c r="AE5" s="15">
-        <f t="shared" ref="AE5:AE26" si="13">M5-V5</f>
-        <v>-4.0488491609208959</v>
+        <f t="shared" ref="AE5:AE15" si="13">M5-V5</f>
+        <v>4.6780444363014873E-4</v>
       </c>
       <c r="AF5" s="15">
-        <f t="shared" ref="AF5:AF26" si="14">N5-W5</f>
-        <v>0.47347426100000001</v>
+        <f t="shared" ref="AF5:AF15" si="14">N5-W5</f>
+        <v>-1.7201441129999999</v>
       </c>
       <c r="AG5" s="15">
-        <f t="shared" ref="AG5:AG26" si="15">O5-X5</f>
-        <v>1.7420860999999999E-2</v>
-      </c>
-      <c r="AH5" s="77" t="e">
-        <f t="shared" ref="AH5:AH26" si="16">P5-Y5</f>
-        <v>#VALUE!</v>
+        <f t="shared" ref="AG5:AG15" si="15">O5-X5</f>
+        <v>-0.88779399300000006</v>
+      </c>
+      <c r="AH5" s="77">
+        <f t="shared" ref="AH5:AH15" si="16">P5-Y5</f>
+        <v>1.5706597800053999</v>
       </c>
       <c r="AI5" s="78">
-        <f t="shared" ref="AI5:AI26" si="17">Q5-Z5</f>
+        <f t="shared" ref="AI5:AI15" si="17">Q5-Z5</f>
         <v>0</v>
       </c>
     </row>
@@ -2171,108 +2183,108 @@
         <v>207</v>
       </c>
       <c r="C6" s="81">
-        <v>46078</v>
+        <v>46161</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="F6" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="G6">
-        <v>9.86721</v>
+        <v>3.1720000000000002</v>
       </c>
       <c r="H6">
-        <v>103.28125</v>
+        <v>89.442544999999996</v>
       </c>
       <c r="I6">
-        <v>5.4188675399999999</v>
+        <v>8.951457971</v>
       </c>
       <c r="J6">
-        <v>183.815661038</v>
+        <v>484.10444195999997</v>
       </c>
       <c r="K6">
-        <v>0.75</v>
-      </c>
-      <c r="L6" t="s">
-        <v>248</v>
+        <v>2.016666667</v>
+      </c>
+      <c r="L6">
+        <v>1.8725124559011599</v>
       </c>
       <c r="M6">
-        <v>0.71498202723147297</v>
+        <v>1.8725124559011599</v>
       </c>
       <c r="N6">
-        <v>0.75808340500000004</v>
+        <v>2.1745326089999999</v>
       </c>
       <c r="O6">
-        <v>3.8248566999999997E-2</v>
+        <v>1.309426625</v>
       </c>
       <c r="P6">
-        <v>5.0454299286501296</v>
+        <v>60.216463049600598</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
       <c r="R6">
-        <v>5.4162452859999997</v>
+        <v>8.951457971</v>
       </c>
       <c r="S6">
-        <v>182.37647052700001</v>
+        <v>484.10444195999997</v>
       </c>
       <c r="T6">
-        <v>0.66666666699999999</v>
+        <v>2.016666667</v>
       </c>
       <c r="U6">
-        <v>7.8800858489135997E-2</v>
+        <v>1.8725124559011599</v>
       </c>
       <c r="V6">
-        <v>0.636702160449926</v>
+        <v>1.8725124559011599</v>
       </c>
       <c r="W6">
-        <v>0.47420277900000002</v>
+        <v>3.917410925</v>
       </c>
       <c r="X6">
-        <v>1.7397675000000001E-2</v>
+        <v>1.9769503450000001</v>
       </c>
       <c r="Y6">
-        <v>3.66882603191155</v>
+        <v>50.465738286059398</v>
       </c>
       <c r="Z6">
         <v>0</v>
       </c>
       <c r="AA6" s="76">
         <f t="shared" si="9"/>
-        <v>2.6222540000002681E-3</v>
+        <v>0</v>
       </c>
       <c r="AB6" s="61">
         <f t="shared" si="10"/>
-        <v>1.4391905109999925</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="77">
         <f t="shared" si="11"/>
-        <v>8.3333333000000009E-2</v>
-      </c>
-      <c r="AD6" s="77" t="e">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="77">
         <f t="shared" si="12"/>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
       <c r="AE6" s="15">
         <f t="shared" si="13"/>
-        <v>7.827986678154697E-2</v>
+        <v>0</v>
       </c>
       <c r="AF6" s="15">
         <f t="shared" si="14"/>
-        <v>0.28388062600000002</v>
+        <v>-1.7428783160000001</v>
       </c>
       <c r="AG6" s="15">
         <f t="shared" si="15"/>
-        <v>2.0850891999999996E-2</v>
+        <v>-0.66752372000000015</v>
       </c>
       <c r="AH6" s="77">
         <f t="shared" si="16"/>
-        <v>1.3766038967385796</v>
+        <v>9.7507247635412</v>
       </c>
       <c r="AI6" s="78">
         <f t="shared" si="17"/>
@@ -2284,108 +2296,108 @@
         <v>207</v>
       </c>
       <c r="C7" s="81">
-        <v>46078</v>
+        <v>46161</v>
       </c>
       <c r="D7" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E7" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="F7" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="G7">
-        <v>11.317209999999999</v>
+        <v>4.5528829999999996</v>
       </c>
       <c r="H7">
-        <v>105.2</v>
+        <v>89.095882020000005</v>
       </c>
       <c r="I7">
-        <v>5.4801712609999997</v>
+        <v>6.9066471009999999</v>
       </c>
       <c r="J7">
-        <v>193.89303531100001</v>
+        <v>250.89935509599999</v>
       </c>
       <c r="K7">
-        <v>0.91666666699999999</v>
-      </c>
-      <c r="L7" t="s">
-        <v>248</v>
+        <v>6.1833333330000002</v>
+      </c>
+      <c r="L7">
+        <v>6.5215456912988401</v>
       </c>
       <c r="M7">
-        <v>0.86301258650189405</v>
+        <v>5.1497075363932696</v>
       </c>
       <c r="N7">
-        <v>0.84145916700000001</v>
+        <v>2.5466147619999999</v>
       </c>
       <c r="O7">
-        <v>4.6297505000000003E-2</v>
+        <v>0.89438616500000001</v>
       </c>
       <c r="P7">
-        <v>5.5020501072038401</v>
+        <v>35.120591396304803</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
       <c r="R7">
-        <v>5.394855776</v>
+        <v>6.7816176339999998</v>
       </c>
       <c r="S7">
-        <v>182.37293944699999</v>
+        <v>230.634132897</v>
       </c>
       <c r="T7">
-        <v>0.74722222199999999</v>
+        <v>7.35</v>
       </c>
       <c r="U7">
-        <v>7.9563839515881099E-2</v>
+        <v>6.6449493486927</v>
       </c>
       <c r="V7">
-        <v>0.71255796284418305</v>
+        <v>5.92726547767331</v>
       </c>
       <c r="W7">
-        <v>0.75874397500000001</v>
+        <v>4.6467143450000004</v>
       </c>
       <c r="X7">
-        <v>3.8194080999999998E-2</v>
+        <v>1.490507515</v>
       </c>
       <c r="Y7">
-        <v>5.0338562490726897</v>
+        <v>32.076590130913203</v>
       </c>
       <c r="Z7">
         <v>0</v>
       </c>
       <c r="AA7" s="76">
         <f t="shared" si="9"/>
-        <v>8.5315484999999747E-2</v>
+        <v>0.12502946700000006</v>
       </c>
       <c r="AB7" s="61">
         <f t="shared" si="10"/>
-        <v>11.520095864000012</v>
+        <v>20.265222198999993</v>
       </c>
       <c r="AC7" s="77">
         <f t="shared" si="11"/>
-        <v>0.169444445</v>
-      </c>
-      <c r="AD7" s="77" t="e">
+        <v>-1.1666666669999994</v>
+      </c>
+      <c r="AD7" s="77">
         <f t="shared" si="12"/>
-        <v>#VALUE!</v>
+        <v>-0.12340365739385994</v>
       </c>
       <c r="AE7" s="15">
         <f t="shared" si="13"/>
-        <v>0.15045462365771101</v>
+        <v>-0.77755794128004041</v>
       </c>
       <c r="AF7" s="15">
         <f t="shared" si="14"/>
-        <v>8.2715191999999993E-2</v>
+        <v>-2.1000995830000004</v>
       </c>
       <c r="AG7" s="15">
         <f t="shared" si="15"/>
-        <v>8.1034240000000049E-3</v>
+        <v>-0.59612134999999999</v>
       </c>
       <c r="AH7" s="77">
         <f t="shared" si="16"/>
-        <v>0.46819385813115044</v>
+        <v>3.0440012653916</v>
       </c>
       <c r="AI7" s="78">
         <f t="shared" si="17"/>
@@ -2397,108 +2409,108 @@
         <v>207</v>
       </c>
       <c r="C8" s="81">
-        <v>46078</v>
+        <v>46161</v>
       </c>
       <c r="D8" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E8" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="F8" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="G8">
-        <v>13.167210000000001</v>
+        <v>4.5810779999999998</v>
       </c>
       <c r="H8">
-        <v>108.144531</v>
+        <v>82.665333000000004</v>
       </c>
       <c r="I8">
-        <v>5.3407397970000003</v>
+        <v>7.0356806110000001</v>
       </c>
       <c r="J8">
-        <v>181.72970571100001</v>
+        <v>242.62070497600001</v>
       </c>
       <c r="K8">
-        <v>1.0833333329999999</v>
-      </c>
-      <c r="L8" t="s">
-        <v>248</v>
+        <v>10.1</v>
+      </c>
+      <c r="L8">
+        <v>9.2827023439196594</v>
       </c>
       <c r="M8">
-        <v>0.99981040095315199</v>
+        <v>7.5926080634066997</v>
       </c>
       <c r="N8">
-        <v>0.63884012999999995</v>
+        <v>2.9422173659999999</v>
       </c>
       <c r="O8">
-        <v>3.2704423000000003E-2</v>
+        <v>0.81855409199999996</v>
       </c>
       <c r="P8">
-        <v>5.1193438646379299</v>
+        <v>27.8209931549972</v>
       </c>
       <c r="Q8">
         <v>0</v>
       </c>
       <c r="R8">
-        <v>5.4520652289999996</v>
+        <v>7.0556097900000001</v>
       </c>
       <c r="S8">
-        <v>192.28782708400001</v>
+        <v>242.81741362099999</v>
       </c>
       <c r="T8">
-        <v>0.91388888899999998</v>
+        <v>10.516666667000001</v>
       </c>
       <c r="U8">
-        <v>8.5550964828893905E-2</v>
+        <v>9.1293022166861597</v>
       </c>
       <c r="V8">
-        <v>0.86070366920151897</v>
+        <v>7.7966099840183301</v>
       </c>
       <c r="W8">
-        <v>0.84244585599999999</v>
+        <v>5.0896662040000002</v>
       </c>
       <c r="X8">
-        <v>4.6281238000000002E-2</v>
+        <v>1.395371165</v>
       </c>
       <c r="Y8">
-        <v>5.4936750736417697</v>
+        <v>27.415769700248099</v>
       </c>
       <c r="Z8">
         <v>0</v>
       </c>
       <c r="AA8" s="76">
         <f t="shared" si="9"/>
-        <v>-0.11132543199999922</v>
+        <v>-1.9929179000000019E-2</v>
       </c>
       <c r="AB8" s="61">
         <f t="shared" si="10"/>
-        <v>-10.558121373000006</v>
+        <v>-0.19670864499997265</v>
       </c>
       <c r="AC8" s="77">
         <f t="shared" si="11"/>
-        <v>0.16944444399999992</v>
-      </c>
-      <c r="AD8" s="77" t="e">
+        <v>-0.41666666700000121</v>
+      </c>
+      <c r="AD8" s="77">
         <f t="shared" si="12"/>
-        <v>#VALUE!</v>
+        <v>0.15340012723349972</v>
       </c>
       <c r="AE8" s="15">
         <f t="shared" si="13"/>
-        <v>0.13910673175163302</v>
+        <v>-0.20400192061163036</v>
       </c>
       <c r="AF8" s="15">
         <f t="shared" si="14"/>
-        <v>-0.20360572600000004</v>
+        <v>-2.1474488380000003</v>
       </c>
       <c r="AG8" s="15">
         <f t="shared" si="15"/>
-        <v>-1.3576814999999999E-2</v>
+        <v>-0.57681707300000007</v>
       </c>
       <c r="AH8" s="77">
         <f t="shared" si="16"/>
-        <v>-0.37433120900383976</v>
+        <v>0.40522345474910182</v>
       </c>
       <c r="AI8" s="78">
         <f t="shared" si="17"/>
@@ -2510,108 +2522,108 @@
         <v>207</v>
       </c>
       <c r="C9" s="81">
-        <v>46078</v>
+        <v>46161</v>
       </c>
       <c r="D9" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>40</v>
+        <v>244</v>
       </c>
       <c r="F9" t="s">
-        <v>41</v>
+        <v>245</v>
       </c>
       <c r="G9">
-        <v>14.26721</v>
+        <v>8.3772640000000003</v>
       </c>
       <c r="H9">
-        <v>110.75</v>
+        <v>100.15922500000001</v>
       </c>
       <c r="I9">
-        <v>5.2604561170000004</v>
+        <v>5.7206654480000001</v>
       </c>
       <c r="J9">
-        <v>174.482540986</v>
+        <v>205.94678052899999</v>
       </c>
       <c r="K9">
-        <v>1.25</v>
-      </c>
-      <c r="L9" t="s">
-        <v>248</v>
+        <v>0.26666666700000002</v>
+      </c>
+      <c r="L9">
+        <v>0.25876942937608</v>
       </c>
       <c r="M9">
-        <v>1.1385441805869201</v>
+        <v>0.25876942937608</v>
       </c>
       <c r="N9">
-        <v>0.74471513899999997</v>
+        <v>3.6708201169999999</v>
       </c>
       <c r="O9">
-        <v>3.8970415000000001E-2</v>
+        <v>1.522282082</v>
       </c>
       <c r="P9">
-        <v>5.2329290703461897</v>
+        <v>41.469808747918002</v>
       </c>
       <c r="Q9">
         <v>0</v>
       </c>
       <c r="R9">
-        <v>5.3653236150000003</v>
+        <v>5.7226425890000003</v>
       </c>
       <c r="S9">
-        <v>185.709916792</v>
+        <v>206.14449854899999</v>
       </c>
       <c r="T9">
-        <v>1.080555556</v>
+        <v>0.26666666700000002</v>
       </c>
       <c r="U9">
-        <v>9.8789601760906801E-2</v>
+        <v>0.25879900528384397</v>
       </c>
       <c r="V9">
-        <v>0.99733899337993903</v>
+        <v>0.25876668175098499</v>
       </c>
       <c r="W9">
-        <v>0.63911900300000002</v>
+        <v>5.5904110190000003</v>
       </c>
       <c r="X9">
-        <v>3.2756825000000003E-2</v>
+        <v>2.3421117910000002</v>
       </c>
       <c r="Y9">
-        <v>5.1253091906578803</v>
+        <v>41.895162681955199</v>
       </c>
       <c r="Z9">
         <v>0</v>
       </c>
       <c r="AA9" s="76">
         <f t="shared" si="9"/>
-        <v>-0.10486749799999995</v>
+        <v>-1.9771410000002376E-3</v>
       </c>
       <c r="AB9" s="61">
         <f t="shared" si="10"/>
-        <v>-11.227375805999998</v>
+        <v>-0.19771801999999639</v>
       </c>
       <c r="AC9" s="77">
         <f t="shared" si="11"/>
-        <v>0.16944444400000003</v>
-      </c>
-      <c r="AD9" s="77" t="e">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="77">
         <f t="shared" si="12"/>
-        <v>#VALUE!</v>
+        <v>-2.9575907763979004E-5</v>
       </c>
       <c r="AE9" s="15">
         <f t="shared" si="13"/>
-        <v>0.14120518720698105</v>
+        <v>2.7476250950009273E-6</v>
       </c>
       <c r="AF9" s="15">
         <f t="shared" si="14"/>
-        <v>0.10559613599999995</v>
+        <v>-1.9195909020000004</v>
       </c>
       <c r="AG9" s="15">
         <f t="shared" si="15"/>
-        <v>6.213589999999998E-3</v>
+        <v>-0.81982970900000018</v>
       </c>
       <c r="AH9" s="77">
         <f t="shared" si="16"/>
-        <v>0.10761987968830944</v>
+        <v>-0.42535393403719723</v>
       </c>
       <c r="AI9" s="78">
         <f t="shared" si="17"/>
@@ -2623,108 +2635,108 @@
         <v>207</v>
       </c>
       <c r="C10" s="81">
-        <v>46078</v>
+        <v>46161</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E10" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="F10" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="G10">
-        <v>15.697279999999999</v>
+        <v>4.2162889999999997</v>
       </c>
       <c r="H10">
-        <v>113.25</v>
+        <v>81.015029080000005</v>
       </c>
       <c r="I10">
-        <v>5.2597473170000004</v>
+        <v>7.1192596860000004</v>
       </c>
       <c r="J10">
-        <v>174.78145048900001</v>
+        <v>252.742054795</v>
       </c>
       <c r="K10">
-        <v>1.3333333329999999</v>
-      </c>
-      <c r="L10" t="s">
-        <v>248</v>
+        <v>9.6833333330000002</v>
+      </c>
+      <c r="L10">
+        <v>8.3972186028375404</v>
       </c>
       <c r="M10">
-        <v>1.2018001227373101</v>
+        <v>7.4208454656769103</v>
       </c>
       <c r="N10">
-        <v>0.851537392</v>
+        <v>3.1280382059999998</v>
       </c>
       <c r="O10">
-        <v>5.0165011000000002E-2</v>
+        <v>1.369391609</v>
       </c>
       <c r="P10">
-        <v>5.8911107687447304</v>
+        <v>43.777969411413302</v>
       </c>
       <c r="Q10">
         <v>0</v>
       </c>
       <c r="R10">
-        <v>5.2254814850000004</v>
+        <v>6.9440934309999998</v>
       </c>
       <c r="S10">
-        <v>172.90878689199999</v>
+        <v>227.412671389</v>
       </c>
       <c r="T10">
-        <v>1.247222222</v>
+        <v>11.433333333</v>
       </c>
       <c r="U10">
-        <v>0.114868992325053</v>
+        <v>8.8485718062523304</v>
       </c>
       <c r="V10">
-        <v>1.13650455440181</v>
+        <v>8.35887551964327</v>
       </c>
       <c r="W10">
-        <v>0.74589581100000002</v>
+        <v>5.3645841269999996</v>
       </c>
       <c r="X10">
-        <v>3.8968309E-2</v>
+        <v>2.3566094980000001</v>
       </c>
       <c r="Y10">
-        <v>5.22436356731329</v>
+        <v>43.929024919921801</v>
       </c>
       <c r="Z10">
         <v>0</v>
       </c>
       <c r="AA10" s="76">
         <f t="shared" si="9"/>
-        <v>3.4265831999999996E-2</v>
+        <v>0.1751662550000006</v>
       </c>
       <c r="AB10" s="61">
         <f t="shared" si="10"/>
-        <v>1.8726635970000132</v>
+        <v>25.329383406000005</v>
       </c>
       <c r="AC10" s="77">
         <f t="shared" si="11"/>
-        <v>8.6111110999999907E-2</v>
-      </c>
-      <c r="AD10" s="77" t="e">
+        <v>-1.75</v>
+      </c>
+      <c r="AD10" s="77">
         <f t="shared" si="12"/>
-        <v>#VALUE!</v>
+        <v>-0.45135320341479002</v>
       </c>
       <c r="AE10" s="15">
         <f t="shared" si="13"/>
-        <v>6.5295568335500098E-2</v>
+        <v>-0.93803005396635974</v>
       </c>
       <c r="AF10" s="15">
         <f t="shared" si="14"/>
-        <v>0.10564158099999998</v>
+        <v>-2.2365459209999998</v>
       </c>
       <c r="AG10" s="15">
         <f t="shared" si="15"/>
-        <v>1.1196702000000003E-2</v>
+        <v>-0.98721788900000007</v>
       </c>
       <c r="AH10" s="77">
         <f t="shared" si="16"/>
-        <v>0.66674720143144039</v>
+        <v>-0.1510555085084988</v>
       </c>
       <c r="AI10" s="78">
         <f t="shared" si="17"/>
@@ -2736,108 +2748,108 @@
         <v>207</v>
       </c>
       <c r="C11" s="81">
-        <v>46078</v>
+        <v>46161</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E11" t="s">
-        <v>158</v>
+        <v>310</v>
       </c>
       <c r="F11" t="s">
-        <v>159</v>
+        <v>311</v>
       </c>
       <c r="G11">
-        <v>11.381690000000001</v>
+        <v>6.2039999999999997</v>
       </c>
       <c r="H11">
-        <v>121.65</v>
+        <v>100.3125</v>
       </c>
       <c r="I11">
-        <v>5.2094194150000002</v>
+        <v>5.92082628</v>
       </c>
       <c r="J11">
-        <v>165.01399560199999</v>
+        <v>180.21978446599999</v>
       </c>
       <c r="K11">
-        <v>4.0833333329999997</v>
-      </c>
-      <c r="L11" t="s">
-        <v>248</v>
+        <v>2.1833333330000002</v>
+      </c>
+      <c r="L11">
+        <v>1.9972428281620001</v>
       </c>
       <c r="M11">
-        <v>3.3423688401150899</v>
+        <v>1.9972428281620001</v>
       </c>
       <c r="N11">
-        <v>1.8535593530000001</v>
+        <v>1.5789718800000001</v>
       </c>
       <c r="O11">
-        <v>0.13136051700000001</v>
+        <v>0.93679669899999995</v>
       </c>
       <c r="P11">
-        <v>7.0869334066584901</v>
+        <v>59.329536571607598</v>
       </c>
       <c r="Q11">
         <v>0</v>
       </c>
       <c r="R11">
-        <v>5.3463423859999999</v>
+        <v>5.92082628</v>
       </c>
       <c r="S11">
-        <v>185.56424450399999</v>
+        <v>180.21978446599999</v>
       </c>
       <c r="T11">
-        <v>1.330555556</v>
+        <v>2.1833333330000002</v>
       </c>
       <c r="U11">
-        <v>0.128226546443962</v>
+        <v>1.9972428281620001</v>
       </c>
       <c r="V11">
-        <v>1.1990315888472001</v>
+        <v>1.9972428281620001</v>
       </c>
       <c r="W11">
-        <v>0.85152371900000001</v>
+        <v>3.8436448730000001</v>
       </c>
       <c r="X11">
-        <v>5.0035835000000001E-2</v>
+        <v>2.2343714750000001</v>
       </c>
       <c r="Y11">
-        <v>5.8760353802898599</v>
+        <v>58.131579498811803</v>
       </c>
       <c r="Z11">
         <v>0</v>
       </c>
       <c r="AA11" s="76">
         <f t="shared" si="9"/>
-        <v>-0.13692297099999973</v>
+        <v>0</v>
       </c>
       <c r="AB11" s="61">
         <f t="shared" si="10"/>
-        <v>-20.550248901999993</v>
+        <v>0</v>
       </c>
       <c r="AC11" s="77">
         <f t="shared" si="11"/>
-        <v>2.7527777769999995</v>
-      </c>
-      <c r="AD11" s="77" t="e">
+        <v>0</v>
+      </c>
+      <c r="AD11" s="77">
         <f t="shared" si="12"/>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
       <c r="AE11" s="15">
         <f t="shared" si="13"/>
-        <v>2.1433372512678899</v>
+        <v>0</v>
       </c>
       <c r="AF11" s="15">
         <f t="shared" si="14"/>
-        <v>1.0020356340000001</v>
+        <v>-2.264672993</v>
       </c>
       <c r="AG11" s="15">
         <f t="shared" si="15"/>
-        <v>8.1324682000000009E-2</v>
+        <v>-1.2975747760000003</v>
       </c>
       <c r="AH11" s="77">
         <f t="shared" si="16"/>
-        <v>1.2108980263686302</v>
+        <v>1.1979570727957949</v>
       </c>
       <c r="AI11" s="78">
         <f t="shared" si="17"/>
@@ -2849,108 +2861,108 @@
         <v>207</v>
       </c>
       <c r="C12" s="81">
-        <v>46078</v>
+        <v>46161</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E12" t="s">
-        <v>160</v>
+        <v>312</v>
       </c>
       <c r="F12" t="s">
-        <v>161</v>
+        <v>313</v>
       </c>
       <c r="G12">
-        <v>8.4172100000000007</v>
+        <v>6.9850000000000003</v>
       </c>
       <c r="H12">
-        <v>112.03125</v>
+        <v>99.821854999999999</v>
       </c>
       <c r="I12">
-        <v>5.3547026119999996</v>
+        <v>6.9881732909999998</v>
       </c>
       <c r="J12">
-        <v>173.99358740700001</v>
+        <v>278.648504543</v>
       </c>
       <c r="K12">
-        <v>4.9222222220000003</v>
-      </c>
-      <c r="L12" t="s">
-        <v>248</v>
+        <v>3.35</v>
+      </c>
+      <c r="L12">
+        <v>2.90896442267077</v>
       </c>
       <c r="M12">
-        <v>4.0762860032357002</v>
+        <v>2.90896442267077</v>
       </c>
       <c r="N12">
-        <v>0.34076076500000002</v>
+        <v>1.9556808400000001</v>
       </c>
       <c r="O12">
-        <v>1.34196E-2</v>
+        <v>1.2207347449999999</v>
       </c>
       <c r="P12">
-        <v>3.9381294381118099</v>
+        <v>62.419936833865002</v>
       </c>
       <c r="Q12">
         <v>0</v>
       </c>
       <c r="R12">
-        <v>5.1692215450000001</v>
+        <v>6.9881732909999998</v>
       </c>
       <c r="S12">
-        <v>166.04340361600001</v>
+        <v>278.648504543</v>
       </c>
       <c r="T12">
-        <v>4.0805555560000002</v>
+        <v>3.35</v>
       </c>
       <c r="U12">
-        <v>0.34808256802301901</v>
+        <v>2.90896442267077</v>
       </c>
       <c r="V12">
-        <v>3.3431574278668301</v>
+        <v>2.90896442267077</v>
       </c>
       <c r="W12">
-        <v>1.8558750399999999</v>
+        <v>4.2209505519999997</v>
       </c>
       <c r="X12">
-        <v>0.131505979</v>
+        <v>2.6265234180000001</v>
       </c>
       <c r="Y12">
-        <v>7.0859285332055499</v>
+        <v>62.225875087673899</v>
       </c>
       <c r="Z12">
         <v>0</v>
       </c>
       <c r="AA12" s="76">
         <f t="shared" si="9"/>
-        <v>0.18548106699999956</v>
+        <v>0</v>
       </c>
       <c r="AB12" s="61">
         <f t="shared" si="10"/>
-        <v>7.9501837910000006</v>
+        <v>0</v>
       </c>
       <c r="AC12" s="77">
         <f t="shared" si="11"/>
-        <v>0.84166666600000006</v>
-      </c>
-      <c r="AD12" s="77" t="e">
+        <v>0</v>
+      </c>
+      <c r="AD12" s="77">
         <f t="shared" si="12"/>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
       <c r="AE12" s="15">
         <f t="shared" si="13"/>
-        <v>0.73312857536887011</v>
+        <v>0</v>
       </c>
       <c r="AF12" s="15">
         <f t="shared" si="14"/>
-        <v>-1.515114275</v>
+        <v>-2.2652697119999994</v>
       </c>
       <c r="AG12" s="15">
         <f t="shared" si="15"/>
-        <v>-0.11808637899999999</v>
+        <v>-1.4057886730000002</v>
       </c>
       <c r="AH12" s="77">
         <f t="shared" si="16"/>
-        <v>-3.14779909509374</v>
+        <v>0.19406174619110317</v>
       </c>
       <c r="AI12" s="78">
         <f t="shared" si="17"/>
@@ -2962,108 +2974,108 @@
         <v>207</v>
       </c>
       <c r="C13" s="81">
-        <v>46078</v>
+        <v>46161</v>
       </c>
       <c r="D13" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E13" t="s">
-        <v>211</v>
+        <v>58</v>
       </c>
       <c r="F13" t="s">
-        <v>212</v>
+        <v>59</v>
       </c>
       <c r="G13">
-        <v>9.1672100000000007</v>
+        <v>3.97275</v>
       </c>
       <c r="H13">
-        <v>121.13</v>
+        <v>73.96546764</v>
       </c>
       <c r="I13">
-        <v>5.7344640389999997</v>
+        <v>7.3673832859999999</v>
       </c>
       <c r="J13">
-        <v>189.66058468</v>
+        <v>268.82981236699999</v>
       </c>
       <c r="K13">
-        <v>7.9166666670000003</v>
-      </c>
-      <c r="L13" t="s">
-        <v>248</v>
+        <v>11.516666667000001</v>
+      </c>
+      <c r="L13">
+        <v>10.2161029871101</v>
       </c>
       <c r="M13">
-        <v>5.8429641121109599</v>
+        <v>8.4965253361034403</v>
       </c>
       <c r="N13">
-        <v>0.30650574600000002</v>
+        <v>3.021600764</v>
       </c>
       <c r="O13">
-        <v>1.3517718999999999E-2</v>
+        <v>1.256530189</v>
       </c>
       <c r="P13">
-        <v>4.4102660966101404</v>
+        <v>41.584917636061299</v>
       </c>
       <c r="Q13">
         <v>0</v>
       </c>
       <c r="R13">
-        <v>5.313084506</v>
+        <v>7.2150438890000004</v>
       </c>
       <c r="S13">
-        <v>175.39506898299999</v>
+        <v>249.57467331199999</v>
       </c>
       <c r="T13">
-        <v>4.9194444439999998</v>
+        <v>12.433333333</v>
       </c>
       <c r="U13">
-        <v>0.23048007497907899</v>
+        <v>10.5493344136991</v>
       </c>
       <c r="V13">
-        <v>4.0785157569874402</v>
+        <v>8.9683083033908506</v>
       </c>
       <c r="W13">
-        <v>0.34086098100000001</v>
+        <v>4.1287460459999998</v>
       </c>
       <c r="X13">
-        <v>1.3329967999999999E-2</v>
+        <v>1.761522096</v>
       </c>
       <c r="Y13">
-        <v>3.9106758306255101</v>
+        <v>42.664820659207003</v>
       </c>
       <c r="Z13">
         <v>0</v>
       </c>
       <c r="AA13" s="76">
         <f t="shared" si="9"/>
-        <v>0.42137953299999964</v>
+        <v>0.15233939699999954</v>
       </c>
       <c r="AB13" s="61">
         <f t="shared" si="10"/>
-        <v>14.265515697000012</v>
+        <v>19.255139055000001</v>
       </c>
       <c r="AC13" s="77">
         <f t="shared" si="11"/>
-        <v>2.9972222230000005</v>
-      </c>
-      <c r="AD13" s="77" t="e">
+        <v>-0.91666666599999935</v>
+      </c>
+      <c r="AD13" s="77">
         <f t="shared" si="12"/>
-        <v>#VALUE!</v>
+        <v>-0.33323142658900018</v>
       </c>
       <c r="AE13" s="15">
         <f t="shared" si="13"/>
-        <v>1.7644483551235197</v>
+        <v>-0.47178296728741032</v>
       </c>
       <c r="AF13" s="15">
         <f t="shared" si="14"/>
-        <v>-3.4355234999999984E-2</v>
+        <v>-1.1071452819999998</v>
       </c>
       <c r="AG13" s="15">
         <f t="shared" si="15"/>
-        <v>1.8775099999999989E-4</v>
+        <v>-0.50499190699999996</v>
       </c>
       <c r="AH13" s="77">
         <f t="shared" si="16"/>
-        <v>0.4995902659846303</v>
+        <v>-1.0799030231457039</v>
       </c>
       <c r="AI13" s="78">
         <f t="shared" si="17"/>
@@ -3075,108 +3087,108 @@
         <v>207</v>
       </c>
       <c r="C14" s="81">
-        <v>46078</v>
+        <v>46161</v>
       </c>
       <c r="D14" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E14" t="s">
-        <v>162</v>
+        <v>60</v>
       </c>
       <c r="F14" t="s">
-        <v>163</v>
+        <v>61</v>
       </c>
       <c r="G14">
-        <v>11.167210000000001</v>
+        <v>4.0440750000000003</v>
       </c>
       <c r="H14">
-        <v>103.85</v>
+        <v>76.119342130000007</v>
       </c>
       <c r="I14">
-        <v>5.3485899310000002</v>
+        <v>7.1258707299999999</v>
       </c>
       <c r="J14">
-        <v>174.75661690199999</v>
+        <v>245.046411898</v>
       </c>
       <c r="K14">
-        <v>0.66944444400000003</v>
-      </c>
-      <c r="L14" t="s">
-        <v>248</v>
+        <v>11.433333333</v>
+      </c>
+      <c r="L14">
+        <v>10.094530496436899</v>
       </c>
       <c r="M14">
-        <v>0.63685947424169798</v>
+        <v>8.4760505864345692</v>
       </c>
       <c r="N14">
-        <v>0.334501251</v>
+        <v>3.2774753159999999</v>
       </c>
       <c r="O14">
-        <v>1.3370205E-2</v>
+        <v>1.3168446090000001</v>
       </c>
       <c r="P14">
-        <v>3.99705680024497</v>
+        <v>40.178627816704498</v>
       </c>
       <c r="Q14">
         <v>0</v>
       </c>
       <c r="R14">
-        <v>5.6962580999999997</v>
+        <v>7.0151063239999996</v>
       </c>
       <c r="S14">
-        <v>190.57301950300001</v>
+        <v>230.324818776</v>
       </c>
       <c r="T14">
-        <v>7.9138888889999999</v>
+        <v>12.266666667000001</v>
       </c>
       <c r="U14">
-        <v>0.54706124411788903</v>
+        <v>10.231533163672101</v>
       </c>
       <c r="V14">
-        <v>5.8496912787913899</v>
+        <v>8.9022798416032494</v>
       </c>
       <c r="W14">
-        <v>0.307282895</v>
+        <v>4.8429398470000002</v>
       </c>
       <c r="X14">
-        <v>1.3540638000000001E-2</v>
+        <v>1.93115953</v>
       </c>
       <c r="Y14">
-        <v>4.4065706944084901</v>
+        <v>39.875769491464403</v>
       </c>
       <c r="Z14">
         <v>0</v>
       </c>
       <c r="AA14" s="76">
         <f t="shared" si="9"/>
-        <v>-0.34766816899999942</v>
+        <v>0.11076440600000037</v>
       </c>
       <c r="AB14" s="61">
         <f t="shared" si="10"/>
-        <v>-15.816402601000021</v>
+        <v>14.721593122000002</v>
       </c>
       <c r="AC14" s="77">
         <f t="shared" si="11"/>
-        <v>-7.2444444450000001</v>
-      </c>
-      <c r="AD14" s="77" t="e">
+        <v>-0.83333333400000065</v>
+      </c>
+      <c r="AD14" s="77">
         <f t="shared" si="12"/>
-        <v>#VALUE!</v>
+        <v>-0.13700266723520116</v>
       </c>
       <c r="AE14" s="15">
         <f t="shared" si="13"/>
-        <v>-5.2128318045496922</v>
+        <v>-0.42622925516868015</v>
       </c>
       <c r="AF14" s="15">
         <f t="shared" si="14"/>
-        <v>2.7218355999999999E-2</v>
+        <v>-1.5654645310000004</v>
       </c>
       <c r="AG14" s="15">
         <f t="shared" si="15"/>
-        <v>-1.7043300000000108E-4</v>
+        <v>-0.61431492099999985</v>
       </c>
       <c r="AH14" s="77">
         <f t="shared" si="16"/>
-        <v>-0.40951389416352013</v>
+        <v>0.30285832524009493</v>
       </c>
       <c r="AI14" s="78">
         <f t="shared" si="17"/>
@@ -3188,2823 +3200,111 @@
         <v>207</v>
       </c>
       <c r="C15" s="81">
-        <v>46078</v>
+        <v>46161</v>
       </c>
       <c r="D15" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E15" t="s">
-        <v>164</v>
+        <v>62</v>
       </c>
       <c r="F15" t="s">
-        <v>165</v>
+        <v>63</v>
       </c>
       <c r="G15">
-        <v>11.46721</v>
+        <v>7.7959100000000001</v>
       </c>
       <c r="H15">
-        <v>104.59375</v>
+        <v>100.32828000000001</v>
       </c>
       <c r="I15">
-        <v>5.2493617439999998</v>
+        <v>6.188159754</v>
       </c>
       <c r="J15">
-        <v>166.83586101099999</v>
+        <v>245.319621423</v>
       </c>
       <c r="K15">
-        <v>0.75</v>
-      </c>
-      <c r="L15" t="s">
-        <v>248</v>
+        <v>0.51666666699999997</v>
+      </c>
+      <c r="L15">
+        <v>0.49542620485469901</v>
       </c>
       <c r="M15">
-        <v>0.71210206919628705</v>
+        <v>0.49547601832703497</v>
       </c>
       <c r="N15">
-        <v>0.400685232</v>
+        <v>4.9015214790000003</v>
       </c>
       <c r="O15">
-        <v>2.0067564E-2</v>
+        <v>3.373476863</v>
       </c>
       <c r="P15">
-        <v>5.0083113619720301</v>
+        <v>68.825095992198996</v>
       </c>
       <c r="Q15">
         <v>0</v>
       </c>
       <c r="R15">
-        <v>5.3176337020000002</v>
+        <v>6.1887903770000001</v>
       </c>
       <c r="S15">
-        <v>172.493607406</v>
+        <v>245.38269231500001</v>
       </c>
       <c r="T15">
-        <v>0.66666666699999999</v>
+        <v>0.51666666699999997</v>
       </c>
       <c r="U15">
-        <v>8.1976883004335102E-2</v>
+        <v>0.49508214134638301</v>
       </c>
       <c r="V15">
-        <v>0.63444388348580505</v>
+        <v>0.49547391323761802</v>
       </c>
       <c r="W15">
-        <v>0.33514227600000002</v>
+        <v>6.7357872150000002</v>
       </c>
       <c r="X15">
-        <v>1.336057E-2</v>
+        <v>4.5642936010000001</v>
       </c>
       <c r="Y15">
-        <v>3.98653675073807</v>
+        <v>67.761843646659798</v>
       </c>
       <c r="Z15">
         <v>0</v>
       </c>
       <c r="AA15" s="76">
         <f t="shared" si="9"/>
-        <v>-6.827195800000041E-2</v>
+        <v>-6.3062300000016336E-4</v>
       </c>
       <c r="AB15" s="61">
         <f t="shared" si="10"/>
-        <v>-5.6577463950000038</v>
+        <v>-6.3070892000013146E-2</v>
       </c>
       <c r="AC15" s="77">
         <f t="shared" si="11"/>
-        <v>8.3333333000000009E-2</v>
-      </c>
-      <c r="AD15" s="77" t="e">
+        <v>0</v>
+      </c>
+      <c r="AD15" s="77">
         <f t="shared" si="12"/>
-        <v>#VALUE!</v>
+        <v>3.4406350831600596E-4</v>
       </c>
       <c r="AE15" s="15">
         <f t="shared" si="13"/>
-        <v>7.7658185710481997E-2</v>
+        <v>2.1050894169483136E-6</v>
       </c>
       <c r="AF15" s="15">
         <f t="shared" si="14"/>
-        <v>6.5542955999999986E-2</v>
+        <v>-1.8342657359999999</v>
       </c>
       <c r="AG15" s="15">
         <f t="shared" si="15"/>
-        <v>6.7069939999999991E-3</v>
+        <v>-1.1908167380000001</v>
       </c>
       <c r="AH15" s="77">
         <f t="shared" si="16"/>
-        <v>1.0217746112339601</v>
+        <v>1.0632523455391976</v>
       </c>
       <c r="AI15" s="78">
         <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
-        <v>207</v>
-      </c>
-      <c r="C16" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D16" t="s">
-        <v>31</v>
-      </c>
-      <c r="E16" t="s">
-        <v>168</v>
-      </c>
-      <c r="F16" t="s">
-        <v>169</v>
-      </c>
-      <c r="G16">
-        <v>9.9172100000000007</v>
-      </c>
-      <c r="H16">
-        <v>102.65625</v>
-      </c>
-      <c r="I16">
-        <v>5.3488216470000003</v>
-      </c>
-      <c r="J16">
-        <v>172.76432298700001</v>
-      </c>
-      <c r="K16">
-        <v>0.58333333300000001</v>
-      </c>
-      <c r="L16" t="s">
-        <v>248</v>
-      </c>
-      <c r="M16">
-        <v>0.55975120657534105</v>
-      </c>
-      <c r="N16">
-        <v>0.46536371100000001</v>
-      </c>
-      <c r="O16">
-        <v>2.8633430000000001E-2</v>
-      </c>
-      <c r="P16">
-        <v>6.1529142309938303</v>
-      </c>
-      <c r="Q16">
-        <v>0</v>
-      </c>
-      <c r="R16">
-        <v>5.4615960169999997</v>
-      </c>
-      <c r="S16">
-        <v>189.01540915499999</v>
-      </c>
-      <c r="T16">
-        <v>0.74722222199999999</v>
-      </c>
-      <c r="U16">
-        <v>8.2919137845634303E-2</v>
-      </c>
-      <c r="V16">
-        <v>0.70885907110864099</v>
-      </c>
-      <c r="W16">
-        <v>0.40015246500000001</v>
-      </c>
-      <c r="X16">
-        <v>2.0002501999999998E-2</v>
-      </c>
-      <c r="Y16">
-        <v>4.9987201753211696</v>
-      </c>
-      <c r="Z16">
-        <v>0</v>
-      </c>
-      <c r="AA16" s="76">
-        <f t="shared" si="9"/>
-        <v>-0.11277436999999946</v>
-      </c>
-      <c r="AB16" s="61">
-        <f t="shared" si="10"/>
-        <v>-16.251086167999972</v>
-      </c>
-      <c r="AC16" s="77">
-        <f t="shared" si="11"/>
-        <v>-0.16388888899999998</v>
-      </c>
-      <c r="AD16" s="77" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE16" s="15">
-        <f t="shared" si="13"/>
-        <v>-0.14910786453329994</v>
-      </c>
-      <c r="AF16" s="15">
-        <f t="shared" si="14"/>
-        <v>6.5211246E-2</v>
-      </c>
-      <c r="AG16" s="15">
-        <f t="shared" si="15"/>
-        <v>8.630928000000003E-3</v>
-      </c>
-      <c r="AH16" s="77">
-        <f t="shared" si="16"/>
-        <v>1.1541940556726606</v>
-      </c>
-      <c r="AI16" s="78">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
-        <v>207</v>
-      </c>
-      <c r="C17" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D17" t="s">
-        <v>31</v>
-      </c>
-      <c r="E17" t="s">
-        <v>170</v>
-      </c>
-      <c r="F17" t="s">
-        <v>171</v>
-      </c>
-      <c r="G17">
-        <v>10.667210000000001</v>
-      </c>
-      <c r="H17">
-        <v>104.325</v>
-      </c>
-      <c r="I17">
-        <v>5.3976119889999996</v>
-      </c>
-      <c r="J17">
-        <v>183.83193711600001</v>
-      </c>
-      <c r="K17">
-        <v>0.84166666700000003</v>
-      </c>
-      <c r="L17" t="s">
-        <v>248</v>
-      </c>
-      <c r="M17">
-        <v>0.79595662209441698</v>
-      </c>
-      <c r="N17">
-        <v>0.55875470599999999</v>
-      </c>
-      <c r="O17">
-        <v>4.6741629E-2</v>
-      </c>
-      <c r="P17">
-        <v>8.3653217589186593</v>
-      </c>
-      <c r="Q17">
-        <v>0</v>
-      </c>
-      <c r="R17">
-        <v>5.3210423049999998</v>
-      </c>
-      <c r="S17">
-        <v>170.70106768400001</v>
-      </c>
-      <c r="T17">
-        <v>0.58055555599999997</v>
-      </c>
-      <c r="U17">
-        <v>7.9541993789952206E-2</v>
-      </c>
-      <c r="V17">
-        <v>0.55727185436834503</v>
-      </c>
-      <c r="W17">
-        <v>0.46512917399999998</v>
-      </c>
-      <c r="X17">
-        <v>2.8592039E-2</v>
-      </c>
-      <c r="Y17">
-        <v>6.14711796168692</v>
-      </c>
-      <c r="Z17">
-        <v>0</v>
-      </c>
-      <c r="AA17" s="76">
-        <f t="shared" si="9"/>
-        <v>7.656968399999986E-2</v>
-      </c>
-      <c r="AB17" s="61">
-        <f t="shared" si="10"/>
-        <v>13.130869431999997</v>
-      </c>
-      <c r="AC17" s="77">
-        <f t="shared" si="11"/>
-        <v>0.26111111100000006</v>
-      </c>
-      <c r="AD17" s="77" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE17" s="15">
-        <f t="shared" si="13"/>
-        <v>0.23868476772607194</v>
-      </c>
-      <c r="AF17" s="15">
-        <f t="shared" si="14"/>
-        <v>9.3625532000000011E-2</v>
-      </c>
-      <c r="AG17" s="15">
-        <f t="shared" si="15"/>
-        <v>1.814959E-2</v>
-      </c>
-      <c r="AH17" s="77">
-        <f t="shared" si="16"/>
-        <v>2.2182037972317392</v>
-      </c>
-      <c r="AI17" s="78">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B18" t="s">
-        <v>207</v>
-      </c>
-      <c r="C18" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E18" t="s">
-        <v>172</v>
-      </c>
-      <c r="F18" t="s">
-        <v>173</v>
-      </c>
-      <c r="G18">
-        <v>12.167210000000001</v>
-      </c>
-      <c r="H18">
-        <v>106.632812</v>
-      </c>
-      <c r="I18">
-        <v>5.3262044230000001</v>
-      </c>
-      <c r="J18">
-        <v>179.953175195</v>
-      </c>
-      <c r="K18">
-        <v>1</v>
-      </c>
-      <c r="L18" t="s">
-        <v>248</v>
-      </c>
-      <c r="M18">
-        <v>0.93653116453498397</v>
-      </c>
-      <c r="N18">
-        <v>0.61873915000000002</v>
-      </c>
-      <c r="O18">
-        <v>3.8814409000000001E-2</v>
-      </c>
-      <c r="P18">
-        <v>6.2731457998091802</v>
-      </c>
-      <c r="Q18">
-        <v>0</v>
-      </c>
-      <c r="R18">
-        <v>5.3709643140000001</v>
-      </c>
-      <c r="S18">
-        <v>182.25207087800001</v>
-      </c>
-      <c r="T18">
-        <v>0.83888888900000003</v>
-      </c>
-      <c r="U18">
-        <v>8.2703730649423601E-2</v>
-      </c>
-      <c r="V18">
-        <v>0.79359373592140303</v>
-      </c>
-      <c r="W18">
-        <v>0.55707205000000004</v>
-      </c>
-      <c r="X18">
-        <v>4.6738254E-2</v>
-      </c>
-      <c r="Y18">
-        <v>8.3899836654881508</v>
-      </c>
-      <c r="Z18">
-        <v>0</v>
-      </c>
-      <c r="AA18" s="76">
-        <f t="shared" si="9"/>
-        <v>-4.4759890999999996E-2</v>
-      </c>
-      <c r="AB18" s="61">
-        <f t="shared" si="10"/>
-        <v>-2.298895683000012</v>
-      </c>
-      <c r="AC18" s="77">
-        <f t="shared" si="11"/>
-        <v>0.16111111099999997</v>
-      </c>
-      <c r="AD18" s="77" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE18" s="15">
-        <f t="shared" si="13"/>
-        <v>0.14293742861358094</v>
-      </c>
-      <c r="AF18" s="15">
-        <f t="shared" si="14"/>
-        <v>6.1667099999999975E-2</v>
-      </c>
-      <c r="AG18" s="15">
-        <f t="shared" si="15"/>
-        <v>-7.9238449999999988E-3</v>
-      </c>
-      <c r="AH18" s="77">
-        <f t="shared" si="16"/>
-        <v>-2.1168378656789706</v>
-      </c>
-      <c r="AI18" s="78">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B19" t="s">
-        <v>207</v>
-      </c>
-      <c r="C19" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D19" t="s">
-        <v>31</v>
-      </c>
-      <c r="E19" t="s">
-        <v>178</v>
-      </c>
-      <c r="F19" t="s">
-        <v>179</v>
-      </c>
-      <c r="G19">
-        <v>14.667210000000001</v>
-      </c>
-      <c r="H19">
-        <v>109.613281</v>
-      </c>
-      <c r="I19">
-        <v>5.4499843129999999</v>
-      </c>
-      <c r="J19">
-        <v>192.607225747</v>
-      </c>
-      <c r="K19">
-        <v>1.0833333329999999</v>
-      </c>
-      <c r="L19" t="s">
-        <v>248</v>
-      </c>
-      <c r="M19">
-        <v>0.99298397061939103</v>
-      </c>
-      <c r="N19">
-        <v>0.65777179799999996</v>
-      </c>
-      <c r="O19">
-        <v>4.9748535000000003E-2</v>
-      </c>
-      <c r="P19">
-        <v>7.5631906310461803</v>
-      </c>
-      <c r="Q19">
-        <v>0</v>
-      </c>
-      <c r="R19">
-        <v>5.2952201370000003</v>
-      </c>
-      <c r="S19">
-        <v>178.20755517200001</v>
-      </c>
-      <c r="T19">
-        <v>0.99722222199999999</v>
-      </c>
-      <c r="U19">
-        <v>9.2193597970580604E-2</v>
-      </c>
-      <c r="V19">
-        <v>0.93429121610334098</v>
-      </c>
-      <c r="W19">
-        <v>0.61907869900000001</v>
-      </c>
-      <c r="X19">
-        <v>3.8780278000000001E-2</v>
-      </c>
-      <c r="Y19">
-        <v>6.2641919456511603</v>
-      </c>
-      <c r="Z19">
-        <v>0</v>
-      </c>
-      <c r="AA19" s="76">
-        <f t="shared" si="9"/>
-        <v>0.15476417599999959</v>
-      </c>
-      <c r="AB19" s="61">
-        <f t="shared" si="10"/>
-        <v>14.399670574999988</v>
-      </c>
-      <c r="AC19" s="77">
-        <f t="shared" si="11"/>
-        <v>8.6111110999999907E-2</v>
-      </c>
-      <c r="AD19" s="77" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE19" s="15">
-        <f t="shared" si="13"/>
-        <v>5.869275451605005E-2</v>
-      </c>
-      <c r="AF19" s="15">
-        <f t="shared" si="14"/>
-        <v>3.8693098999999953E-2</v>
-      </c>
-      <c r="AG19" s="15">
-        <f t="shared" si="15"/>
-        <v>1.0968257000000002E-2</v>
-      </c>
-      <c r="AH19" s="77">
-        <f t="shared" si="16"/>
-        <v>1.2989986853950199</v>
-      </c>
-      <c r="AI19" s="78">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B20" t="s">
-        <v>207</v>
-      </c>
-      <c r="C20" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D20" t="s">
-        <v>213</v>
-      </c>
-      <c r="E20" t="s">
-        <v>214</v>
-      </c>
-      <c r="F20" t="s">
-        <v>215</v>
-      </c>
-      <c r="G20">
-        <v>15.667210000000001</v>
-      </c>
-      <c r="H20">
-        <v>114.749475</v>
-      </c>
-      <c r="I20">
-        <v>5.8026868980000001</v>
-      </c>
-      <c r="J20">
-        <v>230.291131103</v>
-      </c>
-      <c r="K20">
-        <v>1.5888888889999999</v>
-      </c>
-      <c r="L20" t="s">
-        <v>248</v>
-      </c>
-      <c r="M20">
-        <v>1.4073854873845799</v>
-      </c>
-      <c r="N20">
-        <v>1.076510273</v>
-      </c>
-      <c r="O20">
-        <v>0.123687517</v>
-      </c>
-      <c r="P20">
-        <v>11.489673633611501</v>
-      </c>
-      <c r="Q20">
-        <v>0</v>
-      </c>
-      <c r="R20">
-        <v>5.4135034390000003</v>
-      </c>
-      <c r="S20">
-        <v>190.47670634100001</v>
-      </c>
-      <c r="T20">
-        <v>1.080555556</v>
-      </c>
-      <c r="U20">
-        <v>0.10512444929005001</v>
-      </c>
-      <c r="V20">
-        <v>0.99086437436354402</v>
-      </c>
-      <c r="W20">
-        <v>0.65657367099999997</v>
-      </c>
-      <c r="X20">
-        <v>4.9667061999999998E-2</v>
-      </c>
-      <c r="Y20">
-        <v>7.5645832590810702</v>
-      </c>
-      <c r="Z20">
-        <v>0</v>
-      </c>
-      <c r="AA20" s="76">
-        <f t="shared" si="9"/>
-        <v>0.38918345899999984</v>
-      </c>
-      <c r="AB20" s="61">
-        <f t="shared" si="10"/>
-        <v>39.814424761999987</v>
-      </c>
-      <c r="AC20" s="77">
-        <f t="shared" si="11"/>
-        <v>0.50833333299999994</v>
-      </c>
-      <c r="AD20" s="77" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE20" s="15">
-        <f t="shared" si="13"/>
-        <v>0.41652111302103589</v>
-      </c>
-      <c r="AF20" s="15">
-        <f t="shared" si="14"/>
-        <v>0.41993660200000005</v>
-      </c>
-      <c r="AG20" s="15">
-        <f t="shared" si="15"/>
-        <v>7.4020454999999999E-2</v>
-      </c>
-      <c r="AH20" s="77">
-        <f t="shared" si="16"/>
-        <v>3.9250903745304306</v>
-      </c>
-      <c r="AI20" s="78">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
-        <v>207</v>
-      </c>
-      <c r="C21" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D21" t="s">
-        <v>213</v>
-      </c>
-      <c r="E21" t="s">
-        <v>216</v>
-      </c>
-      <c r="F21" t="s">
-        <v>217</v>
-      </c>
-      <c r="G21">
-        <v>8.7172099999999997</v>
-      </c>
-      <c r="H21">
-        <v>103.87375</v>
-      </c>
-      <c r="I21">
-        <v>6.690676882</v>
-      </c>
-      <c r="J21">
-        <v>320.62625412699998</v>
-      </c>
-      <c r="K21">
-        <v>2.4166666669999999</v>
-      </c>
-      <c r="L21" t="s">
-        <v>248</v>
-      </c>
-      <c r="M21">
-        <v>2.1530747662426801</v>
-      </c>
-      <c r="N21">
-        <v>0.50455285000000005</v>
-      </c>
-      <c r="O21">
-        <v>7.5881639000000001E-2</v>
-      </c>
-      <c r="P21">
-        <v>15.039383683988699</v>
-      </c>
-      <c r="Q21">
-        <v>0</v>
-      </c>
-      <c r="R21">
-        <v>5.7606618159999998</v>
-      </c>
-      <c r="S21">
-        <v>228.82854234300001</v>
-      </c>
-      <c r="T21">
-        <v>1.5861111109999999</v>
-      </c>
-      <c r="U21">
-        <v>0.14449127980759699</v>
-      </c>
-      <c r="V21">
-        <v>1.40565059665849</v>
-      </c>
-      <c r="W21">
-        <v>1.0772370529999999</v>
-      </c>
-      <c r="X21">
-        <v>0.123706897</v>
-      </c>
-      <c r="Y21">
-        <v>11.483720937326501</v>
-      </c>
-      <c r="Z21">
-        <v>0</v>
-      </c>
-      <c r="AA21" s="76">
-        <f t="shared" si="9"/>
-        <v>0.93001506600000017</v>
-      </c>
-      <c r="AB21" s="61">
-        <f t="shared" si="10"/>
-        <v>91.797711783999972</v>
-      </c>
-      <c r="AC21" s="77">
-        <f t="shared" si="11"/>
-        <v>0.83055555599999997</v>
-      </c>
-      <c r="AD21" s="77" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE21" s="15">
-        <f t="shared" si="13"/>
-        <v>0.74742416958419011</v>
-      </c>
-      <c r="AF21" s="15">
-        <f t="shared" si="14"/>
-        <v>-0.57268420299999989</v>
-      </c>
-      <c r="AG21" s="15">
-        <f t="shared" si="15"/>
-        <v>-4.7825257999999995E-2</v>
-      </c>
-      <c r="AH21" s="77">
-        <f t="shared" si="16"/>
-        <v>3.5556627466621986</v>
-      </c>
-      <c r="AI21" s="78">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
-        <v>207</v>
-      </c>
-      <c r="C22" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D22" t="s">
-        <v>213</v>
-      </c>
-      <c r="E22" t="s">
-        <v>218</v>
-      </c>
-      <c r="F22" t="s">
-        <v>219</v>
-      </c>
-      <c r="G22">
-        <v>6.1672099999999999</v>
-      </c>
-      <c r="H22">
-        <v>100.69</v>
-      </c>
-      <c r="I22">
-        <v>5.2808620849999999</v>
-      </c>
-      <c r="J22">
-        <v>173.14380468600001</v>
-      </c>
-      <c r="K22">
-        <v>0.87837955199999995</v>
-      </c>
-      <c r="L22" t="s">
-        <v>248</v>
-      </c>
-      <c r="M22">
-        <v>0.84239699572946203</v>
-      </c>
-      <c r="N22">
-        <v>0.50455285000000005</v>
-      </c>
-      <c r="O22">
-        <v>7.5881639000000001E-2</v>
-      </c>
-      <c r="P22">
-        <v>15.039383683988699</v>
-      </c>
-      <c r="Q22">
-        <v>0</v>
-      </c>
-      <c r="R22">
-        <v>6.6533275639999996</v>
-      </c>
-      <c r="S22">
-        <v>321.056554914</v>
-      </c>
-      <c r="T22">
-        <v>2.4138888889999999</v>
-      </c>
-      <c r="U22">
-        <v>-1.7368872058628799</v>
-      </c>
-      <c r="V22">
-        <v>2.1518868944271299</v>
-      </c>
-      <c r="W22">
-        <v>0.50234702799999997</v>
-      </c>
-      <c r="X22">
-        <v>7.5873533000000007E-2</v>
-      </c>
-      <c r="Y22">
-        <v>15.1038084771948</v>
-      </c>
-      <c r="Z22">
-        <v>0</v>
-      </c>
-      <c r="AA22" s="76">
-        <f t="shared" si="9"/>
-        <v>-1.3724654789999997</v>
-      </c>
-      <c r="AB22" s="61">
-        <f t="shared" si="10"/>
-        <v>-147.91275022799999</v>
-      </c>
-      <c r="AC22" s="77">
-        <f t="shared" si="11"/>
-        <v>-1.5355093369999999</v>
-      </c>
-      <c r="AD22" s="77" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE22" s="15">
-        <f t="shared" si="13"/>
-        <v>-1.309489898697668</v>
-      </c>
-      <c r="AF22" s="15">
-        <f t="shared" si="14"/>
-        <v>2.2058220000000794E-3</v>
-      </c>
-      <c r="AG22" s="15">
-        <f t="shared" si="15"/>
-        <v>8.1059999999938404E-6</v>
-      </c>
-      <c r="AH22" s="77">
-        <f t="shared" si="16"/>
-        <v>-6.4424793206100617E-2</v>
-      </c>
-      <c r="AI22" s="78">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B23" t="s">
-        <v>207</v>
-      </c>
-      <c r="C23" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D23" t="s">
-        <v>213</v>
-      </c>
-      <c r="E23" t="s">
-        <v>220</v>
-      </c>
-      <c r="F23" t="s">
-        <v>221</v>
-      </c>
-      <c r="G23">
-        <v>6.9172099999999999</v>
-      </c>
-      <c r="H23">
-        <v>102.1896</v>
-      </c>
-      <c r="I23">
-        <v>5.0397363510000002</v>
-      </c>
-      <c r="J23">
-        <v>153.26793232399999</v>
-      </c>
-      <c r="K23">
-        <v>1.349583728</v>
-      </c>
-      <c r="L23" t="s">
-        <v>248</v>
-      </c>
-      <c r="M23">
-        <v>1.27436085570352</v>
-      </c>
-      <c r="N23">
-        <v>0.50455285000000005</v>
-      </c>
-      <c r="O23">
-        <v>7.5881639000000001E-2</v>
-      </c>
-      <c r="P23">
-        <v>15.039383683988699</v>
-      </c>
-      <c r="Q23">
-        <v>0</v>
-      </c>
-      <c r="R23">
-        <v>5.2611168800000003</v>
-      </c>
-      <c r="S23">
-        <v>172.343188441</v>
-      </c>
-      <c r="T23">
-        <v>0.86755764000000002</v>
-      </c>
-      <c r="U23">
-        <v>-0.13760582282252901</v>
-      </c>
-      <c r="V23">
-        <v>0.83240961267255298</v>
-      </c>
-      <c r="W23">
-        <v>0.50234702799999997</v>
-      </c>
-      <c r="X23">
-        <v>7.5873533000000007E-2</v>
-      </c>
-      <c r="Y23">
-        <v>15.1038084771948</v>
-      </c>
-      <c r="Z23">
-        <v>0</v>
-      </c>
-      <c r="AA23" s="76">
-        <f t="shared" si="9"/>
-        <v>-0.22138052900000016</v>
-      </c>
-      <c r="AB23" s="61">
-        <f t="shared" si="10"/>
-        <v>-19.075256117000009</v>
-      </c>
-      <c r="AC23" s="77">
-        <f t="shared" si="11"/>
-        <v>0.48202608800000002</v>
-      </c>
-      <c r="AD23" s="77" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE23" s="15">
-        <f t="shared" si="13"/>
-        <v>0.441951243030967</v>
-      </c>
-      <c r="AF23" s="15">
-        <f t="shared" si="14"/>
-        <v>2.2058220000000794E-3</v>
-      </c>
-      <c r="AG23" s="15">
-        <f t="shared" si="15"/>
-        <v>8.1059999999938404E-6</v>
-      </c>
-      <c r="AH23" s="77">
-        <f t="shared" si="16"/>
-        <v>-6.4424793206100617E-2</v>
-      </c>
-      <c r="AI23" s="78">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B24" t="s">
-        <v>207</v>
-      </c>
-      <c r="C24" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D24" t="s">
-        <v>213</v>
-      </c>
-      <c r="E24" t="s">
-        <v>222</v>
-      </c>
-      <c r="F24" t="s">
-        <v>223</v>
-      </c>
-      <c r="G24">
-        <v>7.5672100000000002</v>
-      </c>
-      <c r="H24">
-        <v>103.25</v>
-      </c>
-      <c r="I24">
-        <v>5.6344793290000004</v>
-      </c>
-      <c r="J24">
-        <v>215.29800565400001</v>
-      </c>
-      <c r="K24">
-        <v>2.10651476</v>
-      </c>
-      <c r="L24" t="s">
-        <v>248</v>
-      </c>
-      <c r="M24">
-        <v>1.9299076552058101</v>
-      </c>
-      <c r="N24">
-        <v>0.50455285000000005</v>
-      </c>
-      <c r="O24">
-        <v>7.5881639000000001E-2</v>
-      </c>
-      <c r="P24">
-        <v>15.039383683988699</v>
-      </c>
-      <c r="Q24">
-        <v>0</v>
-      </c>
-      <c r="R24">
-        <v>5.0015776340000002</v>
-      </c>
-      <c r="S24">
-        <v>151.62071035299999</v>
-      </c>
-      <c r="T24">
-        <v>1.3332607540000001</v>
-      </c>
-      <c r="U24">
-        <v>-0.85145093336308397</v>
-      </c>
-      <c r="V24">
-        <v>1.2599122151373601</v>
-      </c>
-      <c r="W24">
-        <v>0.50234702799999997</v>
-      </c>
-      <c r="X24">
-        <v>7.5873533000000007E-2</v>
-      </c>
-      <c r="Y24">
-        <v>15.1038084771948</v>
-      </c>
-      <c r="Z24">
-        <v>0</v>
-      </c>
-      <c r="AA24" s="76">
-        <f t="shared" si="9"/>
-        <v>0.63290169500000015</v>
-      </c>
-      <c r="AB24" s="61">
-        <f t="shared" si="10"/>
-        <v>63.677295301000015</v>
-      </c>
-      <c r="AC24" s="77">
-        <f t="shared" si="11"/>
-        <v>0.77325400599999994</v>
-      </c>
-      <c r="AD24" s="77" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE24" s="15">
-        <f t="shared" si="13"/>
-        <v>0.66999544006845002</v>
-      </c>
-      <c r="AF24" s="15">
-        <f t="shared" si="14"/>
-        <v>2.2058220000000794E-3</v>
-      </c>
-      <c r="AG24" s="15">
-        <f t="shared" si="15"/>
-        <v>8.1059999999938404E-6</v>
-      </c>
-      <c r="AH24" s="77">
-        <f t="shared" si="16"/>
-        <v>-6.4424793206100617E-2</v>
-      </c>
-      <c r="AI24" s="78">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B25" t="s">
-        <v>207</v>
-      </c>
-      <c r="C25" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D25" t="s">
-        <v>213</v>
-      </c>
-      <c r="E25" t="s">
-        <v>224</v>
-      </c>
-      <c r="F25" t="s">
-        <v>225</v>
-      </c>
-      <c r="G25">
-        <v>8.86721</v>
-      </c>
-      <c r="H25">
-        <v>106.25</v>
-      </c>
-      <c r="I25">
-        <v>5.9510107220000004</v>
-      </c>
-      <c r="J25">
-        <v>246.43036474100001</v>
-      </c>
-      <c r="K25">
-        <v>2.5833333330000001</v>
-      </c>
-      <c r="L25" t="s">
-        <v>248</v>
-      </c>
-      <c r="M25">
-        <v>2.2971036668235398</v>
-      </c>
-      <c r="N25">
-        <v>1.9857295079999999</v>
-      </c>
-      <c r="O25">
-        <v>0.240699844</v>
-      </c>
-      <c r="P25">
-        <v>12.121481955638</v>
-      </c>
-      <c r="Q25">
-        <v>0</v>
-      </c>
-      <c r="R25">
-        <v>5.5870382999999997</v>
-      </c>
-      <c r="S25">
-        <v>214.39269253399999</v>
-      </c>
-      <c r="T25">
-        <v>2.0876789740000001</v>
-      </c>
-      <c r="U25">
-        <v>-1.4720541491525401</v>
-      </c>
-      <c r="V25">
-        <v>1.9147745975786901</v>
-      </c>
-      <c r="W25">
-        <v>0.50234702799999997</v>
-      </c>
-      <c r="X25">
-        <v>7.5873533000000007E-2</v>
-      </c>
-      <c r="Y25">
-        <v>15.1038084771948</v>
-      </c>
-      <c r="Z25">
-        <v>0</v>
-      </c>
-      <c r="AA25" s="76">
-        <f t="shared" si="9"/>
-        <v>0.36397242200000068</v>
-      </c>
-      <c r="AB25" s="61">
-        <f t="shared" si="10"/>
-        <v>32.037672207000014</v>
-      </c>
-      <c r="AC25" s="77">
-        <f t="shared" si="11"/>
-        <v>0.49565435899999999</v>
-      </c>
-      <c r="AD25" s="77" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE25" s="15">
-        <f t="shared" si="13"/>
-        <v>0.38232906924484977</v>
-      </c>
-      <c r="AF25" s="15">
-        <f t="shared" si="14"/>
-        <v>1.4833824799999999</v>
-      </c>
-      <c r="AG25" s="15">
-        <f t="shared" si="15"/>
-        <v>0.164826311</v>
-      </c>
-      <c r="AH25" s="77">
-        <f t="shared" si="16"/>
-        <v>-2.9823265215568</v>
-      </c>
-      <c r="AI25" s="78">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B26" t="s">
-        <v>207</v>
-      </c>
-      <c r="C26" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D26" t="s">
-        <v>213</v>
-      </c>
-      <c r="E26" t="s">
-        <v>226</v>
-      </c>
-      <c r="F26" t="s">
-        <v>227</v>
-      </c>
-      <c r="G26">
-        <v>10.917210000000001</v>
-      </c>
-      <c r="H26">
-        <v>111</v>
-      </c>
-      <c r="I26">
-        <v>6.1598139950000004</v>
-      </c>
-      <c r="J26">
-        <v>267.15818930900002</v>
-      </c>
-      <c r="K26">
-        <v>2.6666666669999999</v>
-      </c>
-      <c r="L26" t="s">
-        <v>248</v>
-      </c>
-      <c r="M26">
-        <v>2.3117724765765701</v>
-      </c>
-      <c r="N26">
-        <v>1.756665369</v>
-      </c>
-      <c r="O26">
-        <v>0.25225651999999998</v>
-      </c>
-      <c r="P26">
-        <v>14.359964308034399</v>
-      </c>
-      <c r="Q26">
-        <v>0</v>
-      </c>
-      <c r="R26">
-        <v>5.9858454559999998</v>
-      </c>
-      <c r="S26">
-        <v>254.17028324</v>
-      </c>
-      <c r="T26">
-        <v>2.5805555560000002</v>
-      </c>
-      <c r="U26">
-        <v>0.134929649971605</v>
-      </c>
-      <c r="V26">
-        <v>2.2581962830210101</v>
-      </c>
-      <c r="W26">
-        <v>1.915477533</v>
-      </c>
-      <c r="X26">
-        <v>0.23445213600000001</v>
-      </c>
-      <c r="Y26">
-        <v>12.2398791925689</v>
-      </c>
-      <c r="Z26">
-        <v>0</v>
-      </c>
-      <c r="AA26" s="76">
-        <f t="shared" si="9"/>
-        <v>0.17396853900000053</v>
-      </c>
-      <c r="AB26" s="61">
-        <f t="shared" si="10"/>
-        <v>12.987906069000019</v>
-      </c>
-      <c r="AC26" s="77">
-        <f t="shared" si="11"/>
-        <v>8.6111110999999685E-2</v>
-      </c>
-      <c r="AD26" s="77" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE26" s="15">
-        <f t="shared" si="13"/>
-        <v>5.3576193555560092E-2</v>
-      </c>
-      <c r="AF26" s="15">
-        <f t="shared" si="14"/>
-        <v>-0.15881216399999998</v>
-      </c>
-      <c r="AG26" s="15">
-        <f t="shared" si="15"/>
-        <v>1.7804383999999979E-2</v>
-      </c>
-      <c r="AH26" s="77">
-        <f t="shared" si="16"/>
-        <v>2.1200851154654998</v>
-      </c>
-      <c r="AI26" s="78">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
-        <v>207</v>
-      </c>
-      <c r="C27" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D27" t="s">
-        <v>213</v>
-      </c>
-      <c r="E27" t="s">
-        <v>228</v>
-      </c>
-      <c r="F27" t="s">
-        <v>229</v>
-      </c>
-      <c r="G27">
-        <v>10.417210000000001</v>
-      </c>
-      <c r="H27">
-        <v>103.26506999999999</v>
-      </c>
-      <c r="I27">
-        <v>6.4740307660000003</v>
-      </c>
-      <c r="J27">
-        <v>293.587943623</v>
-      </c>
-      <c r="K27">
-        <v>0.878609639</v>
-      </c>
-      <c r="L27" t="s">
-        <v>248</v>
-      </c>
-      <c r="M27">
-        <v>0.82216524619602604</v>
-      </c>
-      <c r="N27">
-        <v>1.9886788909999999</v>
-      </c>
-      <c r="O27">
-        <v>0.188220108</v>
-      </c>
-      <c r="P27">
-        <v>9.4645801718825595</v>
-      </c>
-      <c r="Q27">
-        <v>0</v>
-      </c>
-      <c r="R27">
-        <v>5.5811964359999999</v>
-      </c>
-      <c r="S27">
-        <v>213.77086694900001</v>
-      </c>
-      <c r="T27">
-        <v>2.5805555560000002</v>
-      </c>
-      <c r="U27">
-        <v>5.4688688382957797E-2</v>
-      </c>
-      <c r="V27">
-        <v>2.30098428768243</v>
-      </c>
-      <c r="W27">
-        <v>1.98165094</v>
-      </c>
-      <c r="X27">
-        <v>0.239670205</v>
-      </c>
-      <c r="Y27">
-        <v>12.094471340144301</v>
-      </c>
-      <c r="Z27">
-        <v>0</v>
-      </c>
-      <c r="AA27" s="76">
-        <f t="shared" ref="AA27:AA39" si="18">I27-R27</f>
-        <v>0.89283433000000034</v>
-      </c>
-      <c r="AB27" s="61">
-        <f t="shared" ref="AB27:AB39" si="19">J27-S27</f>
-        <v>79.817076673999992</v>
-      </c>
-      <c r="AC27" s="77">
-        <f t="shared" ref="AC27:AC39" si="20">K27-T27</f>
-        <v>-1.7019459170000002</v>
-      </c>
-      <c r="AD27" s="77" t="e">
-        <f t="shared" ref="AD27:AD39" si="21">L27-U27</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE27" s="15">
-        <f t="shared" ref="AE27:AE39" si="22">M27-V27</f>
-        <v>-1.478819041486404</v>
-      </c>
-      <c r="AF27" s="15">
-        <f t="shared" ref="AF27:AF39" si="23">N27-W27</f>
-        <v>7.0279509999999767E-3</v>
-      </c>
-      <c r="AG27" s="15">
-        <f t="shared" ref="AG27:AG39" si="24">O27-X27</f>
-        <v>-5.1450097E-2</v>
-      </c>
-      <c r="AH27" s="77">
-        <f t="shared" ref="AH27:AH39" si="25">P27-Y27</f>
-        <v>-2.6298911682617412</v>
-      </c>
-      <c r="AI27" s="78">
-        <f t="shared" ref="AI27:AI39" si="26">Q27-Z27</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B28" t="s">
-        <v>207</v>
-      </c>
-      <c r="C28" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D28" t="s">
-        <v>213</v>
-      </c>
-      <c r="E28" t="s">
-        <v>230</v>
-      </c>
-      <c r="F28" t="s">
-        <v>231</v>
-      </c>
-      <c r="G28">
-        <v>10.917210000000001</v>
-      </c>
-      <c r="H28">
-        <v>110.1875</v>
-      </c>
-      <c r="I28">
-        <v>6.1052259439999998</v>
-      </c>
-      <c r="J28">
-        <v>262.02352718899999</v>
-      </c>
-      <c r="K28">
-        <v>2.4166666669999999</v>
-      </c>
-      <c r="L28" t="s">
-        <v>248</v>
-      </c>
-      <c r="M28">
-        <v>2.11736945479297</v>
-      </c>
-      <c r="N28">
-        <v>2.3779842210000002</v>
-      </c>
-      <c r="O28">
-        <v>0.29663607600000003</v>
-      </c>
-      <c r="P28">
-        <v>12.474265950985</v>
-      </c>
-      <c r="Q28">
-        <v>0</v>
-      </c>
-      <c r="R28">
-        <v>6.1202938820000004</v>
-      </c>
-      <c r="S28">
-        <v>267.56749742599999</v>
-      </c>
-      <c r="T28">
-        <v>2.6638888889999999</v>
-      </c>
-      <c r="U28">
-        <v>-0.13160764504505101</v>
-      </c>
-      <c r="V28">
-        <v>2.3109096558558599</v>
-      </c>
-      <c r="W28">
-        <v>1.75663843</v>
-      </c>
-      <c r="X28">
-        <v>0.25274846499999998</v>
-      </c>
-      <c r="Y28">
-        <v>14.388189435204399</v>
-      </c>
-      <c r="Z28">
-        <v>0</v>
-      </c>
-      <c r="AA28" s="76">
-        <f t="shared" si="18"/>
-        <v>-1.5067938000000503E-2</v>
-      </c>
-      <c r="AB28" s="61">
-        <f t="shared" si="19"/>
-        <v>-5.5439702369999964</v>
-      </c>
-      <c r="AC28" s="77">
-        <f t="shared" si="20"/>
-        <v>-0.24722222199999999</v>
-      </c>
-      <c r="AD28" s="77" t="e">
-        <f t="shared" si="21"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE28" s="15">
-        <f t="shared" si="22"/>
-        <v>-0.19354020106288994</v>
-      </c>
-      <c r="AF28" s="15">
-        <f t="shared" si="23"/>
-        <v>0.6213457910000002</v>
-      </c>
-      <c r="AG28" s="15">
-        <f t="shared" si="24"/>
-        <v>4.3887611000000049E-2</v>
-      </c>
-      <c r="AH28" s="77">
-        <f t="shared" si="25"/>
-        <v>-1.9139234842193993</v>
-      </c>
-      <c r="AI28" s="78">
-        <f t="shared" si="26"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B29" t="s">
-        <v>207</v>
-      </c>
-      <c r="C29" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D29" t="s">
-        <v>213</v>
-      </c>
-      <c r="E29" t="s">
-        <v>234</v>
-      </c>
-      <c r="F29" t="s">
-        <v>235</v>
-      </c>
-      <c r="G29">
-        <v>8.61721</v>
-      </c>
-      <c r="H29">
-        <v>102.27056</v>
-      </c>
-      <c r="I29">
-        <v>5.5330544770000003</v>
-      </c>
-      <c r="J29">
-        <v>195.25748501800001</v>
-      </c>
-      <c r="K29">
-        <v>0.75</v>
-      </c>
-      <c r="L29" t="s">
-        <v>248</v>
-      </c>
-      <c r="M29">
-        <v>0.71735371254445102</v>
-      </c>
-      <c r="N29">
-        <v>1.081421333</v>
-      </c>
-      <c r="O29">
-        <v>9.8236611000000001E-2</v>
-      </c>
-      <c r="P29">
-        <v>9.0840274740539098</v>
-      </c>
-      <c r="Q29">
-        <v>0</v>
-      </c>
-      <c r="R29">
-        <v>6.4406517320000001</v>
-      </c>
-      <c r="S29">
-        <v>292.02788993799999</v>
-      </c>
-      <c r="T29">
-        <v>0.87462047200000004</v>
-      </c>
-      <c r="U29">
-        <v>-0.130432525732085</v>
-      </c>
-      <c r="V29">
-        <v>0.81882725010500301</v>
-      </c>
-      <c r="W29">
-        <v>1.9874791890000001</v>
-      </c>
-      <c r="X29">
-        <v>0.186758375</v>
-      </c>
-      <c r="Y29">
-        <v>9.39674619153962</v>
-      </c>
-      <c r="Z29">
-        <v>0</v>
-      </c>
-      <c r="AA29" s="76">
-        <f t="shared" si="18"/>
-        <v>-0.90759725499999977</v>
-      </c>
-      <c r="AB29" s="61">
-        <f t="shared" si="19"/>
-        <v>-96.770404919999976</v>
-      </c>
-      <c r="AC29" s="77">
-        <f t="shared" si="20"/>
-        <v>-0.12462047200000004</v>
-      </c>
-      <c r="AD29" s="77" t="e">
-        <f t="shared" si="21"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE29" s="15">
-        <f t="shared" si="22"/>
-        <v>-0.101473537560552</v>
-      </c>
-      <c r="AF29" s="15">
-        <f t="shared" si="23"/>
-        <v>-0.90605785600000011</v>
-      </c>
-      <c r="AG29" s="15">
-        <f t="shared" si="24"/>
-        <v>-8.8521764000000003E-2</v>
-      </c>
-      <c r="AH29" s="77">
-        <f t="shared" si="25"/>
-        <v>-0.31271871748571023</v>
-      </c>
-      <c r="AI29" s="78">
-        <f t="shared" si="26"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B30" t="s">
-        <v>207</v>
-      </c>
-      <c r="C30" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D30" t="s">
-        <v>213</v>
-      </c>
-      <c r="E30" t="s">
-        <v>236</v>
-      </c>
-      <c r="F30" t="s">
-        <v>237</v>
-      </c>
-      <c r="G30">
-        <v>11.067209999999999</v>
-      </c>
-      <c r="H30">
-        <v>110.75</v>
-      </c>
-      <c r="I30">
-        <v>6.5271280819999999</v>
-      </c>
-      <c r="J30">
-        <v>303.76831997699998</v>
-      </c>
-      <c r="K30">
-        <v>2.755555556</v>
-      </c>
-      <c r="L30" t="s">
-        <v>248</v>
-      </c>
-      <c r="M30">
-        <v>2.3712138058690702</v>
-      </c>
-      <c r="N30">
-        <v>2.032786593</v>
-      </c>
-      <c r="O30">
-        <v>0.34848229400000003</v>
-      </c>
-      <c r="P30">
-        <v>17.143083056530202</v>
-      </c>
-      <c r="Q30">
-        <v>0</v>
-      </c>
-      <c r="R30">
-        <v>6.066222883</v>
-      </c>
-      <c r="S30">
-        <v>262.256762294</v>
-      </c>
-      <c r="T30">
-        <v>2.4138888889999999</v>
-      </c>
-      <c r="U30">
-        <v>0.132027533976185</v>
-      </c>
-      <c r="V30">
-        <v>2.1162442609188798</v>
-      </c>
-      <c r="W30">
-        <v>2.375416623</v>
-      </c>
-      <c r="X30">
-        <v>0.29620568000000003</v>
-      </c>
-      <c r="Y30">
-        <v>12.4696306800241</v>
-      </c>
-      <c r="Z30">
-        <v>0</v>
-      </c>
-      <c r="AA30" s="76">
-        <f t="shared" si="18"/>
-        <v>0.46090519899999993</v>
-      </c>
-      <c r="AB30" s="61">
-        <f t="shared" si="19"/>
-        <v>41.511557682999978</v>
-      </c>
-      <c r="AC30" s="77">
-        <f t="shared" si="20"/>
-        <v>0.34166666700000015</v>
-      </c>
-      <c r="AD30" s="77" t="e">
-        <f t="shared" si="21"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE30" s="15">
-        <f t="shared" si="22"/>
-        <v>0.25496954495019031</v>
-      </c>
-      <c r="AF30" s="15">
-        <f t="shared" si="23"/>
-        <v>-0.34263003000000003</v>
-      </c>
-      <c r="AG30" s="15">
-        <f t="shared" si="24"/>
-        <v>5.2276613999999999E-2</v>
-      </c>
-      <c r="AH30" s="77">
-        <f t="shared" si="25"/>
-        <v>4.673452376506102</v>
-      </c>
-      <c r="AI30" s="78">
-        <f t="shared" si="26"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B31" t="s">
-        <v>207</v>
-      </c>
-      <c r="C31" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D31" t="s">
-        <v>213</v>
-      </c>
-      <c r="E31" t="s">
-        <v>238</v>
-      </c>
-      <c r="F31" t="s">
-        <v>239</v>
-      </c>
-      <c r="G31">
-        <v>8.9172100000000007</v>
-      </c>
-      <c r="H31">
-        <v>103.5</v>
-      </c>
-      <c r="I31">
-        <v>5.6881267940000004</v>
-      </c>
-      <c r="J31">
-        <v>216.762781711</v>
-      </c>
-      <c r="K31">
-        <v>1.1767759259999999</v>
-      </c>
-      <c r="L31" t="s">
-        <v>248</v>
-      </c>
-      <c r="M31">
-        <v>1.1017138917874401</v>
-      </c>
-      <c r="N31">
-        <v>2.032786593</v>
-      </c>
-      <c r="O31">
-        <v>0.34848229400000003</v>
-      </c>
-      <c r="P31">
-        <v>17.143083056530202</v>
-      </c>
-      <c r="Q31">
-        <v>0</v>
-      </c>
-      <c r="R31">
-        <v>3.882717033</v>
-      </c>
-      <c r="S31">
-        <v>22.972483194999999</v>
-      </c>
-      <c r="T31">
-        <v>0.27612560600000002</v>
-      </c>
-      <c r="U31">
-        <v>1.1580457717705699E-2</v>
-      </c>
-      <c r="V31">
-        <v>0.267413700757753</v>
-      </c>
-      <c r="W31">
-        <v>1.574017268</v>
-      </c>
-      <c r="X31">
-        <v>0.22515321399999999</v>
-      </c>
-      <c r="Y31">
-        <v>14.3043674664438</v>
-      </c>
-      <c r="Z31">
-        <v>0</v>
-      </c>
-      <c r="AA31" s="76">
-        <f t="shared" si="18"/>
-        <v>1.8054097610000004</v>
-      </c>
-      <c r="AB31" s="61">
-        <f t="shared" si="19"/>
-        <v>193.79029851600001</v>
-      </c>
-      <c r="AC31" s="77">
-        <f t="shared" si="20"/>
-        <v>0.90065031999999989</v>
-      </c>
-      <c r="AD31" s="77" t="e">
-        <f t="shared" si="21"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE31" s="15">
-        <f t="shared" si="22"/>
-        <v>0.834300191029687</v>
-      </c>
-      <c r="AF31" s="15">
-        <f t="shared" si="23"/>
-        <v>0.45876932500000001</v>
-      </c>
-      <c r="AG31" s="15">
-        <f t="shared" si="24"/>
-        <v>0.12332908000000004</v>
-      </c>
-      <c r="AH31" s="77">
-        <f t="shared" si="25"/>
-        <v>2.8387155900864016</v>
-      </c>
-      <c r="AI31" s="78">
-        <f t="shared" si="26"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B32" t="s">
-        <v>207</v>
-      </c>
-      <c r="C32" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D32" t="s">
-        <v>213</v>
-      </c>
-      <c r="E32" t="s">
-        <v>240</v>
-      </c>
-      <c r="F32" t="s">
-        <v>241</v>
-      </c>
-      <c r="G32">
-        <v>10.167210000000001</v>
-      </c>
-      <c r="H32">
-        <v>108.25</v>
-      </c>
-      <c r="I32">
-        <v>6.2838847539999998</v>
-      </c>
-      <c r="J32">
-        <v>279.76474392699998</v>
-      </c>
-      <c r="K32">
-        <v>2.4751328840000002</v>
-      </c>
-      <c r="L32" t="s">
-        <v>248</v>
-      </c>
-      <c r="M32">
-        <v>2.1762397699769198</v>
-      </c>
-      <c r="N32">
-        <v>2.032786593</v>
-      </c>
-      <c r="O32">
-        <v>0.34848229400000003</v>
-      </c>
-      <c r="P32">
-        <v>17.143083056530202</v>
-      </c>
-      <c r="Q32">
-        <v>0</v>
-      </c>
-      <c r="R32">
-        <v>5.5138670909999998</v>
-      </c>
-      <c r="S32">
-        <v>194.29889766599999</v>
-      </c>
-      <c r="T32">
-        <v>0.74722222199999999</v>
-      </c>
-      <c r="U32">
-        <v>-0.17980733360607301</v>
-      </c>
-      <c r="V32">
-        <v>0.71489226811704099</v>
-      </c>
-      <c r="W32">
-        <v>1.083001283</v>
-      </c>
-      <c r="X32">
-        <v>9.8292900000000002E-2</v>
-      </c>
-      <c r="Y32">
-        <v>9.0759726274488592</v>
-      </c>
-      <c r="Z32">
-        <v>0</v>
-      </c>
-      <c r="AA32" s="76">
-        <f t="shared" si="18"/>
-        <v>0.77001766299999996</v>
-      </c>
-      <c r="AB32" s="61">
-        <f t="shared" si="19"/>
-        <v>85.465846260999996</v>
-      </c>
-      <c r="AC32" s="77">
-        <f t="shared" si="20"/>
-        <v>1.7279106620000002</v>
-      </c>
-      <c r="AD32" s="77" t="e">
-        <f t="shared" si="21"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE32" s="15">
-        <f t="shared" si="22"/>
-        <v>1.4613475018598789</v>
-      </c>
-      <c r="AF32" s="15">
-        <f t="shared" si="23"/>
-        <v>0.94978530999999999</v>
-      </c>
-      <c r="AG32" s="15">
-        <f t="shared" si="24"/>
-        <v>0.25018939400000001</v>
-      </c>
-      <c r="AH32" s="77">
-        <f t="shared" si="25"/>
-        <v>8.0671104290813425</v>
-      </c>
-      <c r="AI32" s="78">
-        <f t="shared" si="26"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B33" t="s">
-        <v>207</v>
-      </c>
-      <c r="C33" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D33" t="s">
-        <v>26</v>
-      </c>
-      <c r="E33" t="s">
-        <v>29</v>
-      </c>
-      <c r="F33" t="s">
-        <v>30</v>
-      </c>
-      <c r="G33">
-        <v>10.381690000000001</v>
-      </c>
-      <c r="H33">
-        <v>104.75</v>
-      </c>
-      <c r="I33">
-        <v>5.4520720359999997</v>
-      </c>
-      <c r="J33">
-        <v>192.59849264900001</v>
-      </c>
-      <c r="K33">
-        <v>1</v>
-      </c>
-      <c r="L33" t="s">
-        <v>248</v>
-      </c>
-      <c r="M33">
-        <v>0.94271945393794498</v>
-      </c>
-      <c r="N33">
-        <v>1.5298918909999999</v>
-      </c>
-      <c r="O33">
-        <v>3.5899874999999998E-2</v>
-      </c>
-      <c r="P33">
-        <v>2.3465628657286599</v>
-      </c>
-      <c r="Q33">
-        <v>0</v>
-      </c>
-      <c r="R33">
-        <v>6.4873939959999998</v>
-      </c>
-      <c r="S33">
-        <v>304.23354872300001</v>
-      </c>
-      <c r="T33">
-        <v>2.752777778</v>
-      </c>
-      <c r="U33">
-        <v>-1.20535528397291</v>
-      </c>
-      <c r="V33">
-        <v>2.3704580397291202</v>
-      </c>
-      <c r="W33">
-        <v>2.0306526709999999</v>
-      </c>
-      <c r="X33">
-        <v>0.34826253899999998</v>
-      </c>
-      <c r="Y33">
-        <v>17.1502760651085</v>
-      </c>
-      <c r="Z33">
-        <v>0</v>
-      </c>
-      <c r="AA33" s="76">
-        <f t="shared" si="18"/>
-        <v>-1.0353219600000001</v>
-      </c>
-      <c r="AB33" s="61">
-        <f t="shared" si="19"/>
-        <v>-111.635056074</v>
-      </c>
-      <c r="AC33" s="77">
-        <f t="shared" si="20"/>
-        <v>-1.752777778</v>
-      </c>
-      <c r="AD33" s="77" t="e">
-        <f t="shared" si="21"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE33" s="15">
-        <f t="shared" si="22"/>
-        <v>-1.4277385857911753</v>
-      </c>
-      <c r="AF33" s="15">
-        <f t="shared" si="23"/>
-        <v>-0.50076078000000002</v>
-      </c>
-      <c r="AG33" s="15">
-        <f t="shared" si="24"/>
-        <v>-0.31236266400000001</v>
-      </c>
-      <c r="AH33" s="77">
-        <f t="shared" si="25"/>
-        <v>-14.803713199379839</v>
-      </c>
-      <c r="AI33" s="78">
-        <f t="shared" si="26"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B34" t="s">
-        <v>207</v>
-      </c>
-      <c r="C34" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D34" t="s">
-        <v>26</v>
-      </c>
-      <c r="E34" t="s">
-        <v>140</v>
-      </c>
-      <c r="F34" t="s">
-        <v>141</v>
-      </c>
-      <c r="G34">
-        <v>14.781689999999999</v>
-      </c>
-      <c r="H34">
-        <v>123.25</v>
-      </c>
-      <c r="I34">
-        <v>5.1927100490000004</v>
-      </c>
-      <c r="J34">
-        <v>170.38030829799999</v>
-      </c>
-      <c r="K34">
-        <v>2.6666666669999999</v>
-      </c>
-      <c r="L34" t="s">
-        <v>248</v>
-      </c>
-      <c r="M34">
-        <v>2.2481608348884401</v>
-      </c>
-      <c r="N34">
-        <v>2.445589172</v>
-      </c>
-      <c r="O34">
-        <v>0.19117047100000001</v>
-      </c>
-      <c r="P34">
-        <v>7.8169495182897402</v>
-      </c>
-      <c r="Q34">
-        <v>0</v>
-      </c>
-      <c r="R34">
-        <v>5.6345304909999996</v>
-      </c>
-      <c r="S34">
-        <v>213.42573598499999</v>
-      </c>
-      <c r="T34">
-        <v>1.1627018870000001</v>
-      </c>
-      <c r="U34">
-        <v>-1.42700079613526</v>
-      </c>
-      <c r="V34">
-        <v>1.0895973787439599</v>
-      </c>
-      <c r="W34">
-        <v>2.0306526709999999</v>
-      </c>
-      <c r="X34">
-        <v>0.34826253899999998</v>
-      </c>
-      <c r="Y34">
-        <v>17.1502760651085</v>
-      </c>
-      <c r="Z34">
-        <v>0</v>
-      </c>
-      <c r="AA34" s="76">
-        <f t="shared" si="18"/>
-        <v>-0.44182044199999915</v>
-      </c>
-      <c r="AB34" s="61">
-        <f t="shared" si="19"/>
-        <v>-43.045427687</v>
-      </c>
-      <c r="AC34" s="77">
-        <f t="shared" si="20"/>
-        <v>1.5039647799999998</v>
-      </c>
-      <c r="AD34" s="77" t="e">
-        <f t="shared" si="21"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE34" s="15">
-        <f t="shared" si="22"/>
-        <v>1.1585634561444802</v>
-      </c>
-      <c r="AF34" s="15">
-        <f t="shared" si="23"/>
-        <v>0.41493650100000012</v>
-      </c>
-      <c r="AG34" s="15">
-        <f t="shared" si="24"/>
-        <v>-0.15709206799999997</v>
-      </c>
-      <c r="AH34" s="77">
-        <f t="shared" si="25"/>
-        <v>-9.3333265468187605</v>
-      </c>
-      <c r="AI34" s="78">
-        <f t="shared" si="26"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B35" t="s">
-        <v>207</v>
-      </c>
-      <c r="C35" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D35" t="s">
-        <v>26</v>
-      </c>
-      <c r="E35" t="s">
-        <v>144</v>
-      </c>
-      <c r="F35" t="s">
-        <v>145</v>
-      </c>
-      <c r="G35">
-        <v>12.131690000000001</v>
-      </c>
-      <c r="H35">
-        <v>119.7</v>
-      </c>
-      <c r="I35">
-        <v>5.2446407319999997</v>
-      </c>
-      <c r="J35">
-        <v>173.467495181</v>
-      </c>
-      <c r="K35">
-        <v>3.25</v>
-      </c>
-      <c r="L35" t="s">
-        <v>248</v>
-      </c>
-      <c r="M35">
-        <v>2.7293926842105298</v>
-      </c>
-      <c r="N35">
-        <v>1.4153066050000001</v>
-      </c>
-      <c r="O35">
-        <v>5.9578033000000002E-2</v>
-      </c>
-      <c r="P35">
-        <v>4.2095495625839998</v>
-      </c>
-      <c r="Q35">
-        <v>0</v>
-      </c>
-      <c r="R35">
-        <v>6.2308050130000003</v>
-      </c>
-      <c r="S35">
-        <v>278.67510031799998</v>
-      </c>
-      <c r="T35">
-        <v>2.4613966469999999</v>
-      </c>
-      <c r="U35">
-        <v>-2.1585909875288598</v>
-      </c>
-      <c r="V35">
-        <v>2.1666686170900702</v>
-      </c>
-      <c r="W35">
-        <v>2.0306526709999999</v>
-      </c>
-      <c r="X35">
-        <v>0.34826253899999998</v>
-      </c>
-      <c r="Y35">
-        <v>17.1502760651085</v>
-      </c>
-      <c r="Z35">
-        <v>0</v>
-      </c>
-      <c r="AA35" s="76">
-        <f t="shared" si="18"/>
-        <v>-0.98616428100000064</v>
-      </c>
-      <c r="AB35" s="61">
-        <f t="shared" si="19"/>
-        <v>-105.20760513699997</v>
-      </c>
-      <c r="AC35" s="77">
-        <f t="shared" si="20"/>
-        <v>0.78860335300000006</v>
-      </c>
-      <c r="AD35" s="77" t="e">
-        <f t="shared" si="21"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE35" s="15">
-        <f t="shared" si="22"/>
-        <v>0.56272406712045964</v>
-      </c>
-      <c r="AF35" s="15">
-        <f t="shared" si="23"/>
-        <v>-0.61534606599999986</v>
-      </c>
-      <c r="AG35" s="15">
-        <f t="shared" si="24"/>
-        <v>-0.28868450599999995</v>
-      </c>
-      <c r="AH35" s="77">
-        <f t="shared" si="25"/>
-        <v>-12.9407265025245</v>
-      </c>
-      <c r="AI35" s="78">
-        <f t="shared" si="26"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B36" t="s">
-        <v>207</v>
-      </c>
-      <c r="C36" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D36" t="s">
-        <v>26</v>
-      </c>
-      <c r="E36" t="s">
-        <v>146</v>
-      </c>
-      <c r="F36" t="s">
-        <v>147</v>
-      </c>
-      <c r="G36">
-        <v>8.6117600000000003</v>
-      </c>
-      <c r="H36">
-        <v>110.3</v>
-      </c>
-      <c r="I36">
-        <v>5.2947931739999996</v>
-      </c>
-      <c r="J36">
-        <v>174.79483713900001</v>
-      </c>
-      <c r="K36">
-        <v>3.8361111110000001</v>
-      </c>
-      <c r="L36" t="s">
-        <v>248</v>
-      </c>
-      <c r="M36">
-        <v>3.2869579048050701</v>
-      </c>
-      <c r="N36">
-        <v>1.1277756969999999</v>
-      </c>
-      <c r="O36">
-        <v>4.3666781000000002E-2</v>
-      </c>
-      <c r="P36">
-        <v>3.8719384640188799</v>
-      </c>
-      <c r="Q36">
-        <v>0</v>
-      </c>
-      <c r="R36">
-        <v>5.2947931739999996</v>
-      </c>
-      <c r="S36">
-        <v>174.79483713900001</v>
-      </c>
-      <c r="T36">
-        <v>3.8361111110000001</v>
-      </c>
-      <c r="U36">
-        <v>0.17444983771532199</v>
-      </c>
-      <c r="V36">
-        <v>3.2869579048050701</v>
-      </c>
-      <c r="W36">
-        <v>1.1242717440000001</v>
-      </c>
-      <c r="X36">
-        <v>4.3728761999999997E-2</v>
-      </c>
-      <c r="Y36">
-        <v>3.88951890264708</v>
-      </c>
-      <c r="Z36">
-        <v>0</v>
-      </c>
-      <c r="AA36" s="76">
-        <f t="shared" si="18"/>
-        <v>0</v>
-      </c>
-      <c r="AB36" s="61">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="AC36" s="77">
-        <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="AD36" s="77" t="e">
-        <f t="shared" si="21"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE36" s="15">
-        <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
-      <c r="AF36" s="15">
-        <f t="shared" si="23"/>
-        <v>3.5039529999998376E-3</v>
-      </c>
-      <c r="AG36" s="15">
-        <f t="shared" si="24"/>
-        <v>-6.1980999999995678E-5</v>
-      </c>
-      <c r="AH36" s="77">
-        <f t="shared" si="25"/>
-        <v>-1.7580438628200135E-2</v>
-      </c>
-      <c r="AI36" s="78">
-        <f t="shared" si="26"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B37" t="s">
-        <v>207</v>
-      </c>
-      <c r="C37" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D37" t="s">
-        <v>26</v>
-      </c>
-      <c r="E37" t="s">
-        <v>148</v>
-      </c>
-      <c r="F37" t="s">
-        <v>149</v>
-      </c>
-      <c r="G37">
-        <v>8.7816899999999993</v>
-      </c>
-      <c r="H37">
-        <v>111</v>
-      </c>
-      <c r="I37">
-        <v>5.2954196260000002</v>
-      </c>
-      <c r="J37">
-        <v>174.87053970100001</v>
-      </c>
-      <c r="K37">
-        <v>3.8361111110000001</v>
-      </c>
-      <c r="L37" t="s">
-        <v>248</v>
-      </c>
-      <c r="M37">
-        <v>3.2779821990990898</v>
-      </c>
-      <c r="N37">
-        <v>1.4795557930000001</v>
-      </c>
-      <c r="O37">
-        <v>7.0656895999999997E-2</v>
-      </c>
-      <c r="P37">
-        <v>4.7755479269040304</v>
-      </c>
-      <c r="Q37">
-        <v>0</v>
-      </c>
-      <c r="R37">
-        <v>5.2954196260000002</v>
-      </c>
-      <c r="S37">
-        <v>174.87053970100001</v>
-      </c>
-      <c r="T37">
-        <v>3.8361111110000001</v>
-      </c>
-      <c r="U37">
-        <v>0.18514749279279499</v>
-      </c>
-      <c r="V37">
-        <v>3.2779821990990898</v>
-      </c>
-      <c r="W37">
-        <v>1.4932585229999999</v>
-      </c>
-      <c r="X37">
-        <v>7.3713964000000007E-2</v>
-      </c>
-      <c r="Y37">
-        <v>4.9364502438537201</v>
-      </c>
-      <c r="Z37">
-        <v>0</v>
-      </c>
-      <c r="AA37" s="76">
-        <f t="shared" si="18"/>
-        <v>0</v>
-      </c>
-      <c r="AB37" s="61">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="AC37" s="77">
-        <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="AD37" s="77" t="e">
-        <f t="shared" si="21"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE37" s="15">
-        <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
-      <c r="AF37" s="15">
-        <f t="shared" si="23"/>
-        <v>-1.3702729999999885E-2</v>
-      </c>
-      <c r="AG37" s="15">
-        <f t="shared" si="24"/>
-        <v>-3.05706800000001E-3</v>
-      </c>
-      <c r="AH37" s="77">
-        <f t="shared" si="25"/>
-        <v>-0.16090231694968971</v>
-      </c>
-      <c r="AI37" s="78">
-        <f t="shared" si="26"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B38" t="s">
-        <v>207</v>
-      </c>
-      <c r="C38" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D38" t="s">
-        <v>26</v>
-      </c>
-      <c r="E38" t="s">
-        <v>150</v>
-      </c>
-      <c r="F38" t="s">
-        <v>151</v>
-      </c>
-      <c r="G38">
-        <v>16.031690000000001</v>
-      </c>
-      <c r="H38">
-        <v>120.75</v>
-      </c>
-      <c r="I38">
-        <v>5.957967934</v>
-      </c>
-      <c r="J38">
-        <v>247.355988174</v>
-      </c>
-      <c r="K38">
-        <v>2.25</v>
-      </c>
-      <c r="L38" t="s">
-        <v>248</v>
-      </c>
-      <c r="M38">
-        <v>1.90950254575569</v>
-      </c>
-      <c r="N38">
-        <v>3.0766105719999999</v>
-      </c>
-      <c r="O38">
-        <v>0.27250920299999998</v>
-      </c>
-      <c r="P38">
-        <v>8.8574486963051395</v>
-      </c>
-      <c r="Q38">
-        <v>0</v>
-      </c>
-      <c r="R38">
-        <v>4.9425166760000003</v>
-      </c>
-      <c r="S38">
-        <v>146.03668555199999</v>
-      </c>
-      <c r="T38">
-        <v>2</v>
-      </c>
-      <c r="U38">
-        <v>-1.80275420041408</v>
-      </c>
-      <c r="V38">
-        <v>1.7359654550724599</v>
-      </c>
-      <c r="W38">
-        <v>3.1511333979999998</v>
-      </c>
-      <c r="X38">
-        <v>0.280185719</v>
-      </c>
-      <c r="Y38">
-        <v>8.8915854586743794</v>
-      </c>
-      <c r="Z38">
-        <v>0</v>
-      </c>
-      <c r="AA38" s="76">
-        <f t="shared" si="18"/>
-        <v>1.0154512579999997</v>
-      </c>
-      <c r="AB38" s="61">
-        <f t="shared" si="19"/>
-        <v>101.31930262200001</v>
-      </c>
-      <c r="AC38" s="77">
-        <f t="shared" si="20"/>
-        <v>0.25</v>
-      </c>
-      <c r="AD38" s="77" t="e">
-        <f t="shared" si="21"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE38" s="15">
-        <f t="shared" si="22"/>
-        <v>0.17353709068323009</v>
-      </c>
-      <c r="AF38" s="15">
-        <f t="shared" si="23"/>
-        <v>-7.4522825999999931E-2</v>
-      </c>
-      <c r="AG38" s="15">
-        <f t="shared" si="24"/>
-        <v>-7.6765160000000221E-3</v>
-      </c>
-      <c r="AH38" s="77">
-        <f t="shared" si="25"/>
-        <v>-3.4136762369239904E-2</v>
-      </c>
-      <c r="AI38" s="78">
-        <f t="shared" si="26"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B39" t="s">
-        <v>207</v>
-      </c>
-      <c r="C39" s="81">
-        <v>46078</v>
-      </c>
-      <c r="D39" t="s">
-        <v>26</v>
-      </c>
-      <c r="E39" t="s">
-        <v>152</v>
-      </c>
-      <c r="F39" t="s">
-        <v>153</v>
-      </c>
-      <c r="G39">
-        <v>15.06176</v>
-      </c>
-      <c r="H39">
-        <v>119.34</v>
-      </c>
-      <c r="I39">
-        <v>5.6450934339999996</v>
-      </c>
-      <c r="J39">
-        <v>216.099126179</v>
-      </c>
-      <c r="K39">
-        <v>2.25</v>
-      </c>
-      <c r="L39" t="s">
-        <v>248</v>
-      </c>
-      <c r="M39">
-        <v>1.9275998516842701</v>
-      </c>
-      <c r="N39">
-        <v>3.2679609840000001</v>
-      </c>
-      <c r="O39">
-        <v>0.33061795399999999</v>
-      </c>
-      <c r="P39">
-        <v>10.1169492420109</v>
-      </c>
-      <c r="Q39">
-        <v>0</v>
-      </c>
-      <c r="R39">
-        <v>4.6944383600000004</v>
-      </c>
-      <c r="S39">
-        <v>121.265774279</v>
-      </c>
-      <c r="T39">
-        <v>2</v>
-      </c>
-      <c r="U39">
-        <v>-1.6978604725992901</v>
-      </c>
-      <c r="V39">
-        <v>1.7503934179654701</v>
-      </c>
-      <c r="W39">
-        <v>3.3299110729999999</v>
-      </c>
-      <c r="X39">
-        <v>0.349690907</v>
-      </c>
-      <c r="Y39">
-        <v>10.5015088791832</v>
-      </c>
-      <c r="Z39">
-        <v>0</v>
-      </c>
-      <c r="AA39" s="76">
-        <f t="shared" si="18"/>
-        <v>0.95065507399999927</v>
-      </c>
-      <c r="AB39" s="61">
-        <f t="shared" si="19"/>
-        <v>94.833351899999997</v>
-      </c>
-      <c r="AC39" s="77">
-        <f t="shared" si="20"/>
-        <v>0.25</v>
-      </c>
-      <c r="AD39" s="77" t="e">
-        <f t="shared" si="21"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AE39" s="15">
-        <f t="shared" si="22"/>
-        <v>0.17720643371879996</v>
-      </c>
-      <c r="AF39" s="15">
-        <f t="shared" si="23"/>
-        <v>-6.1950088999999764E-2</v>
-      </c>
-      <c r="AG39" s="15">
-        <f t="shared" si="24"/>
-        <v>-1.9072953000000004E-2</v>
-      </c>
-      <c r="AH39" s="77">
-        <f t="shared" si="25"/>
-        <v>-0.38455963717230013</v>
-      </c>
-      <c r="AI39" s="78">
-        <f t="shared" si="26"/>
         <v>0</v>
       </c>
     </row>
@@ -6016,8 +3316,8 @@
     <mergeCell ref="AA2:AI2"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
-  <conditionalFormatting sqref="AA4:AA39">
-    <cfRule type="colorScale" priority="71">
+  <conditionalFormatting sqref="AA4:AA15">
+    <cfRule type="colorScale" priority="76">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="num" val="0"/>
@@ -6028,8 +3328,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB4:AB39">
-    <cfRule type="colorScale" priority="72">
+  <conditionalFormatting sqref="AB4:AB15">
+    <cfRule type="colorScale" priority="77">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -6040,8 +3340,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AC4:AC39">
-    <cfRule type="colorScale" priority="73">
+  <conditionalFormatting sqref="AC4:AC15">
+    <cfRule type="colorScale" priority="78">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -6052,8 +3352,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AD4:AD39">
-    <cfRule type="colorScale" priority="74">
+  <conditionalFormatting sqref="AD4:AD15">
+    <cfRule type="colorScale" priority="79">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -6064,8 +3364,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AF4:AF39">
-    <cfRule type="colorScale" priority="75">
+  <conditionalFormatting sqref="AF4:AF15">
+    <cfRule type="colorScale" priority="80">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="num" val="0"/>

</xml_diff>

<commit_message>
Commit pending toolbox work and stop tracking local runtime artifacts.
Adds monthly tracking review, the FCLS PDF helper, dial risk runbook, and reading notes. Drops generated email assets and formatter output, and untracks hook/log state that does not belong in git.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/formatter/risk_diff.xlsx
+++ b/formatter/risk_diff.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\QR\hzeng\howard-toolbox\formatter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E82AEA9E-1F53-4162-B8CD-2B47A3734224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4849C9AA-6B6B-4045-9011-819DC3CD28BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14490" yWindow="1995" windowWidth="49725" windowHeight="21285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13785" yWindow="-21600" windowWidth="42885" windowHeight="21285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1054" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="312">
   <si>
     <t>Base</t>
   </si>
@@ -976,16 +976,10 @@
     <t>83613FAF8</t>
   </si>
   <si>
-    <t>JPMMT 2025-VIS2 M1</t>
+    <t>JPMMT 2025-7MPR XS</t>
   </si>
   <si>
-    <t>46659RAF4</t>
-  </si>
-  <si>
-    <t>NYMT 2025-INV2 B1</t>
-  </si>
-  <si>
-    <t>62957JAJ0</t>
+    <t>46594CAN8</t>
   </si>
 </sst>
 </file>
@@ -1768,7 +1762,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:AI14"/>
+  <dimension ref="B1:AI17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -1957,108 +1951,108 @@
         <v>207</v>
       </c>
       <c r="C4" s="19">
-        <v>46223</v>
+        <v>46244</v>
       </c>
       <c r="D4" s="79" t="s">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="E4" s="79" t="s">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>66</v>
       </c>
       <c r="G4" s="20">
-        <v>8.0232089999999996</v>
+        <v>3.1339199999999998</v>
       </c>
       <c r="H4" s="20">
-        <v>99.949494999999999</v>
+        <v>5.0312349999999997</v>
       </c>
       <c r="I4" s="74">
-        <v>3.0387057990000002</v>
+        <v>28.352096634999999</v>
       </c>
       <c r="J4" s="63">
-        <v>-66.200768877000002</v>
+        <v>2408.7077967999999</v>
       </c>
       <c r="K4" s="75">
-        <v>9.7222221999999997E-2</v>
+        <v>3.1785993690000001</v>
       </c>
       <c r="L4" s="75">
-        <v>9.6264116191889196E-2</v>
+        <v>-6.0583982262804197</v>
       </c>
       <c r="M4" s="20">
-        <v>9.6264116191889196E-2</v>
+        <v>1.4750646113727599</v>
       </c>
       <c r="N4" s="20">
-        <v>7.9244340600000003</v>
+        <v>0.67536616999999999</v>
       </c>
       <c r="O4" s="20">
-        <v>5.2666429969999999</v>
+        <v>0.21101488600000001</v>
       </c>
       <c r="P4" s="63">
-        <v>66.460809152092295</v>
+        <v>31.244515253110801</v>
       </c>
       <c r="Q4" s="63">
         <v>0</v>
       </c>
       <c r="R4" s="74">
-        <v>3.03817366</v>
+        <v>25.930344369</v>
       </c>
       <c r="S4" s="63">
-        <v>-66.253982726999993</v>
+        <v>2166.9339595299998</v>
       </c>
       <c r="T4" s="75">
-        <v>9.7222221999999997E-2</v>
+        <v>2.9890911720000002</v>
       </c>
       <c r="U4" s="75">
-        <v>9.6264368319218599E-2</v>
+        <v>-21.691342980401402</v>
       </c>
       <c r="V4" s="20">
-        <v>9.6264368319218599E-2</v>
+        <v>1.4770366917864</v>
       </c>
       <c r="W4" s="20">
-        <v>4.9996226110000004</v>
+        <v>0.65824554000000002</v>
       </c>
       <c r="X4" s="20">
-        <v>2.8029477119999999</v>
+        <v>0.206722871</v>
       </c>
       <c r="Y4" s="63">
-        <v>56.063185765922597</v>
+        <v>31.4051305231783</v>
       </c>
       <c r="Z4" s="63">
         <v>0</v>
       </c>
       <c r="AA4" s="76">
         <f t="shared" ref="AA4" si="0">I4-R4</f>
-        <v>5.3213900000015357E-4</v>
+        <v>2.4217522659999986</v>
       </c>
       <c r="AB4" s="61">
         <f t="shared" ref="AB4" si="1">J4-S4</f>
-        <v>5.321384999999168E-2</v>
+        <v>241.77383727000006</v>
       </c>
       <c r="AC4" s="77">
         <f t="shared" ref="AC4" si="2">K4-T4</f>
-        <v>0</v>
+        <v>0.18950819699999988</v>
       </c>
       <c r="AD4" s="77">
         <f t="shared" ref="AD4" si="3">L4-U4</f>
-        <v>-2.5212732940316229E-7</v>
+        <v>15.632944754120981</v>
       </c>
       <c r="AE4" s="15">
         <f t="shared" ref="AE4" si="4">M4-V4</f>
-        <v>-2.5212732940316229E-7</v>
+        <v>-1.9720804136400538E-3</v>
       </c>
       <c r="AF4" s="15">
         <f t="shared" ref="AF4" si="5">N4-W4</f>
-        <v>2.9248114489999999</v>
+        <v>1.712062999999997E-2</v>
       </c>
       <c r="AG4" s="15">
         <f t="shared" ref="AG4" si="6">O4-X4</f>
-        <v>2.463695285</v>
+        <v>4.2920150000000101E-3</v>
       </c>
       <c r="AH4" s="77">
         <f t="shared" ref="AH4" si="7">P4-Y4</f>
-        <v>10.397623386169698</v>
+        <v>-0.16061527006749898</v>
       </c>
       <c r="AI4" s="78">
         <f t="shared" ref="AI4" si="8">Q4-Z4</f>
@@ -2070,111 +2064,111 @@
         <v>207</v>
       </c>
       <c r="C5" s="81">
-        <v>46223</v>
+        <v>46244</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="E5" t="s">
-        <v>242</v>
+        <v>67</v>
       </c>
       <c r="F5" t="s">
-        <v>243</v>
+        <v>68</v>
       </c>
       <c r="G5">
-        <v>8.4221400000000006</v>
+        <v>2.6339199999999998</v>
       </c>
       <c r="H5">
-        <v>100.652215</v>
+        <v>4.1680000000000001</v>
       </c>
       <c r="I5">
-        <v>7.6475104780000001</v>
+        <v>27.540608167999999</v>
       </c>
       <c r="J5">
-        <v>352.63904177699999</v>
+        <v>2327.1595467769998</v>
       </c>
       <c r="K5">
-        <v>1.513888889</v>
+        <v>3.2048381880000001</v>
       </c>
       <c r="L5">
-        <v>1.37851996799077</v>
+        <v>-3.0634552783109501</v>
       </c>
       <c r="M5">
-        <v>1.3826864694433201</v>
+        <v>1.49270527831094</v>
       </c>
       <c r="N5">
-        <v>6.2876212049999998</v>
+        <v>0.50628346899999999</v>
       </c>
       <c r="O5">
-        <v>4.2950626879999998</v>
+        <v>0.143716284</v>
       </c>
       <c r="P5">
-        <v>68.309819373096303</v>
+        <v>28.386525099044899</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
       <c r="R5">
-        <v>7.6625083910000003</v>
+        <v>25.268238836999998</v>
       </c>
       <c r="S5">
-        <v>354.13793241100001</v>
+        <v>2100.1341361740001</v>
       </c>
       <c r="T5">
-        <v>1.513888889</v>
+        <v>3.0326576799999998</v>
       </c>
       <c r="U5">
-        <v>1.3777300413247</v>
+        <v>-21.717796401151599</v>
       </c>
       <c r="V5">
-        <v>1.38266736149136</v>
+        <v>1.5017523032629601</v>
       </c>
       <c r="W5">
-        <v>3.7749449319999999</v>
+        <v>0.47814767899999999</v>
       </c>
       <c r="X5">
-        <v>2.1163715409999999</v>
+        <v>0.13604201099999999</v>
       </c>
       <c r="Y5">
-        <v>56.063640109280399</v>
+        <v>28.4518814949638</v>
       </c>
       <c r="Z5">
         <v>0</v>
       </c>
       <c r="AA5" s="76">
-        <f t="shared" ref="AA5:AA14" si="9">I5-R5</f>
-        <v>-1.4997913000000196E-2</v>
+        <f t="shared" ref="AA5:AA17" si="9">I5-R5</f>
+        <v>2.2723693310000002</v>
       </c>
       <c r="AB5" s="61">
-        <f t="shared" ref="AB5:AB14" si="10">J5-S5</f>
-        <v>-1.4988906340000199</v>
+        <f t="shared" ref="AB5:AB17" si="10">J5-S5</f>
+        <v>227.02541060299973</v>
       </c>
       <c r="AC5" s="77">
-        <f t="shared" ref="AC5:AC14" si="11">K5-T5</f>
-        <v>0</v>
+        <f t="shared" ref="AC5:AC17" si="11">K5-T5</f>
+        <v>0.17218050800000029</v>
       </c>
       <c r="AD5" s="77">
-        <f t="shared" ref="AD5:AD14" si="12">L5-U5</f>
-        <v>7.8992666607002882E-4</v>
+        <f t="shared" ref="AD5:AD17" si="12">L5-U5</f>
+        <v>18.654341122840648</v>
       </c>
       <c r="AE5" s="15">
-        <f t="shared" ref="AE5:AE14" si="13">M5-V5</f>
-        <v>1.9107951960029013E-5</v>
+        <f t="shared" ref="AE5:AE17" si="13">M5-V5</f>
+        <v>-9.047024952020033E-3</v>
       </c>
       <c r="AF5" s="15">
-        <f t="shared" ref="AF5:AF14" si="14">N5-W5</f>
-        <v>2.5126762729999998</v>
+        <f t="shared" ref="AF5:AF17" si="14">N5-W5</f>
+        <v>2.8135789999999994E-2</v>
       </c>
       <c r="AG5" s="15">
-        <f t="shared" ref="AG5:AG14" si="15">O5-X5</f>
-        <v>2.1786911469999999</v>
+        <f t="shared" ref="AG5:AG17" si="15">O5-X5</f>
+        <v>7.6742730000000092E-3</v>
       </c>
       <c r="AH5" s="77">
-        <f t="shared" ref="AH5:AH14" si="16">P5-Y5</f>
-        <v>12.246179263815904</v>
+        <f t="shared" ref="AH5:AH17" si="16">P5-Y5</f>
+        <v>-6.5356395918900745E-2</v>
       </c>
       <c r="AI5" s="78">
-        <f t="shared" ref="AI5:AI14" si="17">Q5-Z5</f>
+        <f t="shared" ref="AI5:AI17" si="17">Q5-Z5</f>
         <v>0</v>
       </c>
     </row>
@@ -2183,108 +2177,108 @@
         <v>207</v>
       </c>
       <c r="C6" s="81">
-        <v>46223</v>
+        <v>46244</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="E6" t="s">
-        <v>22</v>
+        <v>255</v>
       </c>
       <c r="F6" t="s">
-        <v>23</v>
+        <v>256</v>
       </c>
       <c r="G6">
-        <v>3.1720000000000002</v>
+        <v>0.96157000000000004</v>
       </c>
       <c r="H6">
-        <v>87.413394999999994</v>
+        <v>2</v>
       </c>
       <c r="I6">
-        <v>10.190303383</v>
+        <v>13.397001011</v>
       </c>
       <c r="J6">
-        <v>595.95834073100002</v>
+        <v>910.446848768</v>
       </c>
       <c r="K6">
-        <v>2.013888889</v>
+        <v>5.2926728379999997</v>
       </c>
       <c r="L6">
-        <v>1.85819391524605</v>
+        <v>-29.166430699999999</v>
       </c>
       <c r="M6">
-        <v>1.85819391524605</v>
+        <v>1.8676903499999999</v>
       </c>
       <c r="N6">
-        <v>3.510419454</v>
+        <v>1.0135926790000001</v>
       </c>
       <c r="O6">
-        <v>2.1443217290000001</v>
+        <v>0.39916096699999998</v>
       </c>
       <c r="P6">
-        <v>61.0844873981262</v>
+        <v>39.380806044673498</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
       <c r="R6">
-        <v>10.190303383</v>
+        <v>11.455528332</v>
       </c>
       <c r="S6">
-        <v>595.95834073100002</v>
+        <v>716.66786478500001</v>
       </c>
       <c r="T6">
-        <v>2.013888889</v>
+        <v>5.2070867539999997</v>
       </c>
       <c r="U6">
-        <v>1.85819391524605</v>
+        <v>-36.382291100000003</v>
       </c>
       <c r="V6">
-        <v>1.85819391524605</v>
+        <v>1.8672009000000001</v>
       </c>
       <c r="W6">
-        <v>2.2363125469999998</v>
+        <v>1.0005349290000001</v>
       </c>
       <c r="X6">
-        <v>1.3456650240000001</v>
+        <v>0.39564566800000001</v>
       </c>
       <c r="Y6">
-        <v>60.173387919555402</v>
+        <v>39.543413881155999</v>
       </c>
       <c r="Z6">
         <v>0</v>
       </c>
       <c r="AA6" s="76">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1.9414726790000003</v>
       </c>
       <c r="AB6" s="61">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>193.77898398299999</v>
       </c>
       <c r="AC6" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>8.5586084000000007E-2</v>
       </c>
       <c r="AD6" s="77">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>7.2158604000000039</v>
       </c>
       <c r="AE6" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>4.8944999999989136E-4</v>
       </c>
       <c r="AF6" s="15">
         <f t="shared" si="14"/>
-        <v>1.2741069070000002</v>
+        <v>1.3057749999999979E-2</v>
       </c>
       <c r="AG6" s="15">
         <f t="shared" si="15"/>
-        <v>0.79865670499999997</v>
+        <v>3.5152989999999718E-3</v>
       </c>
       <c r="AH6" s="77">
         <f t="shared" si="16"/>
-        <v>0.91109947857079732</v>
+        <v>-0.16260783648250055</v>
       </c>
       <c r="AI6" s="78">
         <f t="shared" si="17"/>
@@ -2296,108 +2290,108 @@
         <v>207</v>
       </c>
       <c r="C7" s="81">
-        <v>46223</v>
+        <v>46244</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="E7" t="s">
-        <v>24</v>
+        <v>77</v>
       </c>
       <c r="F7" t="s">
-        <v>25</v>
+        <v>78</v>
       </c>
       <c r="G7">
-        <v>4.5537770000000002</v>
+        <v>0.2</v>
       </c>
       <c r="H7">
-        <v>90.921644999999998</v>
+        <v>0.789385</v>
       </c>
       <c r="I7">
-        <v>6.6242718319999998</v>
+        <v>11.763895246000001</v>
       </c>
       <c r="J7">
-        <v>221.58459362599999</v>
+        <v>726.37827503899996</v>
       </c>
       <c r="K7">
-        <v>6.5972222220000001</v>
+        <v>6.6159844369999998</v>
       </c>
       <c r="L7">
-        <v>6.5305187450139099</v>
+        <v>-7.9164164507813002</v>
       </c>
       <c r="M7">
-        <v>5.4308988976167196</v>
+        <v>3.5451193017348999</v>
       </c>
       <c r="N7">
-        <v>3.1776884500000002</v>
+        <v>0.92850243200000004</v>
       </c>
       <c r="O7">
-        <v>1.662971961</v>
+        <v>-0.75161785599999997</v>
       </c>
       <c r="P7">
-        <v>52.332756567120398</v>
+        <v>-80.949476285270507</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
       <c r="R7">
-        <v>6.5417857609999999</v>
+        <v>11.763819783000001</v>
       </c>
       <c r="S7">
-        <v>216.15391604999999</v>
+        <v>726.37058537400003</v>
       </c>
       <c r="T7">
-        <v>6.0972222220000001</v>
-      </c>
-      <c r="U7">
-        <v>6.1895764919343401</v>
+        <v>6.6159757739999998</v>
+      </c>
+      <c r="U7" t="s">
+        <v>248</v>
       </c>
       <c r="V7">
-        <v>5.1064579506893004</v>
+        <v>3.5451362769751098</v>
       </c>
       <c r="W7">
-        <v>2.6142159290000002</v>
+        <v>0.92850118999999998</v>
       </c>
       <c r="X7">
-        <v>0.93036471300000001</v>
+        <v>-0.751617906</v>
       </c>
       <c r="Y7">
-        <v>35.588671260062497</v>
+        <v>-80.949589951521801</v>
       </c>
       <c r="Z7">
         <v>0</v>
       </c>
       <c r="AA7" s="76">
         <f t="shared" si="9"/>
-        <v>8.2486070999999939E-2</v>
+        <v>7.5462999999942326E-5</v>
       </c>
       <c r="AB7" s="61">
         <f t="shared" si="10"/>
-        <v>5.4306775759999937</v>
+        <v>7.6896649999298461E-3</v>
       </c>
       <c r="AC7" s="77">
         <f t="shared" si="11"/>
-        <v>0.5</v>
-      </c>
-      <c r="AD7" s="77">
+        <v>8.6630000000198493E-6</v>
+      </c>
+      <c r="AD7" s="77" t="e">
         <f t="shared" si="12"/>
-        <v>0.34094225307956982</v>
+        <v>#VALUE!</v>
       </c>
       <c r="AE7" s="15">
         <f t="shared" si="13"/>
-        <v>0.3244409469274192</v>
+        <v>-1.6975240209937681E-5</v>
       </c>
       <c r="AF7" s="15">
         <f t="shared" si="14"/>
-        <v>0.563472521</v>
+        <v>1.242000000067911E-6</v>
       </c>
       <c r="AG7" s="15">
         <f t="shared" si="15"/>
-        <v>0.73260724799999999</v>
+        <v>5.0000000029193359E-8</v>
       </c>
       <c r="AH7" s="77">
         <f t="shared" si="16"/>
-        <v>16.744085307057901</v>
+        <v>1.1366625129483054E-4</v>
       </c>
       <c r="AI7" s="78">
         <f t="shared" si="17"/>
@@ -2409,84 +2403,84 @@
         <v>207</v>
       </c>
       <c r="C8" s="81">
-        <v>46223</v>
+        <v>46244</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="E8" t="s">
-        <v>48</v>
+        <v>87</v>
       </c>
       <c r="F8" t="s">
-        <v>49</v>
+        <v>88</v>
       </c>
       <c r="G8">
-        <v>4.5782379999999998</v>
+        <v>6.8442470000000002</v>
       </c>
       <c r="H8">
-        <v>83.277945000000003</v>
+        <v>99.064965000000001</v>
       </c>
       <c r="I8">
-        <v>7.1029369459999998</v>
+        <v>7.0933572759999999</v>
       </c>
       <c r="J8">
-        <v>255.09147510099999</v>
+        <v>280.82662080699998</v>
       </c>
       <c r="K8">
-        <v>9.8472222219999992</v>
+        <v>2.7083333330000001</v>
       </c>
       <c r="L8">
-        <v>9.5328052607446203</v>
+        <v>2.3375263182094699</v>
       </c>
       <c r="M8">
-        <v>7.4270967805461598</v>
+        <v>2.4059074941378</v>
       </c>
       <c r="N8">
-        <v>3.946571192</v>
+        <v>0.97363489700000005</v>
       </c>
       <c r="O8">
-        <v>1.6610981579999999</v>
+        <v>0.304171144</v>
       </c>
       <c r="P8">
-        <v>42.089653960054498</v>
+        <v>31.240780803689699</v>
       </c>
       <c r="Q8">
         <v>0</v>
       </c>
       <c r="R8">
-        <v>6.9924218079999996</v>
+        <v>7.0839736240000004</v>
       </c>
       <c r="S8">
-        <v>243.944671422</v>
+        <v>279.88700997000001</v>
       </c>
       <c r="T8">
-        <v>9.8472222219999992</v>
+        <v>2.7083333330000001</v>
       </c>
       <c r="U8">
-        <v>8.8232092350501699</v>
+        <v>2.2863543342492498</v>
       </c>
       <c r="V8">
-        <v>7.46132627552229</v>
+        <v>2.4061960653799299</v>
       </c>
       <c r="W8">
-        <v>3.5627944500000002</v>
+        <v>0.97326000199999996</v>
       </c>
       <c r="X8">
-        <v>1.0934949940000001</v>
+        <v>0.30440088999999998</v>
       </c>
       <c r="Y8">
-        <v>30.6920595433172</v>
+        <v>31.276420419463602</v>
       </c>
       <c r="Z8">
         <v>0</v>
       </c>
       <c r="AA8" s="76">
         <f t="shared" si="9"/>
-        <v>0.11051513800000023</v>
+        <v>9.383651999999465E-3</v>
       </c>
       <c r="AB8" s="61">
         <f t="shared" si="10"/>
-        <v>11.146803678999987</v>
+        <v>0.93961083699997516</v>
       </c>
       <c r="AC8" s="77">
         <f t="shared" si="11"/>
@@ -2494,23 +2488,23 @@
       </c>
       <c r="AD8" s="77">
         <f t="shared" si="12"/>
-        <v>0.70959602569445046</v>
+        <v>5.1171983960220047E-2</v>
       </c>
       <c r="AE8" s="15">
         <f t="shared" si="13"/>
-        <v>-3.4229494976130148E-2</v>
+        <v>-2.8857124212988694E-4</v>
       </c>
       <c r="AF8" s="15">
         <f t="shared" si="14"/>
-        <v>0.38377674199999978</v>
+        <v>3.7489500000009723E-4</v>
       </c>
       <c r="AG8" s="15">
         <f t="shared" si="15"/>
-        <v>0.56760316399999988</v>
+        <v>-2.2974599999997514E-4</v>
       </c>
       <c r="AH8" s="77">
         <f t="shared" si="16"/>
-        <v>11.397594416737299</v>
+        <v>-3.5639615773902733E-2</v>
       </c>
       <c r="AI8" s="78">
         <f t="shared" si="17"/>
@@ -2522,108 +2516,108 @@
         <v>207</v>
       </c>
       <c r="C9" s="81">
-        <v>46223</v>
+        <v>46244</v>
       </c>
       <c r="D9" t="s">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="E9" t="s">
-        <v>50</v>
+        <v>89</v>
       </c>
       <c r="F9" t="s">
-        <v>51</v>
+        <v>90</v>
       </c>
       <c r="G9">
-        <v>4.2040439999999997</v>
+        <v>7.2101240000000004</v>
       </c>
       <c r="H9">
-        <v>82.402709999999999</v>
+        <v>99.595529999999997</v>
       </c>
       <c r="I9">
-        <v>6.9944959129999997</v>
+        <v>7.2474972429999998</v>
       </c>
       <c r="J9">
-        <v>241.288333352</v>
+        <v>300.42376022399998</v>
       </c>
       <c r="K9">
-        <v>10.513888889</v>
+        <v>2.125</v>
       </c>
       <c r="L9">
-        <v>8.64594863202921</v>
+        <v>2.1820061753775399</v>
       </c>
       <c r="M9">
-        <v>7.8646132827427602</v>
+        <v>1.91701705287376</v>
       </c>
       <c r="N9">
-        <v>4.0451204839999999</v>
+        <v>0.94410793000000004</v>
       </c>
       <c r="O9">
-        <v>2.2362909449999999</v>
+        <v>0.32134099900000002</v>
       </c>
       <c r="P9">
-        <v>55.283667169998701</v>
+        <v>34.036468584688201</v>
       </c>
       <c r="Q9">
         <v>0</v>
       </c>
       <c r="R9">
-        <v>6.8992727909999996</v>
+        <v>7.2408784649999998</v>
       </c>
       <c r="S9">
-        <v>235.486627497</v>
+        <v>302.821971077</v>
       </c>
       <c r="T9">
-        <v>9.5972222219999992</v>
+        <v>1.875</v>
       </c>
       <c r="U9">
-        <v>8.2768037179845209</v>
+        <v>2.0595439353553302</v>
       </c>
       <c r="V9">
-        <v>7.4016455551037099</v>
+        <v>1.70644393578708</v>
       </c>
       <c r="W9">
-        <v>2.7812450169999998</v>
+        <v>0.92917335999999995</v>
       </c>
       <c r="X9">
-        <v>1.145634117</v>
+        <v>0.31390148600000001</v>
       </c>
       <c r="Y9">
-        <v>41.1914128384037</v>
+        <v>33.782876211603799</v>
       </c>
       <c r="Z9">
         <v>0</v>
       </c>
       <c r="AA9" s="76">
         <f t="shared" si="9"/>
-        <v>9.522312200000016E-2</v>
+        <v>6.6187779999999918E-3</v>
       </c>
       <c r="AB9" s="61">
         <f t="shared" si="10"/>
-        <v>5.8017058549999945</v>
+        <v>-2.3982108530000232</v>
       </c>
       <c r="AC9" s="77">
         <f t="shared" si="11"/>
-        <v>0.91666666700000121</v>
+        <v>0.25</v>
       </c>
       <c r="AD9" s="77">
         <f t="shared" si="12"/>
-        <v>0.36914491404468919</v>
+        <v>0.12246224002220973</v>
       </c>
       <c r="AE9" s="15">
         <f t="shared" si="13"/>
-        <v>0.46296772763905025</v>
+        <v>0.21057311708668003</v>
       </c>
       <c r="AF9" s="15">
         <f t="shared" si="14"/>
-        <v>1.2638754670000001</v>
+        <v>1.4934570000000091E-2</v>
       </c>
       <c r="AG9" s="15">
         <f t="shared" si="15"/>
-        <v>1.090656828</v>
+        <v>7.4395130000000087E-3</v>
       </c>
       <c r="AH9" s="77">
         <f t="shared" si="16"/>
-        <v>14.092254331595001</v>
+        <v>0.25359237308440186</v>
       </c>
       <c r="AI9" s="78">
         <f t="shared" si="17"/>
@@ -2635,84 +2629,84 @@
         <v>207</v>
       </c>
       <c r="C10" s="81">
-        <v>46223</v>
+        <v>46244</v>
       </c>
       <c r="D10" t="s">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="E10" t="s">
-        <v>310</v>
+        <v>257</v>
       </c>
       <c r="F10" t="s">
-        <v>311</v>
+        <v>258</v>
       </c>
       <c r="G10">
-        <v>6.2039999999999997</v>
+        <v>7.1328329999999998</v>
       </c>
       <c r="H10">
-        <v>99.982354999999998</v>
+        <v>99.899519999999995</v>
       </c>
       <c r="I10">
-        <v>6.0700643080000001</v>
+        <v>7.0663776169999997</v>
       </c>
       <c r="J10">
-        <v>184.310056514</v>
+        <v>276.07705351800001</v>
       </c>
       <c r="K10">
-        <v>2.013888889</v>
+        <v>3.0416666669999999</v>
       </c>
       <c r="L10">
-        <v>1.8502640230868701</v>
+        <v>2.65877454065846</v>
       </c>
       <c r="M10">
-        <v>1.8502640230868701</v>
+        <v>2.6633240690245699</v>
       </c>
       <c r="N10">
-        <v>4.9789018829999998</v>
+        <v>0.883067249</v>
       </c>
       <c r="O10">
-        <v>3.506802757</v>
+        <v>0.29685886700000003</v>
       </c>
       <c r="P10">
-        <v>70.433256959203305</v>
+        <v>33.616790492022901</v>
       </c>
       <c r="Q10">
         <v>0</v>
       </c>
       <c r="R10">
-        <v>6.0839366070000001</v>
+        <v>7.0577070639999997</v>
       </c>
       <c r="S10">
-        <v>185.69740145099999</v>
+        <v>275.208844924</v>
       </c>
       <c r="T10">
-        <v>2.013888889</v>
+        <v>3.0416666669999999</v>
       </c>
       <c r="U10">
-        <v>1.85012309380577</v>
+        <v>2.6477816239757699</v>
       </c>
       <c r="V10">
-        <v>1.85012309380577</v>
+        <v>2.6636275219340502</v>
       </c>
       <c r="W10">
-        <v>1.676286851</v>
+        <v>0.83752812099999996</v>
       </c>
       <c r="X10">
-        <v>1.0111258009999999</v>
+        <v>0.28195742000000001</v>
       </c>
       <c r="Y10">
-        <v>60.319377939211698</v>
+        <v>33.665427217338802</v>
       </c>
       <c r="Z10">
         <v>0</v>
       </c>
       <c r="AA10" s="76">
         <f t="shared" si="9"/>
-        <v>-1.3872298999999977E-2</v>
+        <v>8.6705529999999698E-3</v>
       </c>
       <c r="AB10" s="61">
         <f t="shared" si="10"/>
-        <v>-1.3873449369999946</v>
+        <v>0.86820859400000927</v>
       </c>
       <c r="AC10" s="77">
         <f t="shared" si="11"/>
@@ -2720,23 +2714,23 @@
       </c>
       <c r="AD10" s="77">
         <f t="shared" si="12"/>
-        <v>1.409292811000995E-4</v>
+        <v>1.099291668269009E-2</v>
       </c>
       <c r="AE10" s="15">
         <f t="shared" si="13"/>
-        <v>1.409292811000995E-4</v>
+        <v>-3.0345290948030623E-4</v>
       </c>
       <c r="AF10" s="15">
         <f t="shared" si="14"/>
-        <v>3.3026150319999998</v>
+        <v>4.553912800000004E-2</v>
       </c>
       <c r="AG10" s="15">
         <f t="shared" si="15"/>
-        <v>2.4956769560000001</v>
+        <v>1.4901447000000012E-2</v>
       </c>
       <c r="AH10" s="77">
         <f t="shared" si="16"/>
-        <v>10.113879019991607</v>
+        <v>-4.8636725315901685E-2</v>
       </c>
       <c r="AI10" s="78">
         <f t="shared" si="17"/>
@@ -2748,84 +2742,84 @@
         <v>207</v>
       </c>
       <c r="C11" s="81">
-        <v>46223</v>
+        <v>46244</v>
       </c>
       <c r="D11" t="s">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="E11" t="s">
-        <v>312</v>
+        <v>259</v>
       </c>
       <c r="F11" t="s">
-        <v>313</v>
+        <v>260</v>
       </c>
       <c r="G11">
-        <v>6.9850000000000003</v>
+        <v>7.1328329999999998</v>
       </c>
       <c r="H11">
-        <v>99.848609999999994</v>
+        <v>97.725035000000005</v>
       </c>
       <c r="I11">
-        <v>6.9738441050000004</v>
+        <v>7.8947988100000002</v>
       </c>
       <c r="J11">
-        <v>272.49060229399998</v>
+        <v>358.93509365400001</v>
       </c>
       <c r="K11">
-        <v>3.1805555559999998</v>
+        <v>3.0416666669999999</v>
       </c>
       <c r="L11">
-        <v>2.77808574901543</v>
+        <v>2.6444061544720898</v>
       </c>
       <c r="M11">
-        <v>2.77808574901543</v>
+        <v>2.6489736800810602</v>
       </c>
       <c r="N11">
-        <v>6.0880710310000001</v>
+        <v>0.883067249</v>
       </c>
       <c r="O11">
-        <v>4.4505215099999997</v>
+        <v>0.29685886700000003</v>
       </c>
       <c r="P11">
-        <v>73.102325635464496</v>
+        <v>33.616790492022901</v>
       </c>
       <c r="Q11">
         <v>0</v>
       </c>
       <c r="R11">
-        <v>6.9918282359999999</v>
+        <v>7.8860335719999997</v>
       </c>
       <c r="S11">
-        <v>274.28928462599998</v>
+        <v>358.05740464100001</v>
       </c>
       <c r="T11">
-        <v>3.1805555559999998</v>
+        <v>3.0416666669999999</v>
       </c>
       <c r="U11">
-        <v>2.7777533592985999</v>
+        <v>2.6333464480212299</v>
       </c>
       <c r="V11">
-        <v>2.7777533592985999</v>
+        <v>2.6492781537504699</v>
       </c>
       <c r="W11">
-        <v>2.0577725149999999</v>
+        <v>0.83752812099999996</v>
       </c>
       <c r="X11">
-        <v>1.2790980080000001</v>
+        <v>0.28195742000000001</v>
       </c>
       <c r="Y11">
-        <v>62.159349426435497</v>
+        <v>33.665427217338802</v>
       </c>
       <c r="Z11">
         <v>0</v>
       </c>
       <c r="AA11" s="76">
         <f t="shared" si="9"/>
-        <v>-1.7984130999999515E-2</v>
+        <v>8.7652380000005081E-3</v>
       </c>
       <c r="AB11" s="61">
         <f t="shared" si="10"/>
-        <v>-1.7986823319999985</v>
+        <v>0.87768901300000834</v>
       </c>
       <c r="AC11" s="77">
         <f t="shared" si="11"/>
@@ -2833,23 +2827,23 @@
       </c>
       <c r="AD11" s="77">
         <f t="shared" si="12"/>
-        <v>3.3238971683013929E-4</v>
+        <v>1.1059706450859963E-2</v>
       </c>
       <c r="AE11" s="15">
         <f t="shared" si="13"/>
-        <v>3.3238971683013929E-4</v>
+        <v>-3.0447366940977716E-4</v>
       </c>
       <c r="AF11" s="15">
         <f t="shared" si="14"/>
-        <v>4.0302985160000002</v>
+        <v>4.553912800000004E-2</v>
       </c>
       <c r="AG11" s="15">
         <f t="shared" si="15"/>
-        <v>3.1714235019999997</v>
+        <v>1.4901447000000012E-2</v>
       </c>
       <c r="AH11" s="77">
         <f t="shared" si="16"/>
-        <v>10.942976209028998</v>
+        <v>-4.8636725315901685E-2</v>
       </c>
       <c r="AI11" s="78">
         <f t="shared" si="17"/>
@@ -2861,108 +2855,108 @@
         <v>207</v>
       </c>
       <c r="C12" s="81">
-        <v>46223</v>
+        <v>46244</v>
       </c>
       <c r="D12" t="s">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="E12" t="s">
-        <v>58</v>
+        <v>261</v>
       </c>
       <c r="F12" t="s">
-        <v>59</v>
+        <v>262</v>
       </c>
       <c r="G12">
-        <v>3.9646650000000001</v>
+        <v>7.1328329999999998</v>
       </c>
       <c r="H12">
-        <v>77.950710000000001</v>
+        <v>93.091610000000003</v>
       </c>
       <c r="I12">
-        <v>6.9247222969999997</v>
+        <v>9.7392641970000007</v>
       </c>
       <c r="J12">
-        <v>231.98490674199999</v>
+        <v>543.41768254600004</v>
       </c>
       <c r="K12">
-        <v>10.930555556</v>
+        <v>3.0416666669999999</v>
       </c>
       <c r="L12">
-        <v>10.140540995713801</v>
+        <v>2.6126969745178998</v>
       </c>
       <c r="M12">
-        <v>8.2566437124177696</v>
+        <v>2.61730468836021</v>
       </c>
       <c r="N12">
-        <v>2.6432841790000001</v>
+        <v>0.883067249</v>
       </c>
       <c r="O12">
-        <v>1.2469935050000001</v>
+        <v>0.29685886700000003</v>
       </c>
       <c r="P12">
-        <v>47.175915283984303</v>
+        <v>33.616790492022901</v>
       </c>
       <c r="Q12">
         <v>0</v>
       </c>
       <c r="R12">
-        <v>6.8203104449999996</v>
+        <v>9.7302851480000001</v>
       </c>
       <c r="S12">
-        <v>220.39126758500001</v>
+        <v>542.51858560799997</v>
       </c>
       <c r="T12">
-        <v>11.180555556</v>
+        <v>3.0416666669999999</v>
       </c>
       <c r="U12">
-        <v>9.9562868959115196</v>
+        <v>2.6014877430952201</v>
       </c>
       <c r="V12">
-        <v>8.4190623254105006</v>
+        <v>2.6176114195468401</v>
       </c>
       <c r="W12">
-        <v>3.0731743649999999</v>
+        <v>0.83752812099999996</v>
       </c>
       <c r="X12">
-        <v>1.3459800280000001</v>
+        <v>0.28195742000000001</v>
       </c>
       <c r="Y12">
-        <v>43.797711035507703</v>
+        <v>33.665427217338802</v>
       </c>
       <c r="Z12">
         <v>0</v>
       </c>
       <c r="AA12" s="76">
         <f t="shared" si="9"/>
-        <v>0.10441185200000014</v>
+        <v>8.9790490000005718E-3</v>
       </c>
       <c r="AB12" s="61">
         <f t="shared" si="10"/>
-        <v>11.593639156999984</v>
+        <v>0.89909693800007062</v>
       </c>
       <c r="AC12" s="77">
         <f t="shared" si="11"/>
-        <v>-0.25</v>
+        <v>0</v>
       </c>
       <c r="AD12" s="77">
         <f t="shared" si="12"/>
-        <v>0.18425409980228125</v>
+        <v>1.1209231422679711E-2</v>
       </c>
       <c r="AE12" s="15">
         <f t="shared" si="13"/>
-        <v>-0.16241861299273097</v>
+        <v>-3.0673118663004928E-4</v>
       </c>
       <c r="AF12" s="15">
         <f t="shared" si="14"/>
-        <v>-0.42989018599999973</v>
+        <v>4.553912800000004E-2</v>
       </c>
       <c r="AG12" s="15">
         <f t="shared" si="15"/>
-        <v>-9.8986522999999993E-2</v>
+        <v>1.4901447000000012E-2</v>
       </c>
       <c r="AH12" s="77">
         <f t="shared" si="16"/>
-        <v>3.3782042484765995</v>
+        <v>-4.8636725315901685E-2</v>
       </c>
       <c r="AI12" s="78">
         <f t="shared" si="17"/>
@@ -2974,108 +2968,108 @@
         <v>207</v>
       </c>
       <c r="C13" s="81">
-        <v>46223</v>
+        <v>46244</v>
       </c>
       <c r="D13" t="s">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="E13" t="s">
-        <v>60</v>
+        <v>310</v>
       </c>
       <c r="F13" t="s">
-        <v>61</v>
+        <v>311</v>
       </c>
       <c r="G13">
-        <v>4.0400159999999996</v>
+        <v>1.7915399999999999</v>
       </c>
       <c r="H13">
-        <v>78.143829999999994</v>
+        <v>2.7639999999999998</v>
       </c>
       <c r="I13">
-        <v>6.9722333030000003</v>
+        <v>17.956653355</v>
       </c>
       <c r="J13">
-        <v>236.80101277099999</v>
+        <v>1378.149046858</v>
       </c>
       <c r="K13">
-        <v>10.930555556</v>
+        <v>2.1724912289999998</v>
       </c>
       <c r="L13">
-        <v>9.9952842892394695</v>
+        <v>-22.416318958031798</v>
       </c>
       <c r="M13">
-        <v>8.2251801671353899</v>
+        <v>1.1988294138929201</v>
       </c>
       <c r="N13">
-        <v>2.7957284910000002</v>
+        <v>0.883067249</v>
       </c>
       <c r="O13">
-        <v>1.2922879190000001</v>
+        <v>0.29685886700000003</v>
       </c>
       <c r="P13">
-        <v>46.223655950859602</v>
+        <v>33.616790492022901</v>
       </c>
       <c r="Q13">
         <v>0</v>
       </c>
       <c r="R13">
-        <v>6.869167086</v>
+        <v>14.54363386</v>
       </c>
       <c r="S13">
-        <v>225.34384832399999</v>
+        <v>1036.7996621950001</v>
       </c>
       <c r="T13">
-        <v>11.180555556</v>
+        <v>2.0917987280000001</v>
       </c>
       <c r="U13">
-        <v>9.9303586399591595</v>
+        <v>-34.944284949348798</v>
       </c>
       <c r="V13">
-        <v>8.3868385565437595</v>
+        <v>1.21929761215629</v>
       </c>
       <c r="W13">
-        <v>3.3495219270000001</v>
+        <v>0.83752812099999996</v>
       </c>
       <c r="X13">
-        <v>1.357340274</v>
+        <v>0.28195742000000001</v>
       </c>
       <c r="Y13">
-        <v>40.523403147735202</v>
+        <v>33.665427217338802</v>
       </c>
       <c r="Z13">
         <v>0</v>
       </c>
       <c r="AA13" s="76">
         <f t="shared" si="9"/>
-        <v>0.10306621700000029</v>
+        <v>3.4130194950000003</v>
       </c>
       <c r="AB13" s="61">
         <f t="shared" si="10"/>
-        <v>11.457164446999997</v>
+        <v>341.34938466299991</v>
       </c>
       <c r="AC13" s="77">
         <f t="shared" si="11"/>
-        <v>-0.25</v>
+        <v>8.0692500999999694E-2</v>
       </c>
       <c r="AD13" s="77">
         <f t="shared" si="12"/>
-        <v>6.4925649280310083E-2</v>
+        <v>12.527965991317</v>
       </c>
       <c r="AE13" s="15">
         <f t="shared" si="13"/>
-        <v>-0.16165838940836963</v>
+        <v>-2.0468198263369874E-2</v>
       </c>
       <c r="AF13" s="15">
         <f t="shared" si="14"/>
-        <v>-0.55379343599999986</v>
+        <v>4.553912800000004E-2</v>
       </c>
       <c r="AG13" s="15">
         <f t="shared" si="15"/>
-        <v>-6.5052354999999951E-2</v>
+        <v>1.4901447000000012E-2</v>
       </c>
       <c r="AH13" s="77">
         <f t="shared" si="16"/>
-        <v>5.7002528031243997</v>
+        <v>-4.8636725315901685E-2</v>
       </c>
       <c r="AI13" s="78">
         <f t="shared" si="17"/>
@@ -3087,110 +3081,449 @@
         <v>207</v>
       </c>
       <c r="C14" s="81">
-        <v>46223</v>
+        <v>46244</v>
       </c>
       <c r="D14" t="s">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="E14" t="s">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="F14" t="s">
-        <v>63</v>
+        <v>92</v>
       </c>
       <c r="G14">
-        <v>7.7780399999999998</v>
+        <v>0.31317200000000001</v>
       </c>
       <c r="H14">
-        <v>100.18250500000001</v>
+        <v>0.53039499999999995</v>
       </c>
       <c r="I14">
-        <v>6.470128399</v>
+        <v>19.476548693000002</v>
       </c>
       <c r="J14">
-        <v>252.943057982</v>
+        <v>1521.022163268</v>
       </c>
       <c r="K14">
-        <v>0.51388888899999996</v>
+        <v>5.3418362459999997</v>
       </c>
       <c r="L14">
-        <v>0.49199213275811299</v>
+        <v>-47.746141272070801</v>
       </c>
       <c r="M14">
-        <v>0.49218625247991099</v>
+        <v>1.62173455632124</v>
       </c>
       <c r="N14">
-        <v>8.3187985990000008</v>
+        <v>0.78371344099999996</v>
       </c>
       <c r="O14">
-        <v>6.0184517570000002</v>
+        <v>0.29670481399999998</v>
       </c>
       <c r="P14">
-        <v>72.3476074745153</v>
+        <v>37.858839529587698</v>
       </c>
       <c r="Q14">
         <v>0</v>
       </c>
       <c r="R14">
-        <v>6.5503197550000003</v>
+        <v>14.128988043</v>
       </c>
       <c r="S14">
-        <v>260.96217377099998</v>
+        <v>986.71720607500004</v>
       </c>
       <c r="T14">
-        <v>0.51388888899999996</v>
+        <v>5.226958786</v>
       </c>
       <c r="U14">
-        <v>0.49191448226318701</v>
+        <v>-68.2373091752373</v>
       </c>
       <c r="V14">
-        <v>0.49199631941043498</v>
+        <v>1.64397401936292</v>
       </c>
       <c r="W14">
-        <v>5.654692636</v>
+        <v>0.76701628799999999</v>
       </c>
       <c r="X14">
-        <v>3.870288006</v>
+        <v>0.29267415000000002</v>
       </c>
       <c r="Y14">
-        <v>68.443826307379197</v>
+        <v>38.157488254017402</v>
       </c>
       <c r="Z14">
         <v>0</v>
       </c>
       <c r="AA14" s="76">
         <f t="shared" si="9"/>
-        <v>-8.0191356000000269E-2</v>
+        <v>5.3475606500000019</v>
       </c>
       <c r="AB14" s="61">
         <f t="shared" si="10"/>
-        <v>-8.0191157889999829</v>
+        <v>534.30495719299995</v>
       </c>
       <c r="AC14" s="77">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>0.11487745999999976</v>
       </c>
       <c r="AD14" s="77">
         <f t="shared" si="12"/>
-        <v>7.7650494925973756E-5</v>
+        <v>20.491167903166499</v>
       </c>
       <c r="AE14" s="15">
         <f t="shared" si="13"/>
-        <v>1.8993306947601152E-4</v>
+        <v>-2.2239463041680008E-2</v>
       </c>
       <c r="AF14" s="15">
         <f t="shared" si="14"/>
-        <v>2.6641059630000008</v>
+        <v>1.6697152999999965E-2</v>
       </c>
       <c r="AG14" s="15">
         <f t="shared" si="15"/>
-        <v>2.1481637510000002</v>
+        <v>4.0306639999999616E-3</v>
       </c>
       <c r="AH14" s="77">
         <f t="shared" si="16"/>
-        <v>3.9037811671361027</v>
+        <v>-0.2986487244297038</v>
       </c>
       <c r="AI14" s="78">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="2:35" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>207</v>
+      </c>
+      <c r="C15" s="81">
+        <v>46244</v>
+      </c>
+      <c r="D15" t="s">
+        <v>64</v>
+      </c>
+      <c r="E15" t="s">
+        <v>95</v>
+      </c>
+      <c r="F15" t="s">
+        <v>96</v>
+      </c>
+      <c r="G15">
+        <v>2</v>
+      </c>
+      <c r="H15">
+        <v>2.75</v>
+      </c>
+      <c r="I15">
+        <v>29.195159699000001</v>
+      </c>
+      <c r="J15">
+        <v>2495.61010115</v>
+      </c>
+      <c r="K15">
+        <v>2.3435540879999999</v>
+      </c>
+      <c r="L15">
+        <v>-60.581535345454498</v>
+      </c>
+      <c r="M15">
+        <v>1.3003203999999999</v>
+      </c>
+      <c r="N15">
+        <v>0.66606547500000002</v>
+      </c>
+      <c r="O15">
+        <v>0.18802116899999999</v>
+      </c>
+      <c r="P15">
+        <v>28.228631577098302</v>
+      </c>
+      <c r="Q15">
+        <v>0</v>
+      </c>
+      <c r="R15">
+        <v>25.348700129000001</v>
+      </c>
+      <c r="S15">
+        <v>2111.2885021339998</v>
+      </c>
+      <c r="T15">
+        <v>2.1633200430000001</v>
+      </c>
+      <c r="U15">
+        <v>-78.460830981818205</v>
+      </c>
+      <c r="V15">
+        <v>1.3064762181818099</v>
+      </c>
+      <c r="W15">
+        <v>0.64286090299999998</v>
+      </c>
+      <c r="X15">
+        <v>0.17993668800000001</v>
+      </c>
+      <c r="Y15">
+        <v>27.989987750118299</v>
+      </c>
+      <c r="Z15">
+        <v>0</v>
+      </c>
+      <c r="AA15" s="76">
+        <f t="shared" si="9"/>
+        <v>3.8464595700000004</v>
+      </c>
+      <c r="AB15" s="61">
+        <f t="shared" si="10"/>
+        <v>384.32159901600016</v>
+      </c>
+      <c r="AC15" s="77">
+        <f t="shared" si="11"/>
+        <v>0.18023404499999973</v>
+      </c>
+      <c r="AD15" s="77">
+        <f t="shared" si="12"/>
+        <v>17.879295636363707</v>
+      </c>
+      <c r="AE15" s="15">
+        <f t="shared" si="13"/>
+        <v>-6.1558181818099911E-3</v>
+      </c>
+      <c r="AF15" s="15">
+        <f t="shared" si="14"/>
+        <v>2.3204572000000034E-2</v>
+      </c>
+      <c r="AG15" s="15">
+        <f t="shared" si="15"/>
+        <v>8.0844809999999767E-3</v>
+      </c>
+      <c r="AH15" s="77">
+        <f t="shared" si="16"/>
+        <v>0.23864382698000242</v>
+      </c>
+      <c r="AI15" s="78">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="2:35" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>207</v>
+      </c>
+      <c r="C16" s="81">
+        <v>46244</v>
+      </c>
+      <c r="D16" t="s">
+        <v>64</v>
+      </c>
+      <c r="E16" t="s">
+        <v>99</v>
+      </c>
+      <c r="F16" t="s">
+        <v>100</v>
+      </c>
+      <c r="G16">
+        <v>3.0332599999999998</v>
+      </c>
+      <c r="H16">
+        <v>5.5</v>
+      </c>
+      <c r="I16">
+        <v>27.282576035999998</v>
+      </c>
+      <c r="J16">
+        <v>2295.9761514679999</v>
+      </c>
+      <c r="K16">
+        <v>4.2268698149999997</v>
+      </c>
+      <c r="L16">
+        <v>-13.0010127636364</v>
+      </c>
+      <c r="M16">
+        <v>1.76838900000001</v>
+      </c>
+      <c r="N16">
+        <v>0.75045333000000003</v>
+      </c>
+      <c r="O16">
+        <v>0.17430203799999999</v>
+      </c>
+      <c r="P16">
+        <v>23.226232869137899</v>
+      </c>
+      <c r="Q16">
+        <v>0</v>
+      </c>
+      <c r="R16">
+        <v>26.179327288</v>
+      </c>
+      <c r="S16">
+        <v>2185.5652062909999</v>
+      </c>
+      <c r="T16">
+        <v>4.0939856250000002</v>
+      </c>
+      <c r="U16">
+        <v>-29.892031200000002</v>
+      </c>
+      <c r="V16">
+        <v>1.7834362909090999</v>
+      </c>
+      <c r="W16">
+        <v>0.73226718800000001</v>
+      </c>
+      <c r="X16">
+        <v>0.16969759700000001</v>
+      </c>
+      <c r="Y16">
+        <v>23.1742729676971</v>
+      </c>
+      <c r="Z16">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="76">
+        <f t="shared" si="9"/>
+        <v>1.1032487479999986</v>
+      </c>
+      <c r="AB16" s="61">
+        <f t="shared" si="10"/>
+        <v>110.41094517700003</v>
+      </c>
+      <c r="AC16" s="77">
+        <f t="shared" si="11"/>
+        <v>0.13288418999999951</v>
+      </c>
+      <c r="AD16" s="77">
+        <f t="shared" si="12"/>
+        <v>16.891018436363602</v>
+      </c>
+      <c r="AE16" s="15">
+        <f t="shared" si="13"/>
+        <v>-1.5047290909089961E-2</v>
+      </c>
+      <c r="AF16" s="15">
+        <f t="shared" si="14"/>
+        <v>1.8186142000000016E-2</v>
+      </c>
+      <c r="AG16" s="15">
+        <f t="shared" si="15"/>
+        <v>4.6044409999999869E-3</v>
+      </c>
+      <c r="AH16" s="77">
+        <f t="shared" si="16"/>
+        <v>5.1959901440799428E-2</v>
+      </c>
+      <c r="AI16" s="78">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:35" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>207</v>
+      </c>
+      <c r="C17" s="81">
+        <v>46244</v>
+      </c>
+      <c r="D17" t="s">
+        <v>64</v>
+      </c>
+      <c r="E17" t="s">
+        <v>101</v>
+      </c>
+      <c r="F17" t="s">
+        <v>102</v>
+      </c>
+      <c r="G17">
+        <v>0.13406999999999999</v>
+      </c>
+      <c r="H17">
+        <v>0.22933500000000001</v>
+      </c>
+      <c r="I17">
+        <v>16.584399908000002</v>
+      </c>
+      <c r="J17">
+        <v>1233.8160088489999</v>
+      </c>
+      <c r="K17">
+        <v>4.2268698149999997</v>
+      </c>
+      <c r="L17">
+        <v>-45.954590446290403</v>
+      </c>
+      <c r="M17">
+        <v>1.53956657291736</v>
+      </c>
+      <c r="N17">
+        <v>0.75045333000000003</v>
+      </c>
+      <c r="O17">
+        <v>0.17430203799999999</v>
+      </c>
+      <c r="P17">
+        <v>23.226232869137899</v>
+      </c>
+      <c r="Q17">
+        <v>0</v>
+      </c>
+      <c r="R17">
+        <v>11.895817848</v>
+      </c>
+      <c r="S17">
+        <v>765.59291047600004</v>
+      </c>
+      <c r="T17">
+        <v>4.0939856250000002</v>
+      </c>
+      <c r="U17">
+        <v>-65.182531231604401</v>
+      </c>
+      <c r="V17">
+        <v>1.5431033204700499</v>
+      </c>
+      <c r="W17">
+        <v>0.73226718800000001</v>
+      </c>
+      <c r="X17">
+        <v>0.16969759700000001</v>
+      </c>
+      <c r="Y17">
+        <v>23.1742729676971</v>
+      </c>
+      <c r="Z17">
+        <v>0</v>
+      </c>
+      <c r="AA17" s="76">
+        <f t="shared" si="9"/>
+        <v>4.6885820600000017</v>
+      </c>
+      <c r="AB17" s="61">
+        <f t="shared" si="10"/>
+        <v>468.22309837299986</v>
+      </c>
+      <c r="AC17" s="77">
+        <f t="shared" si="11"/>
+        <v>0.13288418999999951</v>
+      </c>
+      <c r="AD17" s="77">
+        <f t="shared" si="12"/>
+        <v>19.227940785313997</v>
+      </c>
+      <c r="AE17" s="15">
+        <f t="shared" si="13"/>
+        <v>-3.5367475526899561E-3</v>
+      </c>
+      <c r="AF17" s="15">
+        <f t="shared" si="14"/>
+        <v>1.8186142000000016E-2</v>
+      </c>
+      <c r="AG17" s="15">
+        <f t="shared" si="15"/>
+        <v>4.6044409999999869E-3</v>
+      </c>
+      <c r="AH17" s="77">
+        <f t="shared" si="16"/>
+        <v>5.1959901440799428E-2</v>
+      </c>
+      <c r="AI17" s="78">
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
@@ -3203,8 +3536,8 @@
     <mergeCell ref="AA2:AI2"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
-  <conditionalFormatting sqref="AA4:AA14">
-    <cfRule type="colorScale" priority="81">
+  <conditionalFormatting sqref="AA4:AA17">
+    <cfRule type="colorScale" priority="86">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="num" val="0"/>
@@ -3215,8 +3548,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB4:AB14">
-    <cfRule type="colorScale" priority="82">
+  <conditionalFormatting sqref="AB4:AB17">
+    <cfRule type="colorScale" priority="87">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3227,8 +3560,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AC4:AC14">
-    <cfRule type="colorScale" priority="83">
+  <conditionalFormatting sqref="AC4:AC17">
+    <cfRule type="colorScale" priority="88">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3239,8 +3572,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AD4:AD14">
-    <cfRule type="colorScale" priority="84">
+  <conditionalFormatting sqref="AD4:AD17">
+    <cfRule type="colorScale" priority="89">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3251,8 +3584,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AF4:AF14">
-    <cfRule type="colorScale" priority="85">
+  <conditionalFormatting sqref="AF4:AF17">
+    <cfRule type="colorScale" priority="90">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="num" val="0"/>

</xml_diff>